<commit_message>
wujiang change up to 15
</commit_message>
<xml_diff>
--- a/docs/武将实现问题清单.xlsx
+++ b/docs/武将实现问题清单.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="说明" sheetId="1" r:id="Ra3cb1c3257e24496"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="问卷" sheetId="2" r:id="Rac5efb487a2c4c53"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="武将设计思想" sheetId="3" r:id="R8541ff0c34eb42b3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="武将符合性审查" sheetId="4" r:id="R30aa0e0bf99c4b7e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="说明" sheetId="1" r:id="R8f51f8bfa8144def"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="问卷" sheetId="2" r:id="R53eccb31602e4669"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="武将设计思想" sheetId="3" r:id="R8fe76335ea544a52"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="武将符合性审查" sheetId="4" r:id="R1627c399c30b4263"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -5944,7 +5944,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="HeroDesignIdeasTable" displayName="HeroDesignIdeasTable" ref="A1:AA16" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="HeroDesignIdeasTable" displayName="HeroDesignIdeasTable" ref="A1:AA19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="27">
     <x:tableColumn id="1" name="批次"/>
     <x:tableColumn id="2" name="源表行"/>
@@ -5979,7 +5979,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="HeroConformanceReviewTable" displayName="HeroConformanceReviewTable" ref="A1:M80" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="HeroConformanceReviewTable" displayName="HeroConformanceReviewTable" ref="A1:M92" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="13">
     <x:tableColumn id="1" name="武将代码"/>
     <x:tableColumn id="2" name="武将名"/>
@@ -22218,7 +22218,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R63bb51251bb04905"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R18e58350f4664a89"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -23294,7 +23294,7 @@
         <x:v>治疗反转误伤、无消费渠道堆点、重复防御、临时状态越队友回合叠加、无价值大招和移动、圣光半轮数量混乱。</x:v>
       </x:c>
       <x:c r="Z12" s="94" t="str">
-        <x:v>武将说明第5节、通用技能、持久吟游诗人索引；源文本时长与资源冲突均在读取实现前记录裁定，无该武将问卷回答。</x:v>
+        <x:v>武将说明第5节、通用技能、持久吟游诗人索引；源文本时长与资源冲突均在读取实现前记录裁定，无该武将问卷回答。 2026-09-10补充源文§8.3：反转是特殊扣血，仍受护盾、魔免等防御；不因写作失去生命就无视防御。支援距离按通用多格规则检查完整身体。</x:v>
       </x:c>
       <x:c r="AA12" s="94" t="str">
         <x:v>2026-09-09完成战斗、AI、预览与测试代码检查修改；静态检查通过，动态验证等待全部73名已开发武将完成后统一进行。</x:v>
@@ -23441,7 +23441,7 @@
         <x:v>["有效终结/重置机会","已有执念对象与可兑现连续普攻","有收益风沙/破盾撕裂","兼顾命中和安全落点的狂沙","保留反应与恢复路线"]</x:v>
       </x:c>
       <x:c r="S14" s="94" t="str">
-        <x:v>["绕过执念或骑乘重定向","把己方/天气/非伤害击破当再动","沙尘中尝试隐身","为零收益天气/狂沙浪费动作","透视隐身与分身真假"]</x:v>
+        <x:v>["绕过执念或骑乘重定向","把队友造成的击破/天气/非伤害击破当再动","沙尘中尝试隐身","为零收益天气/狂沙浪费动作","透视隐身与分身真假"]</x:v>
       </x:c>
       <x:c r="T14" s="94" t="str">
         <x:v>再动收益应与实际击破资格、一次上限及后续可行动机会相乘；移动伤害动作必须共同评估原选区与新身体落点。</x:v>
@@ -23462,10 +23462,10 @@
         <x:v>["伤害回调把天气误算技能击破","击杀后动作计数覆盖重置","狂沙冷却仍按旧半轮","移动后重算原选区","光环只检查锚点"]</x:v>
       </x:c>
       <x:c r="Z14" s="94" t="str">
-        <x:v>docs/武将说明.md第7节；通用规则§8、§15–17；hero-rule-index和project-map明确骑乘后锁坐骑、仅自身攻击/技能击破及守≥4资格。</x:v>
+        <x:v>docs/武将说明.md第7节；通用规则§8、§15–17；hero-rule-index和project-map明确骑乘后锁坐骑、仅自身攻击/技能击破及守≥4资格。 文字勘误：这里排除的是队友造成的击破，并非擅自增加被击破者必须是敌方的限制；仍按源文自身攻击/技能与目标资格判断。</x:v>
       </x:c>
       <x:c r="AA14" s="94" t="str">
-        <x:v>源规则独立设计基线已锁定；待依次读取战斗实现、AI、测试并修正。动态测试留到全部已开发武将完成后。</x:v>
+        <x:v>2026-09-10完成战斗、AI、预览及测试代码逐项检查修改；静态检查通过，动态验证等待全部已开发武将完成后统一运行。</x:v>
       </x:c>
       <x:c r="AB14" s="94" t="str">
         <x:v>[{"topic":"狂沙的固定方向与受阻落点","decision":"声明锁定五格伤害线和第六格落点，整个2×2可放置才允许声明；连锁后终点被占时保留原线伤害但不强行重叠移动。","reasoning":"源文分别列伤害与瞬移；通用规则要求原格结算及最终占格互斥。","rejected_alternatives":"不让反应位移重新瞄准伤害，不推走占位者，不让瞬移失败倒退抹消已声明伤害。","confidence":"中高","gameplay_consequence":"预览/AI/结算同一快照，失败移动有明确反馈。"},{"topic":"风沙一轮","decision":"全局天气持续到施法者下一己方回合开始；天气伤害按受影响单位自己的回合结束结算一次。","reasoning":"全局覆盖不应使多人回合缩短一轮或叠加每个单位伤害，通用己方回合指武将自己。","rejected_alternatives":"不按两个任意武将回合就消失，不每次别人结束回合都伤害全场。","confidence":"中","gameplay_consequence":"多人和双人均给每个目标一个自己的行动窗口。"}]</x:v>
@@ -23549,7 +23549,7 @@
         <x:v>docs/武将说明.md第8节与通用规则§15–17；持久索引/地图明确边界碰撞也产生独立3×3效果、岩吸按成功单位数而非实际降值计数。</x:v>
       </x:c>
       <x:c r="AA15" s="94" t="str">
-        <x:v>源规则独立设计基线已锁定；待依次读取战斗实现、AI、测试并修正。动态测试留到全部已开发武将完成后。</x:v>
+        <x:v>2026-09-10完成战斗、AI、预览及测试代码逐项检查修改；静态检查通过，动态验证等待全部已开发武将完成后统一运行。</x:v>
       </x:c>
       <x:c r="AB15" s="94" t="str">
         <x:v>[{"topic":"岩吸一轮与同源重复","decision":"本次目标减值、自身增益和临时扩体统一到施法者下一己方回合开始前结束；同源同属性不重叠额外层数。","reasoning":"源文将同次吸收的减值、增益和身体共享一轮持续，需保持交换同步。","rejected_alternatives":"不在各目标不同时间点结束而让同次交换长时间失衡，不把旧临时增长永久化。","confidence":"中","gameplay_consequence":"多人局按吸收源时钟统一释放，并正确限制魔容量。"},{"topic":"边界炮弹","decision":"按持久索引处理：没有单位时在边界消失位置也生成一次3×3爆炸。","reasoning":"hero-rule-index与project-map两处明确unit or boundary独立伤害，源说明边界消失未明确禁止爆炸。","rejected_alternatives":"不自动将未碰单位的炮弹全部删除伤害。","confidence":"中高","gameplay_consequence":"可用边缘溅射，但必须计友伤和身体成本。"}]</x:v>
@@ -23633,16 +23633,268 @@
         <x:v>docs/武将说明.md第9节、通用规则§8–9、§15；持久索引明确n须显式且1.25可n1、tick不得递归刷新，生命可超量。</x:v>
       </x:c>
       <x:c r="AA16" s="94" t="str">
-        <x:v>源规则独立设计基线已锁定；待依次读取战斗实现、AI、测试并修正。动态测试留到全部已开发武将完成后。</x:v>
+        <x:v>2026-09-10完成战斗、AI、预览及测试代码逐项检查修改；静态检查通过，动态验证等待全部已开发武将完成后统一运行。</x:v>
       </x:c>
       <x:c r="AB16" s="94" t="str">
         <x:v>[{"topic":"同名效果来源与吸收","decision":"已有末日光时不叠加也不刷新；保留首次施加者，实际扣血仅回复这个有效存活来源，且服从该来源禁疗。","reasoning":"不叠加和四轮给出明确结束窗口，吸收是施加者伤害回流而非多个同名英雄无条件共享。","rejected_alternatives":"不永久刷新，不由第二条龙覆盖所有权，不让每条龙从同一扣血重复获得完整回血。","confidence":"中","gameplay_consequence":"状态记录来源且探测须统计实际HP变化；来源失效不影响剩余四轮但不再吸收。"},{"topic":"无伤普攻与无伤技能","decision":"有效普攻声明龙即使最终被盾挡或回避仍反噬；技能只有真正造成伤害才走反噬伤害条件。","reasoning":"源文用普攻或造成伤害分列触发条件，不能把两者都缩成伤害后。","rejected_alternatives":"不把所有被阻挡技能都算伤害，不让盾完全消去普攻声明反噬。","confidence":"高","gameplay_consequence":"声明与实际伤害触发分开并避免重复加同名状态。"}]</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="260" customHeight="1">
+      <x:c r="A17" s="94" t="str">
+        <x:v>R04</x:v>
+      </x:c>
+      <x:c r="B17" s="94"/>
+      <x:c r="C17" s="94" t="str">
+        <x:v>masamune</x:v>
+      </x:c>
+      <x:c r="D17" s="94" t="str">
+        <x:v>天位骑士。政宗</x:v>
+      </x:c>
+      <x:c r="E17" s="94" t="str">
+        <x:v>仅使用武将说明§10–12、通用规则/技能与持久索引；问卷已按三名精确匹配确认无保存答案。先写入JSON及XLSX后才读本批战斗、AI、测试；代码不作设计来源。</x:v>
+      </x:c>
+      <x:c r="F17" s="94" t="str">
+        <x:v>2026-09-10</x:v>
+      </x:c>
+      <x:c r="G17" s="94" t="str">
+        <x:v>骑乘摩托马突进，用弧形挥斩压迫近身，必要时跃下马转为六刀连击与格挡反击。</x:v>
+      </x:c>
+      <x:c r="H17" s="94" t="str">
+        <x:v>骑乘承伤与下马爆发互换的近身骑士。</x:v>
+      </x:c>
+      <x:c r="I17" s="94" t="str">
+        <x:v>坐骑提供机动和生命缓冲，下马才开放六刀与防守吸血；选择三次普通攻击还是三连重斩必须有实际代价。</x:v>
+      </x:c>
+      <x:c r="J17" s="94" t="str">
+        <x:v>骑乘位置与八方向弧面；保留坐骑还是免费跃下；六刀前先选输出路线；三次攻击合并能否突破守盾；何时治马或重召。</x:v>
+      </x:c>
+      <x:c r="K17" s="94" t="str">
+        <x:v>出场已骑乘；优先由马移动/免费神速带动；选择弧面目标及普通/三连；下马后尚未普攻才可开六刀，利用剩余六次或两次重斩；敌方回合按当前骑乘状态决定格挡反击。</x:v>
+      </x:c>
+      <x:c r="L17" s="94" t="str">
+        <x:v>等级4土人类骑士，攻4守3速3范1魔3。马攻0守5速5范1魔0，纵向1×2，神速0每自身回合一次。六刀0每回合一次；治马0每回合一次血+.5；保护1魔；骑乘飞跃0每回合一次；重斩消耗3普攻次数。</x:v>
+      </x:c>
+      <x:c r="M17" s="94" t="str">
+        <x:v>六刀把攻降至3但允许6次普攻或两次攻6半破魔重斩；下马有效普攻吸血+.25；骑乘时代理保护坐骑，自己跃离会丢失马的承伤。</x:v>
+      </x:c>
+      <x:c r="N17" s="94" t="str">
+        <x:v>坐骑较高速度守、可选多次低伤或合并破盾、下马反应和回血。</x:v>
+      </x:c>
+      <x:c r="O17" s="94" t="str">
+        <x:v>范1且弧面需声明；马占两格易受范围额外伤害；重斩需足够攻击次数；主动下马舍弃承伤，重召有己方回合锁定。</x:v>
+      </x:c>
+      <x:c r="P17" s="94" t="str">
+        <x:v>用走位使声明原格落空、攻击坐骑或控制其落点、在六刀前逼其普攻，利用无马期间输出。</x:v>
+      </x:c>
+      <x:c r="Q17" s="94" t="str">
+        <x:v>优先坐骑带动；免费跃下仅在下马净收益更大时使用；评分包含六刀之后合法弧形攻击、重斩次数机会成本和有效吸血，保护当前承伤体。</x:v>
+      </x:c>
+      <x:c r="R17" s="94" t="str">
+        <x:v>["可兑现击破","合法六刀后连续攻击","坐骑移动与必要治马","有效三连重斩","防守格挡/反击"]</x:v>
+      </x:c>
+      <x:c r="S17" s="94" t="str">
+        <x:v>["无收益自行走离坐骑","攻击后开六刀","剩余少于3次仍重斩","混用马与骑士的移动或次数","把空挥/技能当吸血"]</x:v>
+      </x:c>
+      <x:c r="T17" s="94" t="str">
+        <x:v>状态转换技能要比较转换后整套行动，并按实际承伤体评估反应；高次数合并攻击不能只比单击伤害。</x:v>
+      </x:c>
+      <x:c r="U17" s="94" t="str">
+        <x:v>坐骑默认出场已召唤乘骑，场上自己的马存在时不能再召；破坏后隔一个自身回合才重召。八向弧形只选该弧面的一个有效目标；声明原格固定。飞跃本人直线恰3格可穿单位，马不移动，离开占格即下马。六刀限下马且本回合未普攻，攻-1和上限6仅本回合。三连+3攻击值半破魔消耗3次数；下马才格挡反击与普攻伤后回血。</x:v>
+      </x:c>
+      <x:c r="V17" s="94" t="str">
+        <x:v>骑乘伤害/效果重定向到马，骑士可替马连锁；攻击选择及反应发现同一原格。马与骑士共享所属武将回合而非独立顺位。治愈只针对当前乘骑的摩托马，禁疗仍生效。</x:v>
+      </x:c>
+      <x:c r="W17" s="94" t="str">
+        <x:v>按下列源规则推定明确，无待用户回答项。</x:v>
+      </x:c>
+      <x:c r="X17" s="94" t="str">
+        <x:v>["初始马及骑乘关系正确","八向预览与实际对象一致","两次六刀重斩共耗6次","跃下后马原地且开启下马反应","马破坏锁定公开可追踪"]</x:v>
+      </x:c>
+      <x:c r="Y17" s="94" t="str">
+        <x:v>["声明后错误重定位弧面","骑乘状态转变仍留旧反应","六刀持续跨己方回合","重斩不扣3次","吸血按原伤而非实际造成伤害"]</x:v>
+      </x:c>
+      <x:c r="Z17" s="94" t="str">
+        <x:v>武将说明§10；通用规则§3.1、5–11；通用技能飞跃/神速/保护/格挡/反击；hero-rule-index和project-map明确骑士自己的免费飞跃。</x:v>
+      </x:c>
+      <x:c r="AA17" s="94" t="str">
+        <x:v>设计基线已锁定；等待本批战斗、AI、测试逐项核对。</x:v>
+      </x:c>
+      <x:c r="AB17" s="94" t="str">
+        <x:v>[{"topic":"三连重斩与下马吸血","decision":"重斩+3按伤害公式中的攻击值处理，单次有效普攻伤害只回血一次.25，六刀的攻-1同样影响重斩。","reasoning":"通用规则伤n进入攻守公式，合并三次次数仍是一次普攻；下马战技明确状态条件。","rejected_alternatives":"不按固定扣3HP，不按消耗次数回血三次，不把吸血独立标题解释为骑乘时也有。","confidence":"高","gameplay_consequence":"保留攻击合并的取舍且避免坐骑承伤与无条件吸血叠加。"}]</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="260" customHeight="1">
+      <x:c r="A18" s="94" t="str">
+        <x:v>R04</x:v>
+      </x:c>
+      <x:c r="B18" s="94"/>
+      <x:c r="C18" s="94" t="str">
+        <x:v>jade</x:v>
+      </x:c>
+      <x:c r="D18" s="94" t="str">
+        <x:v>翡翠</x:v>
+      </x:c>
+      <x:c r="E18" s="94" t="str">
+        <x:v>仅使用武将说明§10–12、通用规则/技能与持久索引；问卷已按三名精确匹配确认无保存答案。先写入JSON及XLSX后才读本批战斗、AI、测试；代码不作设计来源。</x:v>
+      </x:c>
+      <x:c r="F18" s="94" t="str">
+        <x:v>2026-09-10</x:v>
+      </x:c>
+      <x:c r="G18" s="94" t="str">
+        <x:v>持续发射机甲火力，用离子与量子防护支援队友；敌人成功阻挡反而促成未来火力成长。</x:v>
+      </x:c>
+      <x:c r="H18" s="94" t="str">
+        <x:v>飞行范围火力兼多目标连锁保护者。</x:v>
+      </x:c>
+      <x:c r="I18" s="94" t="str">
+        <x:v>通过跨自身轮的弹药窗口、交替量子护盾和延迟超频形成节奏，防御立场保护队友但留下自身弱点。</x:v>
+      </x:c>
+      <x:c r="J18" s="94" t="str">
+        <x:v>导弹三发在两轮如何分配；敌友范围净收益；量子盾何时消耗启动下一轮禁用；立场覆盖哪些队友；喷射落点与下轮攻击机会。</x:v>
+      </x:c>
+      <x:c r="K18" s="94" t="str">
+        <x:v>自身回合先按局面强化/机动再挑有净收益区域；导弹首用开窗口；结束后立场保护其他队友；各敌将回合独立刷新离子/量子施放次数；下次己方开始应用超频与窗口计时。</x:v>
+      </x:c>
+      <x:c r="L18" s="94" t="str">
+        <x:v>等级8钢机甲勇者攻4守4速3范3魔0。机枪0每自身回合1；导弹0每首用起2自身轮3发；激光0冷却3自身轮；机甲强化0冷却3自身轮守+1持续2轮回血.5；喷射0每自身回合1；立场0冷却2轮；离子每敌将回合2，量子可用轮每敌将回合3。</x:v>
+      </x:c>
+      <x:c r="M18" s="94" t="str">
+        <x:v>敌方连锁使伤害未兑现时，下次己方开始永久增加对应技能未来次数；导弹正在持续的窗口也受益。飞行调整范围覆盖，强化自保，立场与连锁护盾分担队友防护。</x:v>
+      </x:c>
+      <x:c r="N18" s="94" t="str">
+        <x:v>零魔技能、多发范围火力、多个敌将回合分别有保护次数、受阻后永久成长。</x:v>
+      </x:c>
+      <x:c r="O18" s="94" t="str">
+        <x:v>范围伤害会伤友；量子下一整轮空档，立场不护己且延后启动，冷却火力存在间隙。</x:v>
+      </x:c>
+      <x:c r="P18" s="94" t="str">
+        <x:v>无连锁走位避免超频、集中攻击翡翠本体、利用量子空档、迫使范围包含队友。</x:v>
+      </x:c>
+      <x:c r="Q18" s="94" t="str">
+        <x:v>按实际敌友伤害和新防护价值选区；保留量子应对离子不足/收益更大的威胁，立场按队友当前与潜在位置估值；喷射比较最终位置且遵守移动限制。</x:v>
+      </x:c>
+      <x:c r="R18" s="94" t="str">
+        <x:v>["有效击破与敌友净范围伤害","无浪费的导弹窗口使用","低血强化","多受威胁盟友一次支援","有保护对象的立场"]</x:v>
+      </x:c>
+      <x:c r="S18" s="94" t="str">
+        <x:v>["为超频故意空放或伤友","将已免疫目标算有效输出","在量子禁用轮使用","把其他敌将回合扣作自己的窗口/冷却","无队友仍放立场"]</x:v>
+      </x:c>
+      <x:c r="T18" s="94" t="str">
+        <x:v>跨轮窗口和永久增长需要独立计时；防护技能评价应扣除已免疫/已足够护盾目标，移动技能和范围火力一起评估。</x:v>
+      </x:c>
+      <x:c r="U18" s="94" t="str">
+        <x:v>导弹2×2、激光2×10或10×2远程范围边缘截断，当前攻不破魔；机枪遵循通用敌军直线。离子/量子一施放可选多个当前受威胁的范内直线盟友，每目标一层到连锁结束。量子使用当轮仍可在不同敌将回合使用，下一自身轮整轮禁止，再下一轮恢复。立场随翡翠动态7×7，本回合结束后至下次自身开始保护其他盟友，只挡伤害不挡效果。</x:v>
+      </x:c>
+      <x:c r="V18" s="94" t="str">
+        <x:v>超频要求本技能原本命中的至少一个敌方目标最终没有伤害、对方实际连锁；同回合每技能一次；下次自身开始生效。导弹增量永久进入后续窗口，现窗口未过期也补增量。喷射直线5格或边缘末格，穿单位但完整落点合法且不能移动时不可用。</x:v>
+      </x:c>
+      <x:c r="W18" s="94" t="str">
+        <x:v>按下列源规则推定明确，无待用户回答项。</x:v>
+      </x:c>
+      <x:c r="X18" s="94" t="str">
+        <x:v>["不同敌将回合护盾次数独立","量子下一整轮禁用","导弹剩余与窗口到期可见","连锁后超频排队并下次自己回合生效","立场跟随/不护本体"]</x:v>
+      </x:c>
+      <x:c r="Y18" s="94" t="str">
+        <x:v>["旧两任意回合冷却","量子次数误作整轮","重复/伤害已造成仍超频","立场罩自己或挡非伤害","移动后重算已声明远程区"]</x:v>
+      </x:c>
+      <x:c r="Z18" s="94" t="str">
+        <x:v>武将说明§11、通用规则§2与§10明确每敌将回合；hero-rule-index与最新规则优先于project-map历史段落中per own cycle字样。</x:v>
+      </x:c>
+      <x:c r="AA18" s="94" t="str">
+        <x:v>设计基线已锁定；等待本批战斗、AI、测试逐项核对。</x:v>
+      </x:c>
+      <x:c r="AB18" s="94" t="str">
+        <x:v>[{"topic":"有冷却技能的超频次数","decision":"每永久+1提供同一可用轮额外一次施放，仍保留原冷却轮数；当轮的额外次数不被首次施放立即关闭。","reasoning":"特性写带伤害技能并未排除激光，必须同时兑现次数永久增加与激光冷却3轮。","rejected_alternatives":"不让激光超频成为无效果，也不删除冷却变成每轮额外无限火力。","confidence":"中","gameplay_consequence":"激光可在可用轮按增长次数连发，随后仍等待冷却。"}]</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="260" customHeight="1">
+      <x:c r="A19" s="94" t="str">
+        <x:v>R04</x:v>
+      </x:c>
+      <x:c r="B19" s="94"/>
+      <x:c r="C19" s="94" t="str">
+        <x:v>n</x:v>
+      </x:c>
+      <x:c r="D19" s="94" t="str">
+        <x:v>N</x:v>
+      </x:c>
+      <x:c r="E19" s="94" t="str">
+        <x:v>仅使用武将说明§10–12、通用规则/技能与持久索引；问卷已按三名精确匹配确认无保存答案。先写入JSON及XLSX后才读本批战斗、AI、测试；代码不作设计来源。</x:v>
+      </x:c>
+      <x:c r="F19" s="94" t="str">
+        <x:v>2026-09-10</x:v>
+      </x:c>
+      <x:c r="G19" s="94" t="str">
+        <x:v>把普攻转换为魔力点，再转为无上限魔储备，形成护体、连攻和随时打断的资源循环。</x:v>
+      </x:c>
+      <x:c r="H19" s="94" t="str">
+        <x:v>近战资源成长勇者，靠每段耗魔免伤与磁力波控制行动节奏。</x:v>
+      </x:c>
+      <x:c r="I19" s="94" t="str">
+        <x:v>当前魔同时决定下轮攻击数与承伤次数；魔力点在即刻回魔、存2点随时打断之间取舍，分身以结束本轮输出换逃生。</x:v>
+      </x:c>
+      <x:c r="J19" s="94" t="str">
+        <x:v>当轮固定攻击次数如何转资源；存磁力波还是补护体魔；耗1.5魔穿刺/分身是否值得；磁力波选区净伤害与是否能打断真正当前单位。</x:v>
+      </x:c>
+      <x:c r="K19" s="94" t="str">
+        <x:v>自身开始按floor当前魔+1锁攻击上限；有效攻击或受阻声明均加1魔力点；攻击间把点转魔不能增加当轮攻击数；对方行动时可速度3磁力波；行动用尽或生存需要才分身结束自身行动。</x:v>
+      </x:c>
+      <x:c r="L19" s="94" t="str">
+        <x:v>等级4光人类勇者攻2守3速3范1魔2；保护1魔每敌将回合一次；穿刺1.5魔每自身回合2次；分身1.5魔每自身回合一次；磁力波2魔力点每个武将回合一次；N花1魔力点换1当前魔不限次；当前魔及显示上限不封顶。</x:v>
+      </x:c>
+      <x:c r="M19" s="94" t="str">
+        <x:v>普攻声明即产点支持被护盾挡下时仍成长；N技能补魔既增未来攻击又提供逐段免伤；磁力波抢速阻断当前行动但消耗回魔资源；分身配合随机换位脱险。</x:v>
+      </x:c>
+      <x:c r="N19" s="94" t="str">
+        <x:v>储备足够时逐段无伤、可持续增长攻击与魔、速度3区域打断、信息一致的三分身。</x:v>
+      </x:c>
+      <x:c r="O19" s="94" t="str">
+        <x:v>每段伤害消耗魔且效果仍能命中，范1限制普通攻击，花魔技能削弱防护，回合中补魔不会立即增加普攻。</x:v>
+      </x:c>
+      <x:c r="P19" s="94" t="str">
+        <x:v>多段伤害耗魔、零伤害控制/禁技能、范围覆盖真身与分身，诱导提前消耗磁力波。</x:v>
+      </x:c>
+      <x:c r="Q19" s="94" t="str">
+        <x:v>保留有效普通攻击带来的产点机会；比较补魔防守/下轮收益和磁力波打断，分身不能随意放弃剩余有效攻击；用真实合法目标且不透视敌方真假。</x:v>
+      </x:c>
+      <x:c r="R19" s="94" t="str">
+        <x:v>["能击破或打断的磁力波","能兑现的普攻产点","不足护体时N回魔","净收益穿刺/吸魔","行动末或逃生分身"]</x:v>
+      </x:c>
+      <x:c r="S19" s="94" t="str">
+        <x:v>["把回合中增魔换算为新增攻击","把磁力波控制非当前单位算持续到其下回合","把当前魔与魔力点混用","每回合一开始就分身浪费输出","识别敌方分身内部标记"]</x:v>
+      </x:c>
+      <x:c r="T19" s="94" t="str">
+        <x:v>双资源分别估价并保留即时反应预算；减伤探查不能真实扣资源；控制收益取决于被控者此刻剩余行动。</x:v>
+      </x:c>
+      <x:c r="U19" s="94" t="str">
+        <x:v>每次声明普攻加1点包括落空/护盾，开始快照floor当前魔+1。当前魔&gt;0则每次伤害被取消并魔-1，非伤害附带效果继续，分数魔最低归零。磁力波原3×3远程区当前攻伤害；只让实际被效果命中且此刻处于自己行动回合的单位本回合不能行动，不延后到下次。分身选范内3个合法空格，生3分身随机换位并结束本体，分身入场无行动、不可普攻/技能，对敌公开信息保持真身一致。</x:v>
+      </x:c>
+      <x:c r="V19" s="94" t="str">
+        <x:v>随时技能在每个武将回合独立刷新一次；速度3连锁规则照常；普通盾挡整个技能时不附加行动终止，N护体/其他仅伤害防御保留控制。三分身只需单格候选+required_cells3，不枚举组合。</x:v>
+      </x:c>
+      <x:c r="W19" s="94" t="str">
+        <x:v>按下列源规则推定明确，无待用户回答项。</x:v>
+      </x:c>
+      <x:c r="X19" s="94" t="str">
+        <x:v>["普攻声明就加点","本回合攻击上限不随魔改动","连续伤害分别扣魔","磁力波只禁当前行动单位","敌方不能从魔和技能文本辨真假"]</x:v>
+      </x:c>
+      <x:c r="Y19" s="94" t="str">
+        <x:v>["概率/探查偷改当前魔","无限回魔AI空转","先分身放弃普攻","多武将回合错误清理行动限制","原格选择被连锁位移重瞄"]</x:v>
+      </x:c>
+      <x:c r="Z19" s="94" t="str">
+        <x:v>武将说明§12；通用技能分身/穿刺/保护；通用规则§2、7–11、骑乘与格子结算；hero-rule-index/project-map明确声明产点、快照、每个武将回合磁力波及克隆公开信息。</x:v>
+      </x:c>
+      <x:c r="AA19" s="94" t="str">
+        <x:v>设计基线已锁定；等待本批战斗、AI、测试逐项核对。</x:v>
+      </x:c>
+      <x:c r="AB19" s="94" t="str">
+        <x:v>[{"topic":"分数魔免伤与磁力波后续","decision":"开始时任何正魔都可以承受一段，扣1后最低0；磁力波被仅伤害防护抵消后仍按实际当前行动对象施加行动终止。","reasoning":"源文明确大于0而非至少1，且只抵消伤害不抵消其他影响。","rejected_alternatives":"不要求整1魔，不产生负魔，不因免伤吞掉非伤害控制。","confidence":"高","gameplay_consequence":"资源边界可预测，控制能反制N的无伤。"}]</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5b3f4605549b4198"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2c9e1a6bcaf44859"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -23709,22 +23961,22 @@
     </x:row>
     <x:row r="2" ht="84" hidden="0" customHeight="1">
       <x:c r="A2" s="66" t="str">
-        <x:v>elite_soldier</x:v>
+        <x:v>undead_king_lina</x:v>
       </x:c>
       <x:c r="B2" s="66" t="str">
-        <x:v>精兵</x:v>
+        <x:v>不死王利娜</x:v>
       </x:c>
       <x:c r="C2" s="66" t="str">
-        <x:v>2026-09-09完成战斗、AI、预览与测试代码检查修改；静态检查通过，动态验证等待全部73名已开发武将完成后统一进行。</x:v>
+        <x:v>2026-09-10完成战斗、AI、预览及测试代码逐项检查修改；静态检查通过，动态验证等待全部已开发武将完成后统一运行。</x:v>
       </x:c>
       <x:c r="D2" s="66" t="str">
-        <x:v>战斗实现</x:v>
+        <x:v>战斗/生命周期</x:v>
       </x:c>
       <x:c r="E2" s="65" t="str">
-        <x:v>基础面板、方形普攻、机枪三格/贴边敌方限定、神速、爆头下一普攻与撤步逐项映射。</x:v>
+        <x:v>2×2面板、双攻半破魔、声明执念、合格击破再动与吸魔、天气回复及禁疗逐条核对。</x:v>
       </x:c>
       <x:c r="F2" s="65" t="str">
-        <x:v>first_five.py::EliteSoldier；common.py::PrecisionTrainingTrait/MachineGunSkill/HeadshotSkill/BackstepShotSkill/NextAttackBuffStatus。</x:v>
+        <x:v>next_five.py::UndeadKingLina/HalfPierceAttackTrait/AttackLockTrait/LinaDestroyRewardTrait/NoEnemyHealAuraTrait/LinaSandstormRecoveryTrait。</x:v>
       </x:c>
       <x:c r="G2" s="98" t="str">
         <x:v>已检查并修正，待统一动态验证</x:v>
@@ -23733,16 +23985,16 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="I2" s="65" t="str">
-        <x:v>概率减速限定普攻（含反击），机枪不抽签；减速独立破魔而非伤害破魔。撤步复用共享直线穿人两格可达路径，保留仅来源反击与每对方回合两次。</x:v>
+        <x:v>原执念会因目标暂离且position为空解除，奖励未排除场地伤害；现保留存活目标锁定，奖励限定带攻击/技能标识的直接伤害，禁疗光环不来自被放逐本体。既有半破魔、骑乘后实际对象锁定、双攻与剩余魔收益保留。</x:v>
       </x:c>
       <x:c r="J2" s="65" t="str">
         <x:v>代码与用例已更新；未运行动态测试</x:v>
       </x:c>
       <x:c r="K2" s="65" t="str">
-        <x:v>docs/武将设计思想.json#elite_soldier</x:v>
+        <x:v>docs/武将设计思想.json#undead_king_lina</x:v>
       </x:c>
       <x:c r="L2" s="65" t="str">
-        <x:v>先完成2026-09-08源规则独立基线并同步工作簿，随后逐个读取战斗、AI和测试；2026-09-09完成修正及静态检查，没有本轮动态运行结果。</x:v>
+        <x:v>2026-09-09三份源规则设计基线先写入JSON与XLSX，随后逐个读战斗、AI、测试和前端相关代码；2026-09-10静态复核。无本轮动态验证结果。</x:v>
       </x:c>
       <x:c r="M2" s="65" t="str">
         <x:v>2026-09-06用户调整：连续分批完成全部已开发武将及AI的设计优先检查修改；保留测试用例和静态检查，中途不运行测试、不等待逐批签收，全部完成后统一测试。</x:v>
@@ -23750,22 +24002,22 @@
     </x:row>
     <x:row r="3" ht="84" hidden="0" customHeight="1">
       <x:c r="A3" s="66" t="str">
-        <x:v>elite_soldier</x:v>
+        <x:v>undead_king_lina</x:v>
       </x:c>
       <x:c r="B3" s="66" t="str">
-        <x:v>精兵</x:v>
+        <x:v>不死王利娜</x:v>
       </x:c>
       <x:c r="C3" s="66" t="str">
-        <x:v>2026-09-09完成战斗、AI、预览与测试代码检查修改；静态检查通过，动态验证等待全部73名已开发武将完成后统一进行。</x:v>
+        <x:v>2026-09-10完成战斗、AI、预览及测试代码逐项检查修改；静态检查通过，动态验证等待全部已开发武将完成后统一运行。</x:v>
       </x:c>
       <x:c r="D3" s="66" t="str">
-        <x:v>AI</x:v>
+        <x:v>战斗/声明与天气</x:v>
       </x:c>
       <x:c r="E3" s="65" t="str">
-        <x:v>爆头失去方形射程的代价、可兑现射击收益、随机公平性和撤步脱离原选区。</x:v>
+        <x:v>撕裂、风沙、狂沙声明区固定；狂沙完整身体落点合法，2己方轮冷却；风沙一轮不被多人回合缩短。</x:v>
       </x:c>
       <x:c r="F3" s="65" t="str">
-        <x:v>ai.py::self_buff_score/best_available_attack_score/score_reaction_payload/ai_probe_rollback。</x:v>
+        <x:v>next_five.py::RendingSkill/WindSandSkill/CrazySandSkill/SandstormWeatherEffect；core.py自身回合时钟。</x:v>
       </x:c>
       <x:c r="G3" s="98" t="str">
         <x:v>已检查并修正，待统一动态验证</x:v>
@@ -23774,16 +24026,16 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="I3" s="65" t="str">
-        <x:v>爆头前后探测实际合法普攻并比较收益，探测期间不抽取概率减速；撤步降低仍留在原作用区的落点评分。</x:v>
+        <x:v>狂沙冷却4改2，禁止无法移动时施放，伤害线及落点声明锁定，连锁占据落点只取消位移；风沙到来源下次己方开始自然回复后到期，天气每目标自身结束一次。</x:v>
       </x:c>
       <x:c r="J3" s="65" t="str">
         <x:v>代码与用例已更新；未运行动态测试</x:v>
       </x:c>
       <x:c r="K3" s="65" t="str">
-        <x:v>docs/武将设计思想.json#elite_soldier</x:v>
+        <x:v>docs/武将设计思想.json#undead_king_lina</x:v>
       </x:c>
       <x:c r="L3" s="65" t="str">
-        <x:v>先完成2026-09-08源规则独立基线并同步工作簿，随后逐个读取战斗、AI和测试；2026-09-09完成修正及静态检查，没有本轮动态运行结果。</x:v>
+        <x:v>2026-09-09三份源规则设计基线先写入JSON与XLSX，随后逐个读战斗、AI、测试和前端相关代码；2026-09-10静态复核。无本轮动态验证结果。</x:v>
       </x:c>
       <x:c r="M3" s="65" t="str">
         <x:v>2026-09-06用户调整：连续分批完成全部已开发武将及AI的设计优先检查修改；保留测试用例和静态检查，中途不运行测试、不等待逐批签收，全部完成后统一测试。</x:v>
@@ -23791,22 +24043,22 @@
     </x:row>
     <x:row r="4" ht="84" hidden="0" customHeight="1">
       <x:c r="A4" s="66" t="str">
-        <x:v>elite_soldier</x:v>
+        <x:v>undead_king_lina</x:v>
       </x:c>
       <x:c r="B4" s="66" t="str">
-        <x:v>精兵</x:v>
+        <x:v>不死王利娜</x:v>
       </x:c>
       <x:c r="C4" s="66" t="str">
-        <x:v>2026-09-09完成战斗、AI、预览与测试代码检查修改；静态检查通过，动态验证等待全部73名已开发武将完成后统一进行。</x:v>
+        <x:v>2026-09-10完成战斗、AI、预览及测试代码逐项检查修改；静态检查通过，动态验证等待全部已开发武将完成后统一运行。</x:v>
       </x:c>
       <x:c r="D4" s="66" t="str">
-        <x:v>前端/连锁</x:v>
+        <x:v>AI/预览</x:v>
       </x:c>
       <x:c r="E4" s="65" t="str">
-        <x:v>机枪不能为友军开启反应，前端预览与AI均使用同一效果单位集合；撤步合法路径一致。</x:v>
+        <x:v>狂沙载荷必须包含真实落点并兼顾伤害/安全；执念承诺、合格再动、天气净敌友收益与实际回复。</x:v>
       </x:c>
       <x:c r="F4" s="65" t="str">
-        <x:v>core.py::Skill.excludes_allies_from_effect/build_queued_action；ai.py::skill_effect_units；BackstepShotSkill.preview/retreat_cells。</x:v>
+        <x:v>ai.py::skill_payloads_for_action/reviewed_attack_synergy/sandstorm_value/skill_damage_score；CrazySandSkill.preview；targeting.js::computeHighlights。</x:v>
       </x:c>
       <x:c r="G4" s="98" t="str">
         <x:v>已检查并修正，待统一动态验证</x:v>
@@ -23815,16 +24067,16 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="I4" s="65" t="str">
-        <x:v>新增共享友军排除标志并接入机枪；保留已有连续直线选格和后续仅来源反击流程。</x:v>
+        <x:v>原狂沙仅选区载荷无落点导致AI负评分；现前端和AI共用pattern_destinations与四格落点。普攻考虑新锁定代价，普攻/技能击破合格目标奖励再动；天气回复通过实际治疗探测判断禁疗。</x:v>
       </x:c>
       <x:c r="J4" s="65" t="str">
         <x:v>代码与用例已更新；未运行动态测试</x:v>
       </x:c>
       <x:c r="K4" s="65" t="str">
-        <x:v>docs/武将设计思想.json#elite_soldier</x:v>
+        <x:v>docs/武将设计思想.json#undead_king_lina</x:v>
       </x:c>
       <x:c r="L4" s="65" t="str">
-        <x:v>先完成2026-09-08源规则独立基线并同步工作簿，随后逐个读取战斗、AI和测试；2026-09-09完成修正及静态检查，没有本轮动态运行结果。</x:v>
+        <x:v>2026-09-09三份源规则设计基线先写入JSON与XLSX，随后逐个读战斗、AI、测试和前端相关代码；2026-09-10静态复核。无本轮动态验证结果。</x:v>
       </x:c>
       <x:c r="M4" s="65" t="str">
         <x:v>2026-09-06用户调整：连续分批完成全部已开发武将及AI的设计优先检查修改；保留测试用例和静态检查，中途不运行测试、不等待逐批签收，全部完成后统一测试。</x:v>
@@ -23832,22 +24084,22 @@
     </x:row>
     <x:row r="5" ht="84" hidden="0" customHeight="1">
       <x:c r="A5" s="66" t="str">
-        <x:v>elite_soldier</x:v>
+        <x:v>undead_king_lina</x:v>
       </x:c>
       <x:c r="B5" s="66" t="str">
-        <x:v>精兵</x:v>
+        <x:v>不死王利娜</x:v>
       </x:c>
       <x:c r="C5" s="66" t="str">
-        <x:v>2026-09-09完成战斗、AI、预览与测试代码检查修改；静态检查通过，动态验证等待全部73名已开发武将完成后统一进行。</x:v>
+        <x:v>2026-09-10完成战斗、AI、预览及测试代码逐项检查修改；静态检查通过，动态验证等待全部已开发武将完成后统一运行。</x:v>
       </x:c>
       <x:c r="D5" s="66" t="str">
         <x:v>测试</x:v>
       </x:c>
       <x:c r="E5" s="65" t="str">
-        <x:v>方形射程、强化只消费一次、技能不触发减速、有盾减速及被动边界有确定性覆盖。</x:v>
+        <x:v>多人天气计时/己方伤害、暂离执念、场地击破不再动、连锁受阻狂沙、AI与完整落点预览。</x:v>
       </x:c>
       <x:c r="F5" s="65" t="str">
-        <x:v>tests/test_behavior.py::DevelopedHeroReviewR02BehaviorTests前两项；test_battle.py既有headshot/precision/backstep边界用例。</x:v>
+        <x:v>tests/test_behavior.py::DevelopedHeroReviewR03BehaviorTests；test_battle.py既有利娜面板/半破魔/多格伤害/骑乘锁定/击破奖励。</x:v>
       </x:c>
       <x:c r="G5" s="98" t="str">
         <x:v>已检查并修正，待统一动态验证</x:v>
@@ -23856,16 +24108,16 @@
         <x:v>P2</x:v>
       </x:c>
       <x:c r="I5" s="65" t="str">
-        <x:v>新增机枪无随机、无友军目标，以及爆头射程退化/有盾正向机会与探测状态回滚用例。只写用例，未运行动态测试。</x:v>
+        <x:v>新增对应确定性场景，保留已有正常成功边界。此轮仅静态检查，未运行用例。</x:v>
       </x:c>
       <x:c r="J5" s="65" t="str">
         <x:v>代码与用例已更新；未运行动态测试</x:v>
       </x:c>
       <x:c r="K5" s="65" t="str">
-        <x:v>docs/武将设计思想.json#elite_soldier</x:v>
+        <x:v>docs/武将设计思想.json#undead_king_lina</x:v>
       </x:c>
       <x:c r="L5" s="65" t="str">
-        <x:v>先完成2026-09-08源规则独立基线并同步工作簿，随后逐个读取战斗、AI和测试；2026-09-09完成修正及静态检查，没有本轮动态运行结果。</x:v>
+        <x:v>2026-09-09三份源规则设计基线先写入JSON与XLSX，随后逐个读战斗、AI、测试和前端相关代码；2026-09-10静态复核。无本轮动态验证结果。</x:v>
       </x:c>
       <x:c r="M5" s="65" t="str">
         <x:v>2026-09-06用户调整：连续分批完成全部已开发武将及AI的设计优先检查修改；保留测试用例和静态检查，中途不运行测试、不等待逐批签收，全部完成后统一测试。</x:v>
@@ -23873,22 +24125,22 @@
     </x:row>
     <x:row r="6" ht="84" hidden="0" customHeight="1">
       <x:c r="A6" s="66" t="str">
-        <x:v>bard</x:v>
+        <x:v>rock_god</x:v>
       </x:c>
       <x:c r="B6" s="66" t="str">
-        <x:v>吟游诗人</x:v>
+        <x:v>岩神</x:v>
       </x:c>
       <x:c r="C6" s="66" t="str">
-        <x:v>2026-09-09完成战斗、AI、预览与测试代码检查修改；静态检查通过，动态验证等待全部73名已开发武将完成后统一进行。</x:v>
+        <x:v>2026-09-10完成战斗、AI、预览及测试代码逐项检查修改；静态检查通过，动态验证等待全部已开发武将完成后统一运行。</x:v>
       </x:c>
       <x:c r="D6" s="66" t="str">
-        <x:v>战斗实现</x:v>
+        <x:v>战斗/能力与身体</x:v>
       </x:c>
       <x:c r="E6" s="65" t="str">
-        <x:v>守*2同源不叠加；回血反转；洗礼1轮人类目标；吟唱只加魔力点；原地回复检查所有位移。</x:v>
+        <x:v>岩吸五属性、同次交换统一到期、盾按目标阻挡、最低属性仍计收益、完整连通增长与受阻恢复。</x:v>
       </x:c>
       <x:c r="F6" s="65" t="str">
-        <x:v>first_five.py::Bard；common.py::DefendTwiceSkill/HealSkill/BaptismSkill/ChantSkill/StationaryRecoveryTrait；core.py::move_unit。</x:v>
+        <x:v>next_five.py::RockAbsorbSkill/RockAbsorbStatStatus/RockAbsorbLinkStatus/RockAbsorbFootprintStatus。</x:v>
       </x:c>
       <x:c r="G6" s="98" t="str">
         <x:v>已检查并修正，待统一动态验证</x:v>
@@ -23897,16 +24149,16 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="I6" s="65" t="str">
-        <x:v>补齐暗属性/灵体/恶魔回血反转；拒绝同源守*2重复施放；强制或连锁移动也取消原地回复而不消耗普通移动次数。</x:v>
+        <x:v>原减值在各目标自身开始提前过期、非魔可能降到0、部分目标被盾挡后直接截取列表可能断体；现按源清理交换，非魔最低1，声明区及增长格固定，从选格中逐步增长保持连通，受阻格略过；源死亡清除交换。</x:v>
       </x:c>
       <x:c r="J6" s="65" t="str">
         <x:v>代码与用例已更新；未运行动态测试</x:v>
       </x:c>
       <x:c r="K6" s="65" t="str">
-        <x:v>docs/武将设计思想.json#bard</x:v>
+        <x:v>docs/武将设计思想.json#rock_god</x:v>
       </x:c>
       <x:c r="L6" s="65" t="str">
-        <x:v>先完成2026-09-08源规则独立基线并同步工作簿，随后逐个读取战斗、AI和测试；2026-09-09完成修正及静态检查，没有本轮动态运行结果。</x:v>
+        <x:v>2026-09-09三份源规则设计基线先写入JSON与XLSX，随后逐个读战斗、AI、测试和前端相关代码；2026-09-10静态复核。无本轮动态验证结果。</x:v>
       </x:c>
       <x:c r="M6" s="65" t="str">
         <x:v>2026-09-06用户调整：连续分批完成全部已开发武将及AI的设计优先检查修改；保留测试用例和静态检查，中途不运行测试、不等待逐批签收，全部完成后统一测试。</x:v>
@@ -23914,22 +24166,22 @@
     </x:row>
     <x:row r="7" ht="84" hidden="0" customHeight="1">
       <x:c r="A7" s="66" t="str">
-        <x:v>bard</x:v>
+        <x:v>rock_god</x:v>
       </x:c>
       <x:c r="B7" s="66" t="str">
-        <x:v>吟游诗人</x:v>
+        <x:v>岩神</x:v>
       </x:c>
       <x:c r="C7" s="66" t="str">
-        <x:v>2026-09-09完成战斗、AI、预览与测试代码检查修改；静态检查通过，动态验证等待全部73名已开发武将完成后统一进行。</x:v>
+        <x:v>2026-09-10完成战斗、AI、预览及测试代码逐项检查修改；静态检查通过，动态验证等待全部已开发武将完成后统一运行。</x:v>
       </x:c>
       <x:c r="D7" s="66" t="str">
-        <x:v>场地/时序</x:v>
+        <x:v>战斗/炮击与天气</x:v>
       </x:c>
       <x:c r="E7" s="65" t="str">
-        <x:v>圣光跟随施法者11×11，只有敌方普通移动结束在场内受攻4伤害；友方仅自己的回合末加防；2.5轮不被多人回合缩短。</x:v>
+        <x:v>岩石炮逐弹连锁、方向/发射格固定、每弹按当前碰撞决定攻(3+弹数)3×3敌我伤害；身体至少一格且连通。</x:v>
       </x:c>
       <x:c r="F7" s="65" t="str">
-        <x:v>common.py::GreatHolyLightField/GreatHolyLightSkill；unit_belongs_to_current_turn及全占格判断。</x:v>
+        <x:v>next_five.py::RockCannonSkill.queue_projectile/resolve_projectile；RockGodSandstormAura；core.py::queue_skill_effect_action。</x:v>
       </x:c>
       <x:c r="G7" s="98" t="str">
         <x:v>已检查并修正，待统一动态验证</x:v>
@@ -23938,16 +24190,16 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="I7" s="65" t="str">
-        <x:v>将固定4生命扣减改为攻4公式；按施放者第三个己方回合末到期，守+1按受益者自己的回合结束授予且不叠加，放逐期间不生成场内效果。</x:v>
+        <x:v>原一次预计算所有弹体落点，后续连锁变化无效；改为前弹完成后计算下弹碰撞。声明时验证身体和方向；保留边界爆炸、不破魔与友伤。局部沙尘按单位自身结束，临时放逐不永久丢失光环来源，同回合全局/局部只伤一次。</x:v>
       </x:c>
       <x:c r="J7" s="65" t="str">
         <x:v>代码与用例已更新；未运行动态测试</x:v>
       </x:c>
       <x:c r="K7" s="65" t="str">
-        <x:v>docs/武将设计思想.json#bard</x:v>
+        <x:v>docs/武将设计思想.json#rock_god</x:v>
       </x:c>
       <x:c r="L7" s="65" t="str">
-        <x:v>先完成2026-09-08源规则独立基线并同步工作簿，随后逐个读取战斗、AI和测试；2026-09-09完成修正及静态检查，没有本轮动态运行结果。</x:v>
+        <x:v>2026-09-09三份源规则设计基线先写入JSON与XLSX，随后逐个读战斗、AI、测试和前端相关代码；2026-09-10静态复核。无本轮动态验证结果。</x:v>
       </x:c>
       <x:c r="M7" s="65" t="str">
         <x:v>2026-09-06用户调整：连续分批完成全部已开发武将及AI的设计优先检查修改；保留测试用例和静态检查，中途不运行测试、不等待逐批签收，全部完成后统一测试。</x:v>
@@ -23955,22 +24207,22 @@
     </x:row>
     <x:row r="8" ht="84" hidden="0" customHeight="1">
       <x:c r="A8" s="66" t="str">
-        <x:v>bard</x:v>
+        <x:v>rock_god</x:v>
       </x:c>
       <x:c r="B8" s="66" t="str">
-        <x:v>吟游诗人</x:v>
+        <x:v>岩神</x:v>
       </x:c>
       <x:c r="C8" s="66" t="str">
-        <x:v>2026-09-09完成战斗、AI、预览与测试代码检查修改；静态检查通过，动态验证等待全部73名已开发武将完成后统一进行。</x:v>
+        <x:v>2026-09-10完成战斗、AI、预览及测试代码逐项检查修改；静态检查通过，动态验证等待全部已开发武将完成后统一运行。</x:v>
       </x:c>
       <x:c r="D8" s="66" t="str">
-        <x:v>AI</x:v>
+        <x:v>AI/预览</x:v>
       </x:c>
       <x:c r="E8" s="65" t="str">
-        <x:v>真实治疗收益、不可治疗/满血/反转、魔力点接收者、重复防御与保留站位收益。</x:v>
+        <x:v>岩吸选择实际有效属性及合法增长，炮击命中、重复溅射、友伤和身体成本必须计分。</x:v>
       </x:c>
       <x:c r="F8" s="65" t="str">
-        <x:v>ai.py::score_skill_payload/ally_buff_score/field_skill_score/score_move_destination。</x:v>
+        <x:v>ai.py::rock_absorb_payloads/rock_cannon_payloads/resource_effect_score；targeting.js::statCellSelection/bodyDirectionSelection。</x:v>
       </x:c>
       <x:c r="G8" s="98" t="str">
         <x:v>已检查并修正，待统一动态验证</x:v>
@@ -23979,16 +24231,16 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="I8" s="65" t="str">
-        <x:v>用回滚执行探测实际回血；吟唱只奖励有魔力点用途的友军并按资源需求保留；圣光判断普通移动机会，移动评分计入放弃原地回复的代价。</x:v>
+        <x:v>原岩吸使用增长格当伤害区、炮击使用发射身体当目标导致错误估值；现回滚执行真实效果，逐弹评估，不运行反应。增长改为连通扩展避免组合爆炸；炮击增加相邻双格候选，空炮负分，保留原跟进队列。现有前端属性/增长/身体方向选择协议沿用。</x:v>
       </x:c>
       <x:c r="J8" s="65" t="str">
         <x:v>代码与用例已更新；未运行动态测试</x:v>
       </x:c>
       <x:c r="K8" s="65" t="str">
-        <x:v>docs/武将设计思想.json#bard</x:v>
+        <x:v>docs/武将设计思想.json#rock_god</x:v>
       </x:c>
       <x:c r="L8" s="65" t="str">
-        <x:v>先完成2026-09-08源规则独立基线并同步工作簿，随后逐个读取战斗、AI和测试；2026-09-09完成修正及静态检查，没有本轮动态运行结果。</x:v>
+        <x:v>2026-09-09三份源规则设计基线先写入JSON与XLSX，随后逐个读战斗、AI、测试和前端相关代码；2026-09-10静态复核。无本轮动态验证结果。</x:v>
       </x:c>
       <x:c r="M8" s="65" t="str">
         <x:v>2026-09-06用户调整：连续分批完成全部已开发武将及AI的设计优先检查修改；保留测试用例和静态检查，中途不运行测试、不等待逐批签收，全部完成后统一测试。</x:v>
@@ -23996,22 +24248,22 @@
     </x:row>
     <x:row r="9" ht="84" hidden="0" customHeight="1">
       <x:c r="A9" s="66" t="str">
-        <x:v>bard</x:v>
+        <x:v>rock_god</x:v>
       </x:c>
       <x:c r="B9" s="66" t="str">
-        <x:v>吟游诗人</x:v>
+        <x:v>岩神</x:v>
       </x:c>
       <x:c r="C9" s="66" t="str">
-        <x:v>2026-09-09完成战斗、AI、预览与测试代码检查修改；静态检查通过，动态验证等待全部73名已开发武将完成后统一进行。</x:v>
+        <x:v>2026-09-10完成战斗、AI、预览及测试代码逐项检查修改；静态检查通过，动态验证等待全部已开发武将完成后统一运行。</x:v>
       </x:c>
       <x:c r="D9" s="66" t="str">
         <x:v>测试</x:v>
       </x:c>
       <x:c r="E9" s="65" t="str">
-        <x:v>多人圣光时长、友军回合加防、普通/技能/强制移动、回血反转和魔力点用途。</x:v>
+        <x:v>部分加盾仍连通、属性最低值、源统一过期、后续炮弹读取反应后站位、全局局部天气不叠加与AI队列回滚。</x:v>
       </x:c>
       <x:c r="F9" s="65" t="str">
-        <x:v>tests/test_behavior.py::DevelopedHeroReviewR02BehaviorTests；test_battle.py既有圣光边界。</x:v>
+        <x:v>tests/test_behavior.py::DevelopedHeroReviewR03BehaviorTests；test_battle.py::rock_absorb/rock_cannon/same_named_sandstorm既有场景。</x:v>
       </x:c>
       <x:c r="G9" s="98" t="str">
         <x:v>已检查并修正，待统一动态验证</x:v>
@@ -24020,16 +24272,16 @@
         <x:v>P2</x:v>
       </x:c>
       <x:c r="I9" s="65" t="str">
-        <x:v>新增圣光公式/多人计时、强制移动取消回复、回血反转与禁疗、吟唱用途用例；死亡自动推进旧场景改为0.5生命，保持测试意图与正确公式一致。未运行动态测试。</x:v>
+        <x:v>新增边界场景，旧天气用例改为在受影响者自己的回合末断言。已有魔容量交换、隐身下保护、基础恢复受阻、炮线自挡、多弹连锁与龙息近身选格用例已读。未动态运行。</x:v>
       </x:c>
       <x:c r="J9" s="65" t="str">
         <x:v>代码与用例已更新；未运行动态测试</x:v>
       </x:c>
       <x:c r="K9" s="65" t="str">
-        <x:v>docs/武将设计思想.json#bard</x:v>
+        <x:v>docs/武将设计思想.json#rock_god</x:v>
       </x:c>
       <x:c r="L9" s="65" t="str">
-        <x:v>先完成2026-09-08源规则独立基线并同步工作簿，随后逐个读取战斗、AI和测试；2026-09-09完成修正及静态检查，没有本轮动态运行结果。</x:v>
+        <x:v>2026-09-09三份源规则设计基线先写入JSON与XLSX，随后逐个读战斗、AI、测试和前端相关代码；2026-09-10静态复核。无本轮动态验证结果。</x:v>
       </x:c>
       <x:c r="M9" s="65" t="str">
         <x:v>2026-09-06用户调整：连续分批完成全部已开发武将及AI的设计优先检查修改；保留测试用例和静态检查，中途不运行测试、不等待逐批签收，全部完成后统一测试。</x:v>
@@ -24037,22 +24289,22 @@
     </x:row>
     <x:row r="10" ht="84" hidden="0" customHeight="1">
       <x:c r="A10" s="66" t="str">
-        <x:v>element_hunter</x:v>
+        <x:v>doomlight_dragon</x:v>
       </x:c>
       <x:c r="B10" s="66" t="str">
-        <x:v>元素猎人</x:v>
+        <x:v>神龙。末日光</x:v>
       </x:c>
       <x:c r="C10" s="66" t="str">
-        <x:v>2026-09-09完成战斗、AI、预览与测试代码检查修改；静态检查通过，动态验证等待全部73名已开发武将完成后统一进行。</x:v>
+        <x:v>2026-09-10完成战斗、AI、预览及测试代码逐项检查修改；静态检查通过，动态验证等待全部已开发武将完成后统一运行。</x:v>
       </x:c>
       <x:c r="D10" s="66" t="str">
-        <x:v>战斗实现/控制</x:v>
+        <x:v>战斗/末日光生命周期</x:v>
       </x:c>
       <x:c r="E10" s="65" t="str">
-        <x:v>燃烧5次目标己方回合扣魔，暴风雪3轮仅禁普通移动；伤害与非伤害破魔分离；选区固定。</x:v>
+        <x:v>纯效果大招、反噬、四次目标自身减半、同名不刷新/首次来源保留、实际伤害吸收/超量生命/禁疗。</x:v>
       </x:c>
       <x:c r="F10" s="65" t="str">
-        <x:v>next_five.py::RemoteAreaDamageSkill/BurningManaStatus/blizzard_status_factory/PlantGrowthSkill；common.py::EllieWardTrait。</x:v>
+        <x:v>next_five.py::DoomLightStatus/DoomLightSkill/DoomLightRetaliationTrait；apply_piercing_status_effect(refresh_existing=False)；core.py::DamageContext.actual_damage/on_target_action_declared。</x:v>
       </x:c>
       <x:c r="G10" s="98" t="str">
         <x:v>已检查并修正，待统一动态验证</x:v>
@@ -24061,16 +24313,16 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="I10" s="65" t="str">
-        <x:v>声明时锁定选区；附加控制穿盾只打掉一盾，免伤仍允许非伤害控制，魔免仍阻止技能效果。燃烧/冰雪不叠同名状态；沿用目标自身计时。</x:v>
+        <x:v>原重复施加重置时长和来源，回调可能重复破盾，吸收按理论伤害；现已有状态不刷新，普攻声明即反噬，零伤技能不触发伤害反噬，tick不递归。新增实际伤害量在伤害后回复前记录，仅回复有效首次来源且仍经过禁疗。</x:v>
       </x:c>
       <x:c r="J10" s="65" t="str">
         <x:v>代码与用例已更新；未运行动态测试</x:v>
       </x:c>
       <x:c r="K10" s="65" t="str">
-        <x:v>docs/武将设计思想.json#element_hunter</x:v>
+        <x:v>docs/武将设计思想.json#doomlight_dragon</x:v>
       </x:c>
       <x:c r="L10" s="65" t="str">
-        <x:v>先完成2026-09-08源规则独立基线并同步工作簿，随后逐个读取战斗、AI和测试；2026-09-09完成修正及静态检查，没有本轮动态运行结果。</x:v>
+        <x:v>2026-09-09三份源规则设计基线先写入JSON与XLSX，随后逐个读战斗、AI、测试和前端相关代码；2026-09-10静态复核。无本轮动态验证结果。</x:v>
       </x:c>
       <x:c r="M10" s="65" t="str">
         <x:v>2026-09-06用户调整：连续分批完成全部已开发武将及AI的设计优先检查修改；保留测试用例和静态检查，中途不运行测试、不等待逐批签收，全部完成后统一测试。</x:v>
@@ -24078,22 +24330,22 @@
     </x:row>
     <x:row r="11" ht="84" hidden="0" customHeight="1">
       <x:c r="A11" s="66" t="str">
-        <x:v>element_hunter</x:v>
+        <x:v>doomlight_dragon</x:v>
       </x:c>
       <x:c r="B11" s="66" t="str">
-        <x:v>元素猎人</x:v>
+        <x:v>神龙。末日光</x:v>
       </x:c>
       <x:c r="C11" s="66" t="str">
-        <x:v>2026-09-09完成战斗、AI、预览与测试代码检查修改；静态检查通过，动态验证等待全部73名已开发武将完成后统一进行。</x:v>
+        <x:v>2026-09-10完成战斗、AI、预览及测试代码逐项检查修改；静态检查通过，动态验证等待全部已开发武将完成后统一运行。</x:v>
       </x:c>
       <x:c r="D11" s="66" t="str">
-        <x:v>召唤/增益/场地</x:v>
+        <x:v>战斗/技能边界</x:v>
       </x:c>
       <x:c r="E11" s="65" t="str">
-        <x:v>雷神面板、5轮寿命和敌方直接伤害死亡重置；水波4轮冷却与全五项+1；土行者3分身/随机换位/入场移动/下轮清理；植物双边起点耗点。</x:v>
+        <x:v>石墙、神速、变硬、远程龙息及末日的明确n、先付血、严格小于当前血、固定原选区、边缘截断与友伤。</x:v>
       </x:c>
       <x:c r="F11" s="65" t="str">
-        <x:v>next_five.py::ThunderGodSummon/ThunderGodSkill/WaterWaveSkill/AllStatsPlusStatus/EarthWalkerSkill/SplitSkill/EarthWalkerCleanupStatus/PlantGrowthField。</x:v>
+        <x:v>next_five.py::DoomlightDragon/RemoteDragonBreathSkill/ApocalypseSkill；common.py通用墙/神速/变硬；core.py::use_skill。</x:v>
       </x:c>
       <x:c r="G11" s="98" t="str">
         <x:v>已检查并修正，待统一动态验证</x:v>
@@ -24102,16 +24354,16 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="I11" s="65" t="str">
-        <x:v>雷神生命周期沿用已读实现；水波改4个己方回合冷却且到期收回魔容量；土行者复用通用3分身选择、显示与换位，覆盖入场权限和清理；植物按大型单位起点全占格判断。</x:v>
+        <x:v>末日声明锁定n与原区，不接受传入resolved_n覆盖明确选择，付血后施法者移位不重算范围；龙息锁区并采用实际技能名日志。共用ensure_distance及吟游诗人支援预览改为全占格距离。</x:v>
       </x:c>
       <x:c r="J11" s="65" t="str">
         <x:v>代码与用例已更新；未运行动态测试</x:v>
       </x:c>
       <x:c r="K11" s="65" t="str">
-        <x:v>docs/武将设计思想.json#element_hunter</x:v>
+        <x:v>docs/武将设计思想.json#doomlight_dragon</x:v>
       </x:c>
       <x:c r="L11" s="65" t="str">
-        <x:v>先完成2026-09-08源规则独立基线并同步工作簿，随后逐个读取战斗、AI和测试；2026-09-09完成修正及静态检查，没有本轮动态运行结果。</x:v>
+        <x:v>2026-09-09三份源规则设计基线先写入JSON与XLSX，随后逐个读战斗、AI、测试和前端相关代码；2026-09-10静态复核。无本轮动态验证结果。</x:v>
       </x:c>
       <x:c r="M11" s="65" t="str">
         <x:v>2026-09-06用户调整：连续分批完成全部已开发武将及AI的设计优先检查修改；保留测试用例和静态检查，中途不运行测试、不等待逐批签收，全部完成后统一测试。</x:v>
@@ -24119,22 +24371,22 @@
     </x:row>
     <x:row r="12" ht="84" hidden="0" customHeight="1">
       <x:c r="A12" s="66" t="str">
-        <x:v>element_hunter</x:v>
+        <x:v>doomlight_dragon</x:v>
       </x:c>
       <x:c r="B12" s="66" t="str">
-        <x:v>元素猎人</x:v>
+        <x:v>神龙。末日光</x:v>
       </x:c>
       <x:c r="C12" s="66" t="str">
-        <x:v>2026-09-09完成战斗、AI、预览与测试代码检查修改；静态检查通过，动态验证等待全部73名已开发武将完成后统一进行。</x:v>
+        <x:v>2026-09-10完成战斗、AI、预览及测试代码逐项检查修改；静态检查通过，动态验证等待全部已开发武将完成后统一运行。</x:v>
       </x:c>
       <x:c r="D12" s="66" t="str">
-        <x:v>AI/预览</x:v>
+        <x:v>AI/前端</x:v>
       </x:c>
       <x:c r="E12" s="65" t="str">
-        <x:v>三落点载荷、先兑现有效普攻再结束本体行动；控制不重复计新状态收益；场地敌友代价；水波增益不重复。</x:v>
+        <x:v>纯效果新感染收益、施法者禁疗导致吸收无效、末日生命成本/自伤友伤、显式n及安全余血。</x:v>
       </x:c>
       <x:c r="F12" s="65" t="str">
-        <x:v>ai.py::split_payloads/score_skill_payload/field_skill_score/self_buff_score/probe_skill_damage_impact；targeting.js::patternSelection/required_cells通用入口。</x:v>
+        <x:v>ai.py::resource_effect_score/reviewed_attack_synergy/skill_payloads_for_action；targeting.js::choicePatternSelection。</x:v>
       </x:c>
       <x:c r="G12" s="98" t="str">
         <x:v>已检查并修正，待统一动态验证</x:v>
@@ -24143,16 +24395,16 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="I12" s="65" t="str">
-        <x:v>土行者生成3个合法落点并保留有效普攻；只奖励新增控制，燃烧/冰雪伤害探测不错误破盾且包含附加效果；植物考虑友军拖累，水波检查现有状态与交战距离。前端复用三格选择协议。</x:v>
+        <x:v>原大招按普通即时伤害并重复奖励感染，末日忽略n生命费用；现探测实际效果和生命支付，拒绝重复感染、惩罚低血继续作战、允许实际终结正向边界；保留显式choice_code和截断选区。</x:v>
       </x:c>
       <x:c r="J12" s="65" t="str">
         <x:v>代码与用例已更新；未运行动态测试</x:v>
       </x:c>
       <x:c r="K12" s="65" t="str">
-        <x:v>docs/武将设计思想.json#element_hunter</x:v>
+        <x:v>docs/武将设计思想.json#doomlight_dragon</x:v>
       </x:c>
       <x:c r="L12" s="65" t="str">
-        <x:v>先完成2026-09-08源规则独立基线并同步工作簿，随后逐个读取战斗、AI和测试；2026-09-09完成修正及静态检查，没有本轮动态运行结果。</x:v>
+        <x:v>2026-09-09三份源规则设计基线先写入JSON与XLSX，随后逐个读战斗、AI、测试和前端相关代码；2026-09-10静态复核。无本轮动态验证结果。</x:v>
       </x:c>
       <x:c r="M12" s="65" t="str">
         <x:v>2026-09-06用户调整：连续分批完成全部已开发武将及AI的设计优先检查修改；保留测试用例和静态检查，中途不运行测试、不等待逐批签收，全部完成后统一测试。</x:v>
@@ -24160,22 +24412,22 @@
     </x:row>
     <x:row r="13" ht="84" hidden="0" customHeight="1">
       <x:c r="A13" s="66" t="str">
-        <x:v>element_hunter</x:v>
+        <x:v>doomlight_dragon</x:v>
       </x:c>
       <x:c r="B13" s="66" t="str">
-        <x:v>元素猎人</x:v>
+        <x:v>神龙。末日光</x:v>
       </x:c>
       <x:c r="C13" s="66" t="str">
-        <x:v>2026-09-09完成战斗、AI、预览与测试代码检查修改；静态检查通过，动态验证等待全部73名已开发武将完成后统一进行。</x:v>
+        <x:v>2026-09-10完成战斗、AI、预览及测试代码逐项检查修改；静态检查通过，动态验证等待全部已开发武将完成后统一运行。</x:v>
       </x:c>
       <x:c r="D13" s="66" t="str">
-        <x:v>测试</x:v>
+        <x:v>测试/共享交互</x:v>
       </x:c>
       <x:c r="E13" s="65" t="str">
-        <x:v>控制穿盾/艾莉免伤、冷却与魔容量、雷神死亡来源和三分身生命周期。</x:v>
+        <x:v>首次来源/不刷新/只破一盾、伤害后恢复不抹掉真实吸收、声明反噬、付血锁区与AI负/正向使用边界。</x:v>
       </x:c>
       <x:c r="F13" s="65" t="str">
-        <x:v>tests/test_behavior.py::DevelopedHeroReviewR02BehaviorTests后四项；test_battle.py及既有行为场景的土行者、植物、燃烧、冰雪生命周期用例。</x:v>
+        <x:v>tests/test_behavior.py::DevelopedHeroReviewR03BehaviorTests及R02回血反转用例；test_battle.py既有吸收超量与n=1/1.25严格边界。</x:v>
       </x:c>
       <x:c r="G13" s="98" t="str">
         <x:v>已检查并修正，待统一动态验证</x:v>
@@ -24184,16 +24436,16 @@
         <x:v>P2</x:v>
       </x:c>
       <x:c r="I13" s="65" t="str">
-        <x:v>新增免伤但控制生效/一盾消费与AI回滚、水波自己回合计时、土行者3落点和先攻击、雷神敌方/己方/场地/无来源死亡矩阵；更新旧单分身场景。未运行动态测试。</x:v>
+        <x:v>新增确定性场景及AI回滚断言；另按通用规则8.3修正R02回血反转仍受护盾等防御，并覆盖大型友军支援距离。未动态运行。</x:v>
       </x:c>
       <x:c r="J13" s="65" t="str">
         <x:v>代码与用例已更新；未运行动态测试</x:v>
       </x:c>
       <x:c r="K13" s="65" t="str">
-        <x:v>docs/武将设计思想.json#element_hunter</x:v>
+        <x:v>docs/武将设计思想.json#doomlight_dragon</x:v>
       </x:c>
       <x:c r="L13" s="65" t="str">
-        <x:v>先完成2026-09-08源规则独立基线并同步工作簿，随后逐个读取战斗、AI和测试；2026-09-09完成修正及静态检查，没有本轮动态运行结果。</x:v>
+        <x:v>2026-09-09三份源规则设计基线先写入JSON与XLSX，随后逐个读战斗、AI、测试和前端相关代码；2026-09-10静态复核。无本轮动态验证结果。</x:v>
       </x:c>
       <x:c r="M13" s="65" t="str">
         <x:v>2026-09-06用户调整：连续分批完成全部已开发武将及AI的设计优先检查修改；保留测试用例和静态检查，中途不运行测试、不等待逐批签收，全部完成后统一测试。</x:v>
@@ -24201,22 +24453,22 @@
     </x:row>
     <x:row r="14" ht="84" hidden="0" customHeight="1">
       <x:c r="A14" s="66" t="str">
-        <x:v>ellie</x:v>
+        <x:v>elite_soldier</x:v>
       </x:c>
       <x:c r="B14" s="66" t="str">
-        <x:v>艾莉</x:v>
+        <x:v>精兵</x:v>
       </x:c>
       <x:c r="C14" s="66" t="str">
-        <x:v>2026-09-08完成规则、战斗、AI、预览及测试代码检查和修改；动态验证等待全部已开发武将完成后统一运行。</x:v>
+        <x:v>2026-09-09完成战斗、AI、预览与测试代码检查修改；静态检查通过，动态验证等待全部73名已开发武将完成后统一进行。</x:v>
       </x:c>
       <x:c r="D14" s="66" t="str">
         <x:v>战斗实现</x:v>
       </x:c>
       <x:c r="E14" s="65" t="str">
-        <x:v>面板、魔墙、吸魔、牵引、诅咒、实验、水晶球、美杜莎及特性逐项映射。</x:v>
+        <x:v>基础面板、方形普攻、机枪三格/贴边敌方限定、神速、爆头下一普攻与撤步逐项映射。</x:v>
       </x:c>
       <x:c r="F14" s="65" t="str">
-        <x:v>first_five.py::Ellie/ManaPullSkill/CurseSkill/ExperimentSkill/CrystalBallSkill/MedusaSkill；common.py::EllieWardTrait/ExperimentCountdownStatus；core.py::summon_unit/cleanup_dead_units。</x:v>
+        <x:v>first_five.py::EliteSoldier；common.py::PrecisionTrainingTrait/MachineGunSkill/HeadshotSkill/BackstepShotSkill/NextAttackBuffStatus。</x:v>
       </x:c>
       <x:c r="G14" s="98" t="str">
         <x:v>已检查并修正，待统一动态验证</x:v>
@@ -24225,16 +24477,16 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="I14" s="65" t="str">
-        <x:v>牵引按目标原占格收集反应；诅咒固定0.5生命在声明时支付；实验增加魔力上限并补2魔。魔墙、吸魔、四轮水晶球、四攻召唤物及召唤者死亡级联沿用已读共用实现。 2026-09-09交互补查：EllieWardTrait只取消伤害，保留非伤害后续效果；元素控制用例覆盖此边界。</x:v>
+        <x:v>概率减速限定普攻（含反击），机枪不抽签；减速独立破魔而非伤害破魔。撤步复用共享直线穿人两格可达路径，保留仅来源反击与每对方回合两次。</x:v>
       </x:c>
       <x:c r="J14" s="65" t="str">
         <x:v>代码与用例已更新；未运行动态测试</x:v>
       </x:c>
       <x:c r="K14" s="65" t="str">
-        <x:v>docs/武将设计思想.json#ellie</x:v>
+        <x:v>docs/武将设计思想.json#elite_soldier</x:v>
       </x:c>
       <x:c r="L14" s="65" t="str">
-        <x:v>本轮依据源码和既有测试代码逐项检查；2026-09-08静态语法/格式检查，尚无本轮动态对局或回归结果。</x:v>
+        <x:v>先完成2026-09-08源规则独立基线并同步工作簿，随后逐个读取战斗、AI和测试；2026-09-09完成修正及静态检查，没有本轮动态运行结果。</x:v>
       </x:c>
       <x:c r="M14" s="65" t="str">
         <x:v>2026-09-06用户调整：连续分批完成全部已开发武将及AI的设计优先检查修改；保留测试用例和静态检查，中途不运行测试、不等待逐批签收，全部完成后统一测试。</x:v>
@@ -24242,22 +24494,22 @@
     </x:row>
     <x:row r="15" ht="84" hidden="0" customHeight="1">
       <x:c r="A15" s="66" t="str">
-        <x:v>ellie</x:v>
+        <x:v>elite_soldier</x:v>
       </x:c>
       <x:c r="B15" s="66" t="str">
-        <x:v>艾莉</x:v>
+        <x:v>精兵</x:v>
       </x:c>
       <x:c r="C15" s="66" t="str">
-        <x:v>2026-09-08完成规则、战斗、AI、预览及测试代码检查和修改；动态验证等待全部已开发武将完成后统一运行。</x:v>
+        <x:v>2026-09-09完成战斗、AI、预览与测试代码检查修改；静态检查通过，动态验证等待全部73名已开发武将完成后统一进行。</x:v>
       </x:c>
       <x:c r="D15" s="66" t="str">
         <x:v>AI</x:v>
       </x:c>
       <x:c r="E15" s="65" t="str">
-        <x:v>自损、延迟死亡、真实射程与友敌位移收益必须进入判断。</x:v>
+        <x:v>爆头失去方形射程的代价、可兑现射击收益、随机公平性和撤步脱离原选区。</x:v>
       </x:c>
       <x:c r="F15" s="65" t="str">
-        <x:v>ai.py::skill_payloads_for_action/score_skill_payload/ally_buff_score/self_buff_score；原牵引缺少落点参数，诅咒和实验按廉价伤害/增益评分。</x:v>
+        <x:v>ai.py::self_buff_score/best_available_attack_score/score_reaction_payload/ai_probe_rollback。</x:v>
       </x:c>
       <x:c r="G15" s="98" t="str">
         <x:v>已检查并修正，待统一动态验证</x:v>
@@ -24266,16 +24518,16 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="I15" s="65" t="str">
-        <x:v>牵引枚举后端落点并比较目标站位净收益；诅咒拒绝致命支付/重复诅咒；实验保留能立即结束战斗的正向边界；水晶球只为新增射程计分。</x:v>
+        <x:v>爆头前后探测实际合法普攻并比较收益，探测期间不抽取概率减速；撤步降低仍留在原作用区的落点评分。</x:v>
       </x:c>
       <x:c r="J15" s="65" t="str">
         <x:v>代码与用例已更新；未运行动态测试</x:v>
       </x:c>
       <x:c r="K15" s="65" t="str">
-        <x:v>docs/武将设计思想.json#ellie</x:v>
+        <x:v>docs/武将设计思想.json#elite_soldier</x:v>
       </x:c>
       <x:c r="L15" s="65" t="str">
-        <x:v>本轮依据源码和既有测试代码逐项检查；2026-09-08静态语法/格式检查，尚无本轮动态对局或回归结果。</x:v>
+        <x:v>先完成2026-09-08源规则独立基线并同步工作簿，随后逐个读取战斗、AI和测试；2026-09-09完成修正及静态检查，没有本轮动态运行结果。</x:v>
       </x:c>
       <x:c r="M15" s="65" t="str">
         <x:v>2026-09-06用户调整：连续分批完成全部已开发武将及AI的设计优先检查修改；保留测试用例和静态检查，中途不运行测试、不等待逐批签收，全部完成后统一测试。</x:v>
@@ -24283,22 +24535,22 @@
     </x:row>
     <x:row r="16" ht="84" hidden="0" customHeight="1">
       <x:c r="A16" s="99" t="str">
-        <x:v>ellie</x:v>
+        <x:v>elite_soldier</x:v>
       </x:c>
       <x:c r="B16" s="99" t="str">
-        <x:v>艾莉</x:v>
+        <x:v>精兵</x:v>
       </x:c>
       <x:c r="C16" s="99" t="str">
-        <x:v>2026-09-08完成规则、战斗、AI、预览及测试代码检查和修改；动态验证等待全部已开发武将完成后统一运行。</x:v>
+        <x:v>2026-09-09完成战斗、AI、预览与测试代码检查修改；静态检查通过，动态验证等待全部73名已开发武将完成后统一进行。</x:v>
       </x:c>
       <x:c r="D16" s="99" t="str">
         <x:v>前端/连锁</x:v>
       </x:c>
       <x:c r="E16" s="99" t="str">
-        <x:v>预览与AI落点相同，只影响牵引目标，穿越其他单位不为旁观者开反应。</x:v>
+        <x:v>机枪不能为友军开启反应，前端预览与AI均使用同一效果单位集合；撤步合法路径一致。</x:v>
       </x:c>
       <x:c r="F16" s="99" t="str">
-        <x:v>targeting.js::computeHighlights/descentMomentDestinations；ManaPullSkill.preview/get_target_cells_for_payload。</x:v>
+        <x:v>core.py::Skill.excludes_allies_from_effect/build_queued_action；ai.py::skill_effect_units；BackstepShotSkill.preview/retreat_cells。</x:v>
       </x:c>
       <x:c r="G16" s="99" t="str">
         <x:v>已检查并修正，待统一动态验证</x:v>
@@ -24307,16 +24559,16 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="I16" s="99" t="str">
-        <x:v>前端复用destinations_by_target，避免客户端自行挡住可穿人路径；移除原路径单位错误收集。</x:v>
+        <x:v>新增共享友军排除标志并接入机枪；保留已有连续直线选格和后续仅来源反击流程。</x:v>
       </x:c>
       <x:c r="J16" s="99" t="str">
         <x:v>代码与用例已更新；未运行动态测试</x:v>
       </x:c>
       <x:c r="K16" s="99" t="str">
-        <x:v>docs/武将设计思想.json#ellie</x:v>
+        <x:v>docs/武将设计思想.json#elite_soldier</x:v>
       </x:c>
       <x:c r="L16" s="99" t="str">
-        <x:v>本轮依据源码和既有测试代码逐项检查；2026-09-08静态语法/格式检查，尚无本轮动态对局或回归结果。</x:v>
+        <x:v>先完成2026-09-08源规则独立基线并同步工作簿，随后逐个读取战斗、AI和测试；2026-09-09完成修正及静态检查，没有本轮动态运行结果。</x:v>
       </x:c>
       <x:c r="M16" s="99" t="str">
         <x:v>2026-09-06用户调整：连续分批完成全部已开发武将及AI的设计优先检查修改；保留测试用例和静态检查，中途不运行测试、不等待逐批签收，全部完成后统一测试。</x:v>
@@ -24324,22 +24576,22 @@
     </x:row>
     <x:row r="17" ht="84" hidden="0" customHeight="1">
       <x:c r="A17" s="99" t="str">
-        <x:v>ellie</x:v>
+        <x:v>elite_soldier</x:v>
       </x:c>
       <x:c r="B17" s="99" t="str">
-        <x:v>艾莉</x:v>
+        <x:v>精兵</x:v>
       </x:c>
       <x:c r="C17" s="99" t="str">
-        <x:v>2026-09-08完成规则、战斗、AI、预览及测试代码检查和修改；动态验证等待全部已开发武将完成后统一运行。</x:v>
+        <x:v>2026-09-09完成战斗、AI、预览与测试代码检查修改；静态检查通过，动态验证等待全部73名已开发武将完成后统一进行。</x:v>
       </x:c>
       <x:c r="D17" s="99" t="str">
         <x:v>测试</x:v>
       </x:c>
       <x:c r="E17" s="99" t="str">
-        <x:v>费用不可退款、增益魔力容量、三轮倒计时、全图选择与召唤生命周期。</x:v>
+        <x:v>方形射程、强化只消费一次、技能不触发减速、有盾减速及被动边界有确定性覆盖。</x:v>
       </x:c>
       <x:c r="F17" s="99" t="str">
-        <x:v>tests/test_behavior.py::DevelopedHeroReviewR01BehaviorTests；test_battle.py::test_ellie_experiment_counts_target_own_rounds_not_global_turns/test_ellie_crystal_ball_counts_own_rounds_not_global_turns/test_ellie_crystal_ball_enables_long_range_pull；既有美杜莎与主动技能后免伤用例。</x:v>
+        <x:v>tests/test_behavior.py::DevelopedHeroReviewR02BehaviorTests前两项；test_battle.py既有headshot/precision/backstep边界用例。</x:v>
       </x:c>
       <x:c r="G17" s="99" t="str">
         <x:v>已检查并修正，待统一动态验证</x:v>
@@ -24348,16 +24600,16 @@
         <x:v>P2</x:v>
       </x:c>
       <x:c r="I17" s="99" t="str">
-        <x:v>新增费用被盾挡仍支付、牵引载荷/穿人、实验满魔+2、AI风险与正向使用边界；旧生命周期用例保留。未执行动态测试。</x:v>
+        <x:v>新增机枪无随机、无友军目标，以及爆头射程退化/有盾正向机会与探测状态回滚用例。只写用例，未运行动态测试。</x:v>
       </x:c>
       <x:c r="J17" s="99" t="str">
         <x:v>代码与用例已更新；未运行动态测试</x:v>
       </x:c>
       <x:c r="K17" s="99" t="str">
-        <x:v>docs/武将设计思想.json#ellie</x:v>
+        <x:v>docs/武将设计思想.json#elite_soldier</x:v>
       </x:c>
       <x:c r="L17" s="99" t="str">
-        <x:v>本轮依据源码和既有测试代码逐项检查；2026-09-08静态语法/格式检查，尚无本轮动态对局或回归结果。</x:v>
+        <x:v>先完成2026-09-08源规则独立基线并同步工作簿，随后逐个读取战斗、AI和测试；2026-09-09完成修正及静态检查，没有本轮动态运行结果。</x:v>
       </x:c>
       <x:c r="M17" s="99" t="str">
         <x:v>2026-09-06用户调整：连续分批完成全部已开发武将及AI的设计优先检查修改；保留测试用例和静态检查，中途不运行测试、不等待逐批签收，全部完成后统一测试。</x:v>
@@ -24365,22 +24617,22 @@
     </x:row>
     <x:row r="18" ht="84" hidden="0" customHeight="1">
       <x:c r="A18" s="99" t="str">
-        <x:v>dark_human</x:v>
+        <x:v>bard</x:v>
       </x:c>
       <x:c r="B18" s="99" t="str">
-        <x:v>E。暗人</x:v>
+        <x:v>吟游诗人</x:v>
       </x:c>
       <x:c r="C18" s="99" t="str">
-        <x:v>2026-09-08完成规则、战斗、AI、预览及测试代码检查和修改；动态验证等待全部已开发武将完成后统一运行。</x:v>
+        <x:v>2026-09-09完成战斗、AI、预览与测试代码检查修改；静态检查通过，动态验证等待全部73名已开发武将完成后统一进行。</x:v>
       </x:c>
       <x:c r="D18" s="99" t="str">
-        <x:v>规则/战斗实现</x:v>
+        <x:v>战斗实现</x:v>
       </x:c>
       <x:c r="E18" s="99" t="str">
-        <x:v>飞跃3格、回避1格、保护、隐身重置手套、三攻飞行；手套攻4破魔仅禁普通移动3轮；飞踢2轮冷却；遁入黑暗4轮冷却/持续2轮。</x:v>
+        <x:v>守*2同源不叠加；回血反转；洗礼1轮人类目标；吟唱只加魔力点；原地回复检查所有位移。</x:v>
       </x:c>
       <x:c r="F18" s="99" t="str">
-        <x:v>持久hero-rule-index中dark_human条目；first_five.py::DarkHuman/ParalyzingGloveSkill/FateKickSkill/IntoDarknessSkill；common.py::DelayedDarknessStatus/InvincibleUntilActionStatus/StealthSkill。</x:v>
+        <x:v>first_five.py::Bard；common.py::DefendTwiceSkill/HealSkill/BaptismSkill/ChantSkill/StationaryRecoveryTrait；core.py::move_unit。</x:v>
       </x:c>
       <x:c r="G18" s="99" t="str">
         <x:v>已检查并修正，待统一动态验证</x:v>
@@ -24389,16 +24641,16 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="I18" s="99" t="str">
-        <x:v>按已保存规则修订旧说明半轮换算残留；黑暗持续2个己方轮次，独立保留禁疗和首击增幅。飞踢保持公开50%结果及只对目标消失段开启反应，回场沿用原格/最近合法格。</x:v>
+        <x:v>补齐暗属性/灵体/恶魔回血反转；拒绝同源守*2重复施放；强制或连锁移动也取消原地回复而不消耗普通移动次数。 2026-09-10源规则8.3交互补查：反转失血仍走护盾/魔免等伤害防御；大型目标支援的执行与预览按全占格距离。</x:v>
       </x:c>
       <x:c r="J18" s="99" t="str">
         <x:v>代码与用例已更新；未运行动态测试</x:v>
       </x:c>
       <x:c r="K18" s="99" t="str">
-        <x:v>docs/武将设计思想.json#dark_human</x:v>
+        <x:v>docs/武将设计思想.json#bard</x:v>
       </x:c>
       <x:c r="L18" s="99" t="str">
-        <x:v>本轮依据源码和既有测试代码逐项检查；2026-09-08静态语法/格式检查，尚无本轮动态对局或回归结果。</x:v>
+        <x:v>先完成2026-09-08源规则独立基线并同步工作簿，随后逐个读取战斗、AI和测试；2026-09-09完成修正及静态检查，没有本轮动态运行结果。</x:v>
       </x:c>
       <x:c r="M18" s="99" t="str">
         <x:v>2026-09-06用户调整：连续分批完成全部已开发武将及AI的设计优先检查修改；保留测试用例和静态检查，中途不运行测试、不等待逐批签收，全部完成后统一测试。</x:v>
@@ -24406,22 +24658,22 @@
     </x:row>
     <x:row r="19" ht="84" hidden="0" customHeight="1">
       <x:c r="A19" s="99" t="str">
-        <x:v>dark_human</x:v>
+        <x:v>bard</x:v>
       </x:c>
       <x:c r="B19" s="99" t="str">
-        <x:v>E。暗人</x:v>
+        <x:v>吟游诗人</x:v>
       </x:c>
       <x:c r="C19" s="99" t="str">
-        <x:v>2026-09-08完成规则、战斗、AI、预览及测试代码检查和修改；动态验证等待全部已开发武将完成后统一运行。</x:v>
+        <x:v>2026-09-09完成战斗、AI、预览与测试代码检查修改；静态检查通过，动态验证等待全部73名已开发武将完成后统一进行。</x:v>
       </x:c>
       <x:c r="D19" s="99" t="str">
-        <x:v>通用引擎</x:v>
+        <x:v>场地/时序</x:v>
       </x:c>
       <x:c r="E19" s="99" t="str">
-        <x:v>冷却不可随每名其他武将的回合加速。</x:v>
+        <x:v>圣光跟随施法者11×11，只有敌方普通移动结束在场内受攻4伤害；友方仅自己的回合末加防；2.5轮不被多人回合缩短。</x:v>
       </x:c>
       <x:c r="F19" s="99" t="str">
-        <x:v>core.py::Skill.on_any_turn_end此前每个全局回合末减1；unit_belongs_to_current_turn按控制武将及召唤物行动组判定。</x:v>
+        <x:v>common.py::GreatHolyLightField/GreatHolyLightSkill；unit_belongs_to_current_turn及全占格判断。</x:v>
       </x:c>
       <x:c r="G19" s="99" t="str">
         <x:v>已检查并修正，待统一动态验证</x:v>
@@ -24430,16 +24682,16 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="I19" s="99" t="str">
-        <x:v>只在技能持有者自己的回合末减冷却；使用当回合计入。共享修正须在最终全73名回归中验证。</x:v>
+        <x:v>将固定4生命扣减改为攻4公式；按施放者第三个己方回合末到期，守+1按受益者自己的回合结束授予且不叠加，放逐期间不生成场内效果。</x:v>
       </x:c>
       <x:c r="J19" s="99" t="str">
         <x:v>代码与用例已更新；未运行动态测试</x:v>
       </x:c>
       <x:c r="K19" s="99" t="str">
-        <x:v>docs/武将设计思想.json#dark_human</x:v>
+        <x:v>docs/武将设计思想.json#bard</x:v>
       </x:c>
       <x:c r="L19" s="99" t="str">
-        <x:v>本轮依据源码和既有测试代码逐项检查；2026-09-08静态语法/格式检查，尚无本轮动态对局或回归结果。</x:v>
+        <x:v>先完成2026-09-08源规则独立基线并同步工作簿，随后逐个读取战斗、AI和测试；2026-09-09完成修正及静态检查，没有本轮动态运行结果。</x:v>
       </x:c>
       <x:c r="M19" s="99" t="str">
         <x:v>2026-09-06用户调整：连续分批完成全部已开发武将及AI的设计优先检查修改；保留测试用例和静态检查，中途不运行测试、不等待逐批签收，全部完成后统一测试。</x:v>
@@ -24447,22 +24699,22 @@
     </x:row>
     <x:row r="20" ht="84" hidden="0" customHeight="1">
       <x:c r="A20" s="99" t="str">
-        <x:v>dark_human</x:v>
+        <x:v>bard</x:v>
       </x:c>
       <x:c r="B20" s="99" t="str">
-        <x:v>E。暗人</x:v>
+        <x:v>吟游诗人</x:v>
       </x:c>
       <x:c r="C20" s="99" t="str">
-        <x:v>2026-09-08完成规则、战斗、AI、预览及测试代码检查和修改；动态验证等待全部已开发武将完成后统一运行。</x:v>
+        <x:v>2026-09-09完成战斗、AI、预览与测试代码检查修改；静态检查通过，动态验证等待全部73名已开发武将完成后统一进行。</x:v>
       </x:c>
       <x:c r="D20" s="99" t="str">
         <x:v>AI</x:v>
       </x:c>
       <x:c r="E20" s="99" t="str">
-        <x:v>三攻接敌、手套重置、黑暗强化普攻和飞踢自我消失风险。</x:v>
+        <x:v>真实治疗收益、不可治疗/满血/反转、魔力点接收者、重复防御与保留站位收益。</x:v>
       </x:c>
       <x:c r="F20" s="99" t="str">
-        <x:v>ai.py::score_skill_payload/self_buff_score；原飞踢与普通位移同价、隐身未判断已用手套。</x:v>
+        <x:v>ai.py::score_skill_payload/ally_buff_score/field_skill_score/score_move_destination。</x:v>
       </x:c>
       <x:c r="G20" s="99" t="str">
         <x:v>已检查并修正，待统一动态验证</x:v>
@@ -24471,16 +24723,16 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="I20" s="99" t="str">
-        <x:v>飞踢按50%敌我价值差并扣未兑现攻击机会；手套已用且资源/目标允许时提高隐身价值；黑暗有即刻普攻机会时优先，避免重复增益。</x:v>
+        <x:v>用回滚执行探测实际回血；吟唱只奖励有魔力点用途的友军并按资源需求保留；圣光判断普通移动机会，移动评分计入放弃原地回复的代价。</x:v>
       </x:c>
       <x:c r="J20" s="99" t="str">
         <x:v>代码与用例已更新；未运行动态测试</x:v>
       </x:c>
       <x:c r="K20" s="99" t="str">
-        <x:v>docs/武将设计思想.json#dark_human</x:v>
+        <x:v>docs/武将设计思想.json#bard</x:v>
       </x:c>
       <x:c r="L20" s="99" t="str">
-        <x:v>本轮依据源码和既有测试代码逐项检查；2026-09-08静态语法/格式检查，尚无本轮动态对局或回归结果。</x:v>
+        <x:v>先完成2026-09-08源规则独立基线并同步工作簿，随后逐个读取战斗、AI和测试；2026-09-09完成修正及静态检查，没有本轮动态运行结果。</x:v>
       </x:c>
       <x:c r="M20" s="99" t="str">
         <x:v>2026-09-06用户调整：连续分批完成全部已开发武将及AI的设计优先检查修改；保留测试用例和静态检查，中途不运行测试、不等待逐批签收，全部完成后统一测试。</x:v>
@@ -24488,22 +24740,22 @@
     </x:row>
     <x:row r="21" ht="84" hidden="0" customHeight="1">
       <x:c r="A21" s="99" t="str">
-        <x:v>dark_human</x:v>
+        <x:v>bard</x:v>
       </x:c>
       <x:c r="B21" s="99" t="str">
-        <x:v>E。暗人</x:v>
+        <x:v>吟游诗人</x:v>
       </x:c>
       <x:c r="C21" s="99" t="str">
-        <x:v>2026-09-08完成规则、战斗、AI、预览及测试代码检查和修改；动态验证等待全部已开发武将完成后统一运行。</x:v>
+        <x:v>2026-09-09完成战斗、AI、预览与测试代码检查修改；静态检查通过，动态验证等待全部73名已开发武将完成后统一进行。</x:v>
       </x:c>
       <x:c r="D21" s="99" t="str">
         <x:v>测试</x:v>
       </x:c>
       <x:c r="E21" s="99" t="str">
-        <x:v>分段反应、隐身攻/技能解除、沙尘只除隐身、破魔单effect及消失回场。</x:v>
+        <x:v>多人圣光时长、友军回合加防、普通/技能/强制移动、回血反转和魔力点用途。</x:v>
       </x:c>
       <x:c r="F21" s="99" t="str">
-        <x:v>test_battle.py既有fate_kick/paralyzing_glove/into_darkness与banished_unit_reappears系列；test_behavior.py::DevelopedHeroReviewR01BehaviorTests。</x:v>
+        <x:v>tests/test_behavior.py::DevelopedHeroReviewR02BehaviorTests；test_battle.py既有圣光边界。</x:v>
       </x:c>
       <x:c r="G21" s="99" t="str">
         <x:v>已检查并修正，待统一动态验证</x:v>
@@ -24512,16 +24764,16 @@
         <x:v>P2</x:v>
       </x:c>
       <x:c r="I21" s="99" t="str">
-        <x:v>补多人冷却/黑暗计时与飞踢AI不抽随机数、风险比较；保留既有技能移动不受麻痹、沙尘保留增幅和回场选择用例。未执行动态测试。</x:v>
+        <x:v>新增圣光公式/多人计时、强制移动取消回复、回血反转与禁疗、吟唱用途用例；死亡自动推进旧场景改为0.5生命，保持测试意图与正确公式一致。未运行动态测试。</x:v>
       </x:c>
       <x:c r="J21" s="99" t="str">
         <x:v>代码与用例已更新；未运行动态测试</x:v>
       </x:c>
       <x:c r="K21" s="99" t="str">
-        <x:v>docs/武将设计思想.json#dark_human</x:v>
+        <x:v>docs/武将设计思想.json#bard</x:v>
       </x:c>
       <x:c r="L21" s="99" t="str">
-        <x:v>本轮依据源码和既有测试代码逐项检查；2026-09-08静态语法/格式检查，尚无本轮动态对局或回归结果。</x:v>
+        <x:v>先完成2026-09-08源规则独立基线并同步工作簿，随后逐个读取战斗、AI和测试；2026-09-09完成修正及静态检查，没有本轮动态运行结果。</x:v>
       </x:c>
       <x:c r="M21" s="99" t="str">
         <x:v>2026-09-06用户调整：连续分批完成全部已开发武将及AI的设计优先检查修改；保留测试用例和静态检查，中途不运行测试、不等待逐批签收，全部完成后统一测试。</x:v>
@@ -24529,22 +24781,22 @@
     </x:row>
     <x:row r="22" ht="84" hidden="0" customHeight="1">
       <x:c r="A22" s="99" t="str">
-        <x:v>fire_funeral</x:v>
+        <x:v>element_hunter</x:v>
       </x:c>
       <x:c r="B22" s="99" t="str">
-        <x:v>火葬者</x:v>
+        <x:v>元素猎人</x:v>
       </x:c>
       <x:c r="C22" s="99" t="str">
-        <x:v>2026-09-08完成规则、战斗、AI、预览及测试代码检查和修改；动态验证等待全部已开发武将完成后统一运行。</x:v>
+        <x:v>2026-09-09完成战斗、AI、预览与测试代码检查修改；静态检查通过，动态验证等待全部73名已开发武将完成后统一进行。</x:v>
       </x:c>
       <x:c r="D22" s="99" t="str">
-        <x:v>战斗实现</x:v>
+        <x:v>战斗实现/控制</x:v>
       </x:c>
       <x:c r="E22" s="99" t="str">
-        <x:v>大火葬十字双方攻5、声明格锁定、自身免伤、减攻最低1、余烬不叠加且只按受影响者自己的回合末触发。</x:v>
+        <x:v>燃烧5次目标己方回合扣魔，暴风雪3轮仅禁普通移动；伤害与非伤害破魔分离；选区固定。</x:v>
       </x:c>
       <x:c r="F22" s="99" t="str">
-        <x:v>first_five.py::GreatFireFuneralSkill/GreatFireFuneralField；原执行重算施法者当前位置、只查单位锚点，余烬按玩家阵营触发。</x:v>
+        <x:v>next_five.py::RemoteAreaDamageSkill/BurningManaStatus/blizzard_status_factory/PlantGrowthSkill；common.py::EllieWardTrait。</x:v>
       </x:c>
       <x:c r="G22" s="99" t="str">
         <x:v>已检查并修正，待统一动态验证</x:v>
@@ -24553,16 +24805,16 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="I22" s="99" t="str">
-        <x:v>锁定声明十字；目标与穿越判断覆盖完整占格；自身排除作为共用声明/AI契约；余烬按控制武将行动组计时，保留穿越半血与同格不叠加。</x:v>
+        <x:v>声明时锁定选区；附加控制穿盾只打掉一盾，免伤仍允许非伤害控制，魔免仍阻止技能效果。燃烧/冰雪不叠同名状态；沿用目标自身计时。</x:v>
       </x:c>
       <x:c r="J22" s="99" t="str">
         <x:v>代码与用例已更新；未运行动态测试</x:v>
       </x:c>
       <x:c r="K22" s="99" t="str">
-        <x:v>docs/武将设计思想.json#fire_funeral</x:v>
+        <x:v>docs/武将设计思想.json#element_hunter</x:v>
       </x:c>
       <x:c r="L22" s="99" t="str">
-        <x:v>本轮依据源码和既有测试代码逐项检查；2026-09-08静态语法/格式检查，尚无本轮动态对局或回归结果。</x:v>
+        <x:v>先完成2026-09-08源规则独立基线并同步工作簿，随后逐个读取战斗、AI和测试；2026-09-09完成修正及静态检查，没有本轮动态运行结果。</x:v>
       </x:c>
       <x:c r="M22" s="99" t="str">
         <x:v>2026-09-06用户调整：连续分批完成全部已开发武将及AI的设计优先检查修改；保留测试用例和静态检查，中途不运行测试、不等待逐批签收，全部完成后统一测试。</x:v>
@@ -24570,22 +24822,22 @@
     </x:row>
     <x:row r="23" ht="84" hidden="0" customHeight="1">
       <x:c r="A23" s="99" t="str">
-        <x:v>fire_funeral</x:v>
+        <x:v>element_hunter</x:v>
       </x:c>
       <x:c r="B23" s="99" t="str">
-        <x:v>火葬者</x:v>
+        <x:v>元素猎人</x:v>
       </x:c>
       <x:c r="C23" s="99" t="str">
-        <x:v>2026-09-08完成规则、战斗、AI、预览及测试代码检查和修改；动态验证等待全部已开发武将完成后统一运行。</x:v>
+        <x:v>2026-09-09完成战斗、AI、预览与测试代码检查修改；静态检查通过，动态验证等待全部73名已开发武将完成后统一进行。</x:v>
       </x:c>
       <x:c r="D23" s="99" t="str">
-        <x:v>战斗实现/前端</x:v>
+        <x:v>召唤/增益/场地</x:v>
       </x:c>
       <x:c r="E23" s="99" t="str">
-        <x:v>审判日攻1解锁、攻6公式、最低能力并列豁免、无视魔免/不可回避/禁疗3轮，护盾取消整个effect。</x:v>
+        <x:v>雷神面板、5轮寿命和敌方直接伤害死亡重置；水波4轮冷却与全五项+1；土行者3分身/随机换位/入场移动/下轮清理；植物双边起点耗点。</x:v>
       </x:c>
       <x:c r="F23" s="99" t="str">
-        <x:v>JudgmentFireSkill及Skill.ignores_magic_immunity_for_payload/cannot_evade_for_payload；原raw_damage=6、能力总和漏魔、禁疗按全局回合减且护盾后仍附加。</x:v>
+        <x:v>next_five.py::ThunderGodSummon/ThunderGodSkill/WaterWaveSkill/AllStatsPlusStatus/EarthWalkerSkill/SplitSkill/EarthWalkerCleanupStatus/PlantGrowthField。</x:v>
       </x:c>
       <x:c r="G23" s="99" t="str">
         <x:v>已检查并修正，待统一动态验证</x:v>
@@ -24594,16 +24846,16 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="I23" s="99" t="str">
-        <x:v>按当前攻守速普通范与魔力计算在场最低集合，锁定声明格；双方预览与AI一致；以攻6结算并按目标自己的3轮禁疗；护盾挡伤害同时挡禁疗。</x:v>
+        <x:v>雷神生命周期沿用已读实现；水波改4个己方回合冷却且到期收回魔容量；土行者复用通用3分身选择、显示与换位，覆盖入场权限和清理；植物按大型单位起点全占格判断。</x:v>
       </x:c>
       <x:c r="J23" s="99" t="str">
         <x:v>代码与用例已更新；未运行动态测试</x:v>
       </x:c>
       <x:c r="K23" s="99" t="str">
-        <x:v>docs/武将设计思想.json#fire_funeral</x:v>
+        <x:v>docs/武将设计思想.json#element_hunter</x:v>
       </x:c>
       <x:c r="L23" s="99" t="str">
-        <x:v>本轮依据源码和既有测试代码逐项检查；2026-09-08静态语法/格式检查，尚无本轮动态对局或回归结果。</x:v>
+        <x:v>先完成2026-09-08源规则独立基线并同步工作簿，随后逐个读取战斗、AI和测试；2026-09-09完成修正及静态检查，没有本轮动态运行结果。</x:v>
       </x:c>
       <x:c r="M23" s="99" t="str">
         <x:v>2026-09-06用户调整：连续分批完成全部已开发武将及AI的设计优先检查修改；保留测试用例和静态检查，中途不运行测试、不等待逐批签收，全部完成后统一测试。</x:v>
@@ -24611,22 +24863,22 @@
     </x:row>
     <x:row r="24" ht="84" hidden="0" customHeight="1">
       <x:c r="A24" s="99" t="str">
-        <x:v>fire_funeral</x:v>
+        <x:v>element_hunter</x:v>
       </x:c>
       <x:c r="B24" s="99" t="str">
-        <x:v>火葬者</x:v>
+        <x:v>元素猎人</x:v>
       </x:c>
       <x:c r="C24" s="99" t="str">
-        <x:v>2026-09-08完成规则、战斗、AI、预览及测试代码检查和修改；动态验证等待全部已开发武将完成后统一运行。</x:v>
+        <x:v>2026-09-09完成战斗、AI、预览与测试代码检查修改；静态检查通过，动态验证等待全部73名已开发武将完成后统一进行。</x:v>
       </x:c>
       <x:c r="D24" s="99" t="str">
-        <x:v>AI</x:v>
+        <x:v>AI/预览</x:v>
       </x:c>
       <x:c r="E24" s="99" t="str">
-        <x:v>十字与终局须计算真实敌友影响、自身豁免、重复火区、降攻机会成本及无视魔免。</x:v>
+        <x:v>三落点载荷、先兑现有效普攻再结束本体行动；控制不重复计新状态收益；场地敌友代价；水波增益不重复。</x:v>
       </x:c>
       <x:c r="F24" s="99" t="str">
-        <x:v>ai.py::great_fire_funeral_score/skill_effect_units/probe_skill_damage_impact；原对已覆盖火区重复计分、自身算友伤，伤害探查遗漏无视魔免。</x:v>
+        <x:v>ai.py::split_payloads/score_skill_payload/field_skill_score/self_buff_score/probe_skill_damage_impact；targeting.js::patternSelection/required_cells通用入口。</x:v>
       </x:c>
       <x:c r="G24" s="99" t="str">
         <x:v>已检查并修正，待统一动态验证</x:v>
@@ -24635,16 +24887,16 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="I24" s="99" t="str">
-        <x:v>新增火区才计算场地增益；降攻扣普攻机会成本并评价攻1阶段；排除自身虚假友伤；伤害探查共享无视魔免/不可回避钩子。</x:v>
+        <x:v>土行者生成3个合法落点并保留有效普攻；只奖励新增控制，燃烧/冰雪伤害探测不错误破盾且包含附加效果；植物考虑友军拖累，水波检查现有状态与交战距离。前端复用三格选择协议。</x:v>
       </x:c>
       <x:c r="J24" s="99" t="str">
         <x:v>代码与用例已更新；未运行动态测试</x:v>
       </x:c>
       <x:c r="K24" s="99" t="str">
-        <x:v>docs/武将设计思想.json#fire_funeral</x:v>
+        <x:v>docs/武将设计思想.json#element_hunter</x:v>
       </x:c>
       <x:c r="L24" s="99" t="str">
-        <x:v>本轮依据源码和既有测试代码逐项检查；2026-09-08静态语法/格式检查，尚无本轮动态对局或回归结果。</x:v>
+        <x:v>先完成2026-09-08源规则独立基线并同步工作簿，随后逐个读取战斗、AI和测试；2026-09-09完成修正及静态检查，没有本轮动态运行结果。</x:v>
       </x:c>
       <x:c r="M24" s="99" t="str">
         <x:v>2026-09-06用户调整：连续分批完成全部已开发武将及AI的设计优先检查修改；保留测试用例和静态检查，中途不运行测试、不等待逐批签收，全部完成后统一测试。</x:v>
@@ -24652,22 +24904,22 @@
     </x:row>
     <x:row r="25" ht="84" hidden="0" customHeight="1">
       <x:c r="A25" s="99" t="str">
-        <x:v>fire_funeral</x:v>
+        <x:v>element_hunter</x:v>
       </x:c>
       <x:c r="B25" s="99" t="str">
-        <x:v>火葬者</x:v>
+        <x:v>元素猎人</x:v>
       </x:c>
       <x:c r="C25" s="99" t="str">
-        <x:v>2026-09-08完成规则、战斗、AI、预览及测试代码检查和修改；动态验证等待全部已开发武将完成后统一运行。</x:v>
+        <x:v>2026-09-09完成战斗、AI、预览与测试代码检查修改；静态检查通过，动态验证等待全部73名已开发武将完成后统一进行。</x:v>
       </x:c>
       <x:c r="D25" s="99" t="str">
         <x:v>测试</x:v>
       </x:c>
       <x:c r="E25" s="99" t="str">
-        <x:v>公式、并列豁免、护盾、声明后资源/位置变化、独立武将回合、伤害探查不改变真实状态。</x:v>
+        <x:v>控制穿盾/艾莉免伤、冷却与魔容量、雷神死亡来源和三分身生命周期。</x:v>
       </x:c>
       <x:c r="F25" s="99" t="str">
-        <x:v>test_behavior.py::DevelopedHeroReviewR01BehaviorTests；test_battle.py既有great_fire_funeral/judgment_fire/knockback/pierce用例。</x:v>
+        <x:v>tests/test_behavior.py::DevelopedHeroReviewR02BehaviorTests后四项；test_battle.py及既有行为场景的土行者、植物、燃烧、冰雪生命周期用例。</x:v>
       </x:c>
       <x:c r="G25" s="99" t="str">
         <x:v>已检查并修正，待统一动态验证</x:v>
@@ -24676,16 +24928,16 @@
         <x:v>P2</x:v>
       </x:c>
       <x:c r="I25" s="99" t="str">
-        <x:v>新增高防公式、并列最低、声明后能力变化仍打原格、护盾禁疗边界、施法者位移不改变十字、多人余烬和魔免探查回滚。未执行动态测试。</x:v>
+        <x:v>新增免伤但控制生效/一盾消费与AI回滚、水波自己回合计时、土行者3落点和先攻击、雷神敌方/己方/场地/无来源死亡矩阵；更新旧单分身场景。未运行动态测试。</x:v>
       </x:c>
       <x:c r="J25" s="99" t="str">
         <x:v>代码与用例已更新；未运行动态测试</x:v>
       </x:c>
       <x:c r="K25" s="99" t="str">
-        <x:v>docs/武将设计思想.json#fire_funeral</x:v>
+        <x:v>docs/武将设计思想.json#element_hunter</x:v>
       </x:c>
       <x:c r="L25" s="99" t="str">
-        <x:v>本轮依据源码和既有测试代码逐项检查；2026-09-08静态语法/格式检查，尚无本轮动态对局或回归结果。</x:v>
+        <x:v>先完成2026-09-08源规则独立基线并同步工作簿，随后逐个读取战斗、AI和测试；2026-09-09完成修正及静态检查，没有本轮动态运行结果。</x:v>
       </x:c>
       <x:c r="M25" s="99" t="str">
         <x:v>2026-09-06用户调整：连续分批完成全部已开发武将及AI的设计优先检查修改；保留测试用例和静态检查，中途不运行测试、不等待逐批签收，全部完成后统一测试。</x:v>
@@ -24693,40 +24945,40 @@
     </x:row>
     <x:row r="26" ht="84" hidden="0" customHeight="1">
       <x:c r="A26" s="99" t="str">
-        <x:v>excel_r126</x:v>
+        <x:v>ellie</x:v>
       </x:c>
       <x:c r="B26" s="99" t="str">
-        <x:v>太阳神</x:v>
+        <x:v>艾莉</x:v>
       </x:c>
       <x:c r="C26" s="99" t="str">
-        <x:v>2026-09-06复核新10场：第7场已避开托尔致命反击陷阱，第5场审判击破两敌；933项回归本批仅剩一项测试沿用过期两格回避口径，现按技能索引一格规则修正测试与说明，待复跑。</x:v>
+        <x:v>2026-09-08完成规则、战斗、AI、预览及测试代码检查和修改；动态验证等待全部已开发武将完成后统一运行。</x:v>
       </x:c>
       <x:c r="D26" s="99" t="str">
         <x:v>战斗实现</x:v>
       </x:c>
       <x:c r="E26" s="99" t="str">
-        <x:v>基础面板、石墙、爆炎、斯芬克斯炮和审判必须完整映射源表。</x:v>
+        <x:v>面板、魔墙、吸魔、牵引、诅咒、实验、水晶球、美杜莎及特性逐项映射。</x:v>
       </x:c>
       <x:c r="F26" s="99" t="str">
-        <x:v>src/wujiang/tactical/heroes/excel_roster.py::_special_skill_factory、SolarFlameSkill、SphinxCannonSkill、SolarJudgmentSkill；通用石墙由技能映射生成。</x:v>
+        <x:v>first_five.py::Ellie/ManaPullSkill/CurseSkill/ExperimentSkill/CrystalBallSkill/MedusaSkill；common.py::EllieWardTrait/ExperimentCountdownStatus；core.py::summon_unit/cleanup_dead_units。</x:v>
       </x:c>
       <x:c r="G26" s="99" t="str">
-        <x:v>符合</x:v>
+        <x:v>已检查并修正，待统一动态验证</x:v>
       </x:c>
       <x:c r="H26" s="99" t="str">
-        <x:v>P3</x:v>
+        <x:v>P1</x:v>
       </x:c>
       <x:c r="I26" s="99" t="str">
-        <x:v>不改规则数值；补足分层测试。</x:v>
+        <x:v>牵引按目标原占格收集反应；诅咒固定0.5生命在声明时支付；实验增加魔力上限并补2魔。魔墙、吸魔、四轮水晶球、四攻召唤物及召唤者死亡级联沿用已读共用实现。 2026-09-09交互补查：EllieWardTrait只取消伤害，保留非伤害后续效果；元素控制用例覆盖此边界。</x:v>
       </x:c>
       <x:c r="J26" s="99" t="str">
-        <x:v>已审查</x:v>
+        <x:v>代码与用例已更新；未运行动态测试</x:v>
       </x:c>
       <x:c r="K26" s="99" t="str">
-        <x:v>docs/武将设计思想.json#excel_r126</x:v>
+        <x:v>docs/武将设计思想.json#ellie</x:v>
       </x:c>
       <x:c r="L26" s="99" t="str">
-        <x:v>9月4日新10场4胜5负、1场500步未决，自动高信号0；炮台7次、爆炎4次、审判7次、石墙19次。第5场步骤19爆炎、22审判，击破咏唱者与蝴蝶刺客；蕾米阵亡带走蝙蝠。第7场17审判、18托尔反击、19太阳神先阵亡，审判未结算。第2场末尾为盖泽尔与李持续交战，不能归为太阳神卡死。929项回归32条失败/错误，本批1条为审判选区测试缺陷，其余31条为既有战略/房间/前端/军团炮/时间停止范围。</x:v>
+        <x:v>本轮依据源码和既有测试代码逐项检查；2026-09-08静态语法/格式检查，尚无本轮动态对局或回归结果。</x:v>
       </x:c>
       <x:c r="M26" s="99" t="str">
         <x:v>2026-09-06用户调整：连续分批完成全部已开发武将及AI的设计优先检查修改；保留测试用例和静态检查，中途不运行测试、不等待逐批签收，全部完成后统一测试。</x:v>
@@ -24734,40 +24986,40 @@
     </x:row>
     <x:row r="27" ht="84" hidden="0" customHeight="1">
       <x:c r="A27" s="99" t="str">
-        <x:v>excel_r126</x:v>
+        <x:v>ellie</x:v>
       </x:c>
       <x:c r="B27" s="99" t="str">
-        <x:v>太阳神</x:v>
+        <x:v>艾莉</x:v>
       </x:c>
       <x:c r="C27" s="99" t="str">
-        <x:v>2026-09-06复核新10场：第7场已避开托尔致命反击陷阱，第5场审判击破两敌；933项回归本批仅剩一项测试沿用过期两格回避口径，现按技能索引一格规则修正测试与说明，待复跑。</x:v>
+        <x:v>2026-09-08完成规则、战斗、AI、预览及测试代码检查和修改；动态验证等待全部已开发武将完成后统一运行。</x:v>
       </x:c>
       <x:c r="D27" s="99" t="str">
         <x:v>AI</x:v>
       </x:c>
       <x:c r="E27" s="99" t="str">
-        <x:v>审判应先判断当前合法反击能否在原动作结算前击破施法者；不能把无法兑现的范围伤害当作收益。</x:v>
+        <x:v>自损、延迟死亡、真实射程与友敌位移收益必须进入判断。</x:v>
       </x:c>
       <x:c r="F27" s="99" t="str">
-        <x:v>9月4日第7场曾向托尔交出审判后被反击先击破；9月6日新第7场不再使用审判，改用爆炎和普攻。933项用户回归中，致命反击、护盾/物免、射程/目标和探查回滚相关新增测试未列入失败。</x:v>
+        <x:v>ai.py::skill_payloads_for_action/score_skill_payload/ally_buff_score/self_buff_score；原牵引缺少落点参数，诅咒和实验按廉价伤害/增益评分。</x:v>
       </x:c>
       <x:c r="G27" s="99" t="str">
-        <x:v>修复获用户复测支持</x:v>
+        <x:v>已检查并修正，待统一动态验证</x:v>
       </x:c>
       <x:c r="H27" s="99" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="I27" s="99" t="str">
-        <x:v>9月5日已加入公开合法反击的可回滚探查；已有护盾、物免、射程之外或未被选区影响的敌人不会导致错误禁用。补致命反击、反向边界及探查不改状态的行为测试。</x:v>
+        <x:v>牵引枚举后端落点并比较目标站位净收益；诅咒拒绝致命支付/重复诅咒；实验保留能立即结束战斗的正向边界；水晶球只为新增射程计分。</x:v>
       </x:c>
       <x:c r="J27" s="99" t="str">
-        <x:v>本项复测未见原缺陷；本批仍待太阳神回避边界测试复跑后签收</x:v>
+        <x:v>代码与用例已更新；未运行动态测试</x:v>
       </x:c>
       <x:c r="K27" s="99" t="str">
-        <x:v>docs/武将设计思想.json#excel_r126</x:v>
+        <x:v>docs/武将设计思想.json#ellie</x:v>
       </x:c>
       <x:c r="L27" s="99" t="str">
-        <x:v>9月4日新10场4胜5负、1场500步未决，自动高信号0；炮台7次、爆炎4次、审判7次、石墙19次。第5场步骤19爆炎、22审判，击破咏唱者与蝴蝶刺客；蕾米阵亡带走蝙蝠。第7场17审判、18托尔反击、19太阳神先阵亡，审判未结算。第2场末尾为盖泽尔与李持续交战，不能归为太阳神卡死。929项回归32条失败/错误，本批1条为审判选区测试缺陷，其余31条为既有战略/房间/前端/军团炮/时间停止范围。</x:v>
+        <x:v>本轮依据源码和既有测试代码逐项检查；2026-09-08静态语法/格式检查，尚无本轮动态对局或回归结果。</x:v>
       </x:c>
       <x:c r="M27" s="99" t="str">
         <x:v>2026-09-06用户调整：连续分批完成全部已开发武将及AI的设计优先检查修改；保留测试用例和静态检查，中途不运行测试、不等待逐批签收，全部完成后统一测试。</x:v>
@@ -24775,40 +25027,40 @@
     </x:row>
     <x:row r="28" ht="84" hidden="0" customHeight="1">
       <x:c r="A28" s="99" t="str">
-        <x:v>excel_r126</x:v>
+        <x:v>ellie</x:v>
       </x:c>
       <x:c r="B28" s="99" t="str">
-        <x:v>太阳神</x:v>
+        <x:v>艾莉</x:v>
       </x:c>
       <x:c r="C28" s="99" t="str">
-        <x:v>2026-09-06复核新10场：第7场已避开托尔致命反击陷阱，第5场审判击破两敌；933项回归本批仅剩一项测试沿用过期两格回避口径，现按技能索引一格规则修正测试与说明，待复跑。</x:v>
+        <x:v>2026-09-08完成规则、战斗、AI、预览及测试代码检查和修改；动态验证等待全部已开发武将完成后统一运行。</x:v>
       </x:c>
       <x:c r="D28" s="99" t="str">
-        <x:v>战斗实现</x:v>
+        <x:v>前端/连锁</x:v>
       </x:c>
       <x:c r="E28" s="99" t="str">
-        <x:v>爆炎按远程龙息：2魔、每回合2次、远程边界裁切2×2、当前攻、未指定阵营时可伤双方。</x:v>
+        <x:v>预览与AI落点相同，只影响牵引目标，穿越其他单位不为旁观者开反应。</x:v>
       </x:c>
       <x:c r="F28" s="99" t="str">
-        <x:v>SolarFlameSkill继承RemoteDragonBreathSkill；DragonBreathSkill按所选格逐单位结算且仅排除施法者。</x:v>
+        <x:v>targeting.js::computeHighlights/descentMomentDestinations；ManaPullSkill.preview/get_target_cells_for_payload。</x:v>
       </x:c>
       <x:c r="G28" s="99" t="str">
-        <x:v>符合</x:v>
+        <x:v>已检查并修正，待统一动态验证</x:v>
       </x:c>
       <x:c r="H28" s="99" t="str">
-        <x:v>P3</x:v>
+        <x:v>P1</x:v>
       </x:c>
       <x:c r="I28" s="99" t="str">
-        <x:v>新增太阳神专属回归断言，避免只依赖通用技能测试。</x:v>
+        <x:v>前端复用destinations_by_target，避免客户端自行挡住可穿人路径；移除原路径单位错误收集。</x:v>
       </x:c>
       <x:c r="J28" s="99" t="str">
-        <x:v>专属测试已加入统一总测试，待用户运行</x:v>
+        <x:v>代码与用例已更新；未运行动态测试</x:v>
       </x:c>
       <x:c r="K28" s="99" t="str">
-        <x:v>docs/武将设计思想.json#excel_r126</x:v>
+        <x:v>docs/武将设计思想.json#ellie</x:v>
       </x:c>
       <x:c r="L28" s="99" t="str">
-        <x:v>9月4日新10场4胜5负、1场500步未决，自动高信号0；炮台7次、爆炎4次、审判7次、石墙19次。第5场步骤19爆炎、22审判，击破咏唱者与蝴蝶刺客；蕾米阵亡带走蝙蝠。第7场17审判、18托尔反击、19太阳神先阵亡，审判未结算。第2场末尾为盖泽尔与李持续交战，不能归为太阳神卡死。929项回归32条失败/错误，本批1条为审判选区测试缺陷，其余31条为既有战略/房间/前端/军团炮/时间停止范围。</x:v>
+        <x:v>本轮依据源码和既有测试代码逐项检查；2026-09-08静态语法/格式检查，尚无本轮动态对局或回归结果。</x:v>
       </x:c>
       <x:c r="M28" s="99" t="str">
         <x:v>2026-09-06用户调整：连续分批完成全部已开发武将及AI的设计优先检查修改；保留测试用例和静态检查，中途不运行测试、不等待逐批签收，全部完成后统一测试。</x:v>
@@ -24816,40 +25068,40 @@
     </x:row>
     <x:row r="29" ht="84" hidden="0" customHeight="1">
       <x:c r="A29" s="99" t="str">
-        <x:v>excel_r126</x:v>
+        <x:v>ellie</x:v>
       </x:c>
       <x:c r="B29" s="99" t="str">
-        <x:v>太阳神</x:v>
+        <x:v>艾莉</x:v>
       </x:c>
       <x:c r="C29" s="99" t="str">
-        <x:v>2026-09-06复核新10场：第7场已避开托尔致命反击陷阱，第5场审判击破两敌；933项回归本批仅剩一项测试沿用过期两格回避口径，现按技能索引一格规则修正测试与说明，待复跑。</x:v>
+        <x:v>2026-09-08完成规则、战斗、AI、预览及测试代码检查和修改；动态验证等待全部已开发武将完成后统一运行。</x:v>
       </x:c>
       <x:c r="D29" s="99" t="str">
-        <x:v>战斗实现</x:v>
+        <x:v>测试</x:v>
       </x:c>
       <x:c r="E29" s="99" t="str">
-        <x:v>斯芬克斯炮2轮一次，攻4守5速1范7；召唤物默认入场回合不能行动、随召唤者离场。</x:v>
+        <x:v>费用不可退款、增益魔力容量、三轮倒计时、全图选择与召唤生命周期。</x:v>
       </x:c>
       <x:c r="F29" s="99" t="str">
-        <x:v>SphinxCannonSkill cooldown_turns=2；SphinxCannonSummon面板正确；Battle.summon_unit令turn_ready=false；下一次所属回合refresh后可行动；cleanup_dead_units清除召唤者遗留召唤物。实测4次召唤中3次随太阳神提前阵亡，1次下回合正常行动。</x:v>
+        <x:v>tests/test_behavior.py::DevelopedHeroReviewR01BehaviorTests；test_battle.py::test_ellie_experiment_counts_target_own_rounds_not_global_turns/test_ellie_crystal_ball_counts_own_rounds_not_global_turns/test_ellie_crystal_ball_enables_long_range_pull；既有美杜莎与主动技能后免伤用例。</x:v>
       </x:c>
       <x:c r="G29" s="99" t="str">
-        <x:v>符合</x:v>
+        <x:v>已检查并修正，待统一动态验证</x:v>
       </x:c>
       <x:c r="H29" s="99" t="str">
-        <x:v>P3</x:v>
+        <x:v>P2</x:v>
       </x:c>
       <x:c r="I29" s="99" t="str">
-        <x:v>新增入场禁动、下回合可动及随召唤者消散测试；审计中把‘召唤后未行动’与‘存活到行动机会仍未行动’分开。</x:v>
+        <x:v>新增费用被盾挡仍支付、牵引载荷/穿人、实验满魔+2、AI风险与正向使用边界；旧生命周期用例保留。未执行动态测试。</x:v>
       </x:c>
       <x:c r="J29" s="99" t="str">
-        <x:v>测试与审计决策点指标已加入，待用户统一测试</x:v>
+        <x:v>代码与用例已更新；未运行动态测试</x:v>
       </x:c>
       <x:c r="K29" s="99" t="str">
-        <x:v>docs/武将设计思想.json#excel_r126</x:v>
+        <x:v>docs/武将设计思想.json#ellie</x:v>
       </x:c>
       <x:c r="L29" s="99" t="str">
-        <x:v>9月4日新10场4胜5负、1场500步未决，自动高信号0；炮台7次、爆炎4次、审判7次、石墙19次。第5场步骤19爆炎、22审判，击破咏唱者与蝴蝶刺客；蕾米阵亡带走蝙蝠。第7场17审判、18托尔反击、19太阳神先阵亡，审判未结算。第2场末尾为盖泽尔与李持续交战，不能归为太阳神卡死。929项回归32条失败/错误，本批1条为审判选区测试缺陷，其余31条为既有战略/房间/前端/军团炮/时间停止范围。</x:v>
+        <x:v>本轮依据源码和既有测试代码逐项检查；2026-09-08静态语法/格式检查，尚无本轮动态对局或回归结果。</x:v>
       </x:c>
       <x:c r="M29" s="99" t="str">
         <x:v>2026-09-06用户调整：连续分批完成全部已开发武将及AI的设计优先检查修改；保留测试用例和静态检查，中途不运行测试、不等待逐批签收，全部完成后统一测试。</x:v>
@@ -24857,40 +25109,40 @@
     </x:row>
     <x:row r="30" ht="84" hidden="0" customHeight="1">
       <x:c r="A30" s="99" t="str">
-        <x:v>excel_r126</x:v>
+        <x:v>dark_human</x:v>
       </x:c>
       <x:c r="B30" s="99" t="str">
-        <x:v>太阳神</x:v>
+        <x:v>E。暗人</x:v>
       </x:c>
       <x:c r="C30" s="99" t="str">
-        <x:v>2026-09-06复核新10场：第7场已避开托尔致命反击陷阱，第5场审判击破两敌；933项回归本批仅剩一项测试沿用过期两格回避口径，现按技能索引一格规则修正测试与说明，待复跑。</x:v>
+        <x:v>2026-09-08完成规则、战斗、AI、预览及测试代码检查和修改；动态验证等待全部已开发武将完成后统一运行。</x:v>
       </x:c>
       <x:c r="D30" s="99" t="str">
-        <x:v>战斗实现</x:v>
+        <x:v>规则/战斗实现</x:v>
       </x:c>
       <x:c r="E30" s="99" t="str">
-        <x:v>炮台的3×3区域普攻未写敌方限定，按通用对象规则必须同时影响敌我；AI仍应强烈规避友伤。</x:v>
+        <x:v>飞跃3格、回避1格、保护、隐身重置手套、三攻飞行；手套攻4破魔仅禁普通移动3轮；飞踢2轮冷却；遁入黑暗4轮冷却/持续2轮。</x:v>
       </x:c>
       <x:c r="F30" s="99" t="str">
-        <x:v>原Battle.basic_area_attack_with_payload统一过滤己方，导致太阳神的炮击不会伤到己方。现增加按武将组件声明的basic_attack_area_affects_allies钩子，并只为SphinxCannonAreaAttackTrait启用；AI区域评分原本已包含己方惩罚。</x:v>
+        <x:v>持久hero-rule-index中dark_human条目；first_five.py::DarkHuman/ParalyzingGloveSkill/FateKickSkill/IntoDarknessSkill；common.py::DelayedDarknessStatus/InvincibleUntilActionStatus/StealthSkill。</x:v>
       </x:c>
       <x:c r="G30" s="99" t="str">
-        <x:v>已修复待验证</x:v>
+        <x:v>已检查并修正，待统一动态验证</x:v>
       </x:c>
       <x:c r="H30" s="99" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="I30" s="99" t="str">
-        <x:v>已加入炮台同一区域同时伤敌我、同时破坏墙体的定向回归测试。</x:v>
+        <x:v>按已保存规则修订旧说明半轮换算残留；黑暗持续2个己方轮次，独立保留禁疗和首击增幅。飞踢保持公开50%结果及只对目标消失段开启反应，回场沿用原格/最近合法格。</x:v>
       </x:c>
       <x:c r="J30" s="99" t="str">
-        <x:v>待用户统一测试</x:v>
+        <x:v>代码与用例已更新；未运行动态测试</x:v>
       </x:c>
       <x:c r="K30" s="99" t="str">
-        <x:v>docs/武将设计思想.json#excel_r126</x:v>
+        <x:v>docs/武将设计思想.json#dark_human</x:v>
       </x:c>
       <x:c r="L30" s="99" t="str">
-        <x:v>9月4日新10场4胜5负、1场500步未决，自动高信号0；炮台7次、爆炎4次、审判7次、石墙19次。第5场步骤19爆炎、22审判，击破咏唱者与蝴蝶刺客；蕾米阵亡带走蝙蝠。第7场17审判、18托尔反击、19太阳神先阵亡，审判未结算。第2场末尾为盖泽尔与李持续交战，不能归为太阳神卡死。929项回归32条失败/错误，本批1条为审判选区测试缺陷，其余31条为既有战略/房间/前端/军团炮/时间停止范围。</x:v>
+        <x:v>本轮依据源码和既有测试代码逐项检查；2026-09-08静态语法/格式检查，尚无本轮动态对局或回归结果。</x:v>
       </x:c>
       <x:c r="M30" s="99" t="str">
         <x:v>2026-09-06用户调整：连续分批完成全部已开发武将及AI的设计优先检查修改；保留测试用例和静态检查，中途不运行测试、不等待逐批签收，全部完成后统一测试。</x:v>
@@ -24898,40 +25150,40 @@
     </x:row>
     <x:row r="31" ht="84" hidden="0" customHeight="1">
       <x:c r="A31" s="99" t="str">
-        <x:v>excel_r126</x:v>
+        <x:v>dark_human</x:v>
       </x:c>
       <x:c r="B31" s="99" t="str">
-        <x:v>太阳神</x:v>
+        <x:v>E。暗人</x:v>
       </x:c>
       <x:c r="C31" s="99" t="str">
-        <x:v>2026-09-06复核新10场：第7场已避开托尔致命反击陷阱，第5场审判击破两敌；933项回归本批仅剩一项测试沿用过期两格回避口径，现按技能索引一格规则修正测试与说明，待复跑。</x:v>
+        <x:v>2026-09-08完成规则、战斗、AI、预览及测试代码检查和修改；动态验证等待全部已开发武将完成后统一运行。</x:v>
       </x:c>
       <x:c r="D31" s="99" t="str">
-        <x:v>规则歧义</x:v>
+        <x:v>通用引擎</x:v>
       </x:c>
       <x:c r="E31" s="99" t="str">
-        <x:v>斯芬克斯炮只能在太阳神周围合法格部署；其普攻按范7自由声明边界可截断3×3，不要求以单位为中心。</x:v>
+        <x:v>冷却不可随每名其他武将的回合加速。</x:v>
       </x:c>
       <x:c r="F31" s="99" t="str">
-        <x:v>源文没有远程部署词语，炮台自身已有范7；周围部署保留低速脆弱本体的布阵风险。通用远程区域规则规定未写‘身前’的3×3按范点格，且源文没有‘目标周围/以目标为中心’。当前实现与该设计推断一致。</x:v>
+        <x:v>core.py::Skill.on_any_turn_end此前每个全局回合末减1；unit_belongs_to_current_turn按控制武将及召唤物行动组判定。</x:v>
       </x:c>
       <x:c r="G31" s="99" t="str">
-        <x:v>设计推断已锁定，符合</x:v>
+        <x:v>已检查并修正，待统一动态验证</x:v>
       </x:c>
       <x:c r="H31" s="99" t="str">
-        <x:v>P2</x:v>
+        <x:v>P1</x:v>
       </x:c>
       <x:c r="I31" s="99" t="str">
-        <x:v>保留当前实现；补充邻接部署拒绝远格、自由区域不以目标居中的定向断言。</x:v>
+        <x:v>只在技能持有者自己的回合末减冷却；使用当回合计入。共享修正须在最终全73名回归中验证。</x:v>
       </x:c>
       <x:c r="J31" s="99" t="str">
-        <x:v>已裁定并补测试，待用户当前批次复测</x:v>
+        <x:v>代码与用例已更新；未运行动态测试</x:v>
       </x:c>
       <x:c r="K31" s="99" t="str">
-        <x:v>docs/武将设计思想.json#excel_r126</x:v>
+        <x:v>docs/武将设计思想.json#dark_human</x:v>
       </x:c>
       <x:c r="L31" s="99" t="str">
-        <x:v>9月4日新10场4胜5负、1场500步未决，自动高信号0；炮台7次、爆炎4次、审判7次、石墙19次。第5场步骤19爆炎、22审判，击破咏唱者与蝴蝶刺客；蕾米阵亡带走蝙蝠。第7场17审判、18托尔反击、19太阳神先阵亡，审判未结算。第2场末尾为盖泽尔与李持续交战，不能归为太阳神卡死。929项回归32条失败/错误，本批1条为审判选区测试缺陷，其余31条为既有战略/房间/前端/军团炮/时间停止范围。</x:v>
+        <x:v>本轮依据源码和既有测试代码逐项检查；2026-09-08静态语法/格式检查，尚无本轮动态对局或回归结果。</x:v>
       </x:c>
       <x:c r="M31" s="99" t="str">
         <x:v>2026-09-06用户调整：连续分批完成全部已开发武将及AI的设计优先检查修改；保留测试用例和静态检查，中途不运行测试、不等待逐批签收，全部完成后统一测试。</x:v>
@@ -24939,40 +25191,40 @@
     </x:row>
     <x:row r="32" ht="84" hidden="0" customHeight="1">
       <x:c r="A32" s="99" t="str">
-        <x:v>excel_r126</x:v>
+        <x:v>dark_human</x:v>
       </x:c>
       <x:c r="B32" s="99" t="str">
-        <x:v>太阳神</x:v>
+        <x:v>E。暗人</x:v>
       </x:c>
       <x:c r="C32" s="99" t="str">
-        <x:v>2026-09-06复核新10场：第7场已避开托尔致命反击陷阱，第5场审判击破两敌；933项回归本批仅剩一项测试沿用过期两格回避口径，现按技能索引一格规则修正测试与说明，待复跑。</x:v>
+        <x:v>2026-09-08完成规则、战斗、AI、预览及测试代码检查和修改；动态验证等待全部已开发武将完成后统一运行。</x:v>
       </x:c>
       <x:c r="D32" s="99" t="str">
-        <x:v>战斗实现</x:v>
+        <x:v>AI</x:v>
       </x:c>
       <x:c r="E32" s="99" t="str">
-        <x:v>炮击和审判应破坏范围内一切非单位地形，以及被定义为地形的单位。</x:v>
+        <x:v>三攻接敌、手套重置、黑暗强化普攻和飞踢自我消失风险。</x:v>
       </x:c>
       <x:c r="F32" s="99" t="str">
-        <x:v>审查时发现_destroy_terrain_in_cells只能清除地形单位与is_terrain场地效果，漏掉Battle.blocked_cells墙体；现已统一移除范围内墙体并记录具体坐标。</x:v>
+        <x:v>ai.py::score_skill_payload/self_buff_score；原飞踢与普通位移同价、隐身未判断已用手套。</x:v>
       </x:c>
       <x:c r="G32" s="99" t="str">
-        <x:v>已修复待验证</x:v>
+        <x:v>已检查并修正，待统一动态验证</x:v>
       </x:c>
       <x:c r="H32" s="99" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="I32" s="99" t="str">
-        <x:v>让统一地形破坏函数同时移除范围内blocked_cells，并输出具体墙体坐标日志。</x:v>
+        <x:v>飞踢按50%敌我价值差并扣未兑现攻击机会；手套已用且资源/目标允许时提高隐身价值；黑暗有即刻普攻机会时优先，避免重复增益。</x:v>
       </x:c>
       <x:c r="J32" s="99" t="str">
-        <x:v>已修复待用户统一测试</x:v>
+        <x:v>代码与用例已更新；未运行动态测试</x:v>
       </x:c>
       <x:c r="K32" s="99" t="str">
-        <x:v>docs/武将设计思想.json#excel_r126</x:v>
+        <x:v>docs/武将设计思想.json#dark_human</x:v>
       </x:c>
       <x:c r="L32" s="99" t="str">
-        <x:v>9月4日新10场4胜5负、1场500步未决，自动高信号0；炮台7次、爆炎4次、审判7次、石墙19次。第5场步骤19爆炎、22审判，击破咏唱者与蝴蝶刺客；蕾米阵亡带走蝙蝠。第7场17审判、18托尔反击、19太阳神先阵亡，审判未结算。第2场末尾为盖泽尔与李持续交战，不能归为太阳神卡死。929项回归32条失败/错误，本批1条为审判选区测试缺陷，其余31条为既有战略/房间/前端/军团炮/时间停止范围。</x:v>
+        <x:v>本轮依据源码和既有测试代码逐项检查；2026-09-08静态语法/格式检查，尚无本轮动态对局或回归结果。</x:v>
       </x:c>
       <x:c r="M32" s="99" t="str">
         <x:v>2026-09-06用户调整：连续分批完成全部已开发武将及AI的设计优先检查修改；保留测试用例和静态检查，中途不运行测试、不等待逐批签收，全部完成后统一测试。</x:v>
@@ -24980,40 +25232,40 @@
     </x:row>
     <x:row r="33" ht="84" hidden="0" customHeight="1">
       <x:c r="A33" s="99" t="str">
-        <x:v>excel_r126</x:v>
+        <x:v>dark_human</x:v>
       </x:c>
       <x:c r="B33" s="99" t="str">
-        <x:v>太阳神</x:v>
+        <x:v>E。暗人</x:v>
       </x:c>
       <x:c r="C33" s="99" t="str">
-        <x:v>2026-09-06复核新10场：第7场已避开托尔致命反击陷阱，第5场审判击破两敌；933项回归本批仅剩一项测试沿用过期两格回避口径，现按技能索引一格规则修正测试与说明，待复跑。</x:v>
+        <x:v>2026-09-08完成规则、战斗、AI、预览及测试代码检查和修改；动态验证等待全部已开发武将完成后统一运行。</x:v>
       </x:c>
       <x:c r="D33" s="99" t="str">
-        <x:v>规则歧义</x:v>
+        <x:v>测试</x:v>
       </x:c>
       <x:c r="E33" s="99" t="str">
-        <x:v>炮击与审判先结算单位伤害，再独立破坏声明区地形；个体伤害被防御取消仍破坏地形，整个动作取消/失效才不结算两者。</x:v>
+        <x:v>分段反应、隐身攻/技能解除、沙尘只除隐身、破魔单effect及消失回场。</x:v>
       </x:c>
       <x:c r="F33" s="99" t="str">
-        <x:v>‘破坏地形’与伤害并列而非写成‘造成伤害后’条件；审判文字先列威力/穿透、后列破坏地形。先伤害后拆地形避免同一effect中途改变本次伤害环境。当前炮台结束回调与审判逐单位伤害后的地形清理符合。</x:v>
+        <x:v>test_battle.py既有fate_kick/paralyzing_glove/into_darkness与banished_unit_reappears系列；test_behavior.py::DevelopedHeroReviewR01BehaviorTests。</x:v>
       </x:c>
       <x:c r="G33" s="99" t="str">
-        <x:v>设计推断已锁定，符合</x:v>
+        <x:v>已检查并修正，待统一动态验证</x:v>
       </x:c>
       <x:c r="H33" s="99" t="str">
         <x:v>P2</x:v>
       </x:c>
       <x:c r="I33" s="99" t="str">
-        <x:v>保留当前实现；补充伤害日志先于地形日志、无单位受伤仍能清地形的定向断言。</x:v>
+        <x:v>补多人冷却/黑暗计时与飞踢AI不抽随机数、风险比较；保留既有技能移动不受麻痹、沙尘保留增幅和回场选择用例。未执行动态测试。</x:v>
       </x:c>
       <x:c r="J33" s="99" t="str">
-        <x:v>已裁定并补测试，待用户当前批次复测</x:v>
+        <x:v>代码与用例已更新；未运行动态测试</x:v>
       </x:c>
       <x:c r="K33" s="99" t="str">
-        <x:v>docs/武将设计思想.json#excel_r126</x:v>
+        <x:v>docs/武将设计思想.json#dark_human</x:v>
       </x:c>
       <x:c r="L33" s="99" t="str">
-        <x:v>9月4日新10场4胜5负、1场500步未决，自动高信号0；炮台7次、爆炎4次、审判7次、石墙19次。第5场步骤19爆炎、22审判，击破咏唱者与蝴蝶刺客；蕾米阵亡带走蝙蝠。第7场17审判、18托尔反击、19太阳神先阵亡，审判未结算。第2场末尾为盖泽尔与李持续交战，不能归为太阳神卡死。929项回归32条失败/错误，本批1条为审判选区测试缺陷，其余31条为既有战略/房间/前端/军团炮/时间停止范围。</x:v>
+        <x:v>本轮依据源码和既有测试代码逐项检查；2026-09-08静态语法/格式检查，尚无本轮动态对局或回归结果。</x:v>
       </x:c>
       <x:c r="M33" s="99" t="str">
         <x:v>2026-09-06用户调整：连续分批完成全部已开发武将及AI的设计优先检查修改；保留测试用例和静态检查，中途不运行测试、不等待逐批签收，全部完成后统一测试。</x:v>
@@ -25021,40 +25273,40 @@
     </x:row>
     <x:row r="34" ht="84" hidden="0" customHeight="1">
       <x:c r="A34" s="99" t="str">
-        <x:v>excel_r126</x:v>
+        <x:v>fire_funeral</x:v>
       </x:c>
       <x:c r="B34" s="99" t="str">
-        <x:v>太阳神</x:v>
+        <x:v>火葬者</x:v>
       </x:c>
       <x:c r="C34" s="99" t="str">
-        <x:v>2026-09-06复核新10场：第7场已避开托尔致命反击陷阱，第5场审判击破两敌；933项回归本批仅剩一项测试沿用过期两格回避口径，现按技能索引一格规则修正测试与说明，待复跑。</x:v>
+        <x:v>2026-09-08完成规则、战斗、AI、预览及测试代码检查和修改；动态验证等待全部已开发武将完成后统一运行。</x:v>
       </x:c>
       <x:c r="D34" s="99" t="str">
         <x:v>战斗实现</x:v>
       </x:c>
       <x:c r="E34" s="99" t="str">
-        <x:v>审判每场一次、远程边界裁切10×10、威力6、半破魔、无视魔免、同时影响敌我。</x:v>
+        <x:v>大火葬十字双方攻5、声明格锁定、自身免伤、减攻最低1、余烬不叠加且只按受影响者自己的回合末触发。</x:v>
       </x:c>
       <x:c r="F34" s="99" t="str">
-        <x:v>SolarJudgmentSkill max_uses_per_battle=1；patterns使用remote_rectangle_patterns；DamageContext固定6、half_ignore_shield与ignore_magic_immunity；units_at_cells不按阵营过滤。</x:v>
+        <x:v>first_five.py::GreatFireFuneralSkill/GreatFireFuneralField；原执行重算施法者当前位置、只查单位锚点，余烬按玩家阵营触发。</x:v>
       </x:c>
       <x:c r="G34" s="99" t="str">
-        <x:v>符合</x:v>
+        <x:v>已检查并修正，待统一动态验证</x:v>
       </x:c>
       <x:c r="H34" s="99" t="str">
-        <x:v>P3</x:v>
+        <x:v>P1</x:v>
       </x:c>
       <x:c r="I34" s="99" t="str">
-        <x:v>保留实现；把一次/场、友伤、边界裁切与防御交互拆成明确测试。</x:v>
+        <x:v>锁定声明十字；目标与穿越判断覆盖完整占格；自身排除作为共用声明/AI契约；余烬按控制武将行动组计时，保留穿越半血与同格不叠加。</x:v>
       </x:c>
       <x:c r="J34" s="99" t="str">
-        <x:v>防御交互、墙体与每场一次断言已加入，待用户统一测试</x:v>
+        <x:v>代码与用例已更新；未运行动态测试</x:v>
       </x:c>
       <x:c r="K34" s="99" t="str">
-        <x:v>docs/武将设计思想.json#excel_r126</x:v>
+        <x:v>docs/武将设计思想.json#fire_funeral</x:v>
       </x:c>
       <x:c r="L34" s="99" t="str">
-        <x:v>9月4日新10场4胜5负、1场500步未决，自动高信号0；炮台7次、爆炎4次、审判7次、石墙19次。第5场步骤19爆炎、22审判，击破咏唱者与蝴蝶刺客；蕾米阵亡带走蝙蝠。第7场17审判、18托尔反击、19太阳神先阵亡，审判未结算。第2场末尾为盖泽尔与李持续交战，不能归为太阳神卡死。929项回归32条失败/错误，本批1条为审判选区测试缺陷，其余31条为既有战略/房间/前端/军团炮/时间停止范围。</x:v>
+        <x:v>本轮依据源码和既有测试代码逐项检查；2026-09-08静态语法/格式检查，尚无本轮动态对局或回归结果。</x:v>
       </x:c>
       <x:c r="M34" s="99" t="str">
         <x:v>2026-09-06用户调整：连续分批完成全部已开发武将及AI的设计优先检查修改；保留测试用例和静态检查，中途不运行测试、不等待逐批签收，全部完成后统一测试。</x:v>
@@ -25062,40 +25314,40 @@
     </x:row>
     <x:row r="35" ht="84" hidden="0" customHeight="1">
       <x:c r="A35" s="99" t="str">
-        <x:v>excel_r126</x:v>
+        <x:v>fire_funeral</x:v>
       </x:c>
       <x:c r="B35" s="99" t="str">
-        <x:v>太阳神</x:v>
+        <x:v>火葬者</x:v>
       </x:c>
       <x:c r="C35" s="99" t="str">
-        <x:v>2026-09-06复核新10场：第7场已避开托尔致命反击陷阱，第5场审判击破两敌；933项回归本批仅剩一项测试沿用过期两格回避口径，现按技能索引一格规则修正测试与说明，待复跑。</x:v>
+        <x:v>2026-09-08完成规则、战斗、AI、预览及测试代码检查和修改；动态验证等待全部已开发武将完成后统一运行。</x:v>
       </x:c>
       <x:c r="D35" s="99" t="str">
-        <x:v>AI</x:v>
+        <x:v>战斗实现/前端</x:v>
       </x:c>
       <x:c r="E35" s="99" t="str">
-        <x:v>太阳神应管理石墙与爆炎共享的魔力，优先保住自身关键生存资源，避免对已有防御链的非致命盟友伤害重复投入。</x:v>
+        <x:v>审判日攻1解锁、攻6公式、最低能力并列豁免、无视魔免/不可回避/禁疗3轮，护盾取消整个effect。</x:v>
       </x:c>
       <x:c r="F35" s="99" t="str">
-        <x:v>用户实测10场石墙30次；多次与格挡、保护、光墙或震开叠加。审查时score_reaction_payload只看原始威胁且shield_targets_for_reaction按威胁升序截断；现已按致命性/威胁降序生成逐级目标组合，并在评分中计算已排队保护和主动伤害技能魔力储备。</x:v>
+        <x:v>JudgmentFireSkill及Skill.ignores_magic_immunity_for_payload/cannot_evade_for_payload；原raw_damage=6、能力总和漏魔、禁疗按全局回合减且护盾后仍附加。</x:v>
       </x:c>
       <x:c r="G35" s="99" t="str">
-        <x:v>已修复待验证</x:v>
+        <x:v>已检查并修正，待统一动态验证</x:v>
       </x:c>
       <x:c r="H35" s="99" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="I35" s="99" t="str">
-        <x:v>改进通用护盾反应AI：按致命性/威胁降序选目标、识别已排队护盾保护、为可用主动技能保留资源，致命自保可突破保留线。</x:v>
+        <x:v>按当前攻守速普通范与魔力计算在场最低集合，锁定声明格；双方预览与AI一致；以攻6结算并按目标自己的3轮禁疗；护盾挡伤害同时挡禁疗。</x:v>
       </x:c>
       <x:c r="J35" s="99" t="str">
-        <x:v>已修复待用户统一测试</x:v>
+        <x:v>代码与用例已更新；未运行动态测试</x:v>
       </x:c>
       <x:c r="K35" s="99" t="str">
-        <x:v>docs/武将设计思想.json#excel_r126</x:v>
+        <x:v>docs/武将设计思想.json#fire_funeral</x:v>
       </x:c>
       <x:c r="L35" s="99" t="str">
-        <x:v>9月4日新10场4胜5负、1场500步未决，自动高信号0；炮台7次、爆炎4次、审判7次、石墙19次。第5场步骤19爆炎、22审判，击破咏唱者与蝴蝶刺客；蕾米阵亡带走蝙蝠。第7场17审判、18托尔反击、19太阳神先阵亡，审判未结算。第2场末尾为盖泽尔与李持续交战，不能归为太阳神卡死。929项回归32条失败/错误，本批1条为审判选区测试缺陷，其余31条为既有战略/房间/前端/军团炮/时间停止范围。</x:v>
+        <x:v>本轮依据源码和既有测试代码逐项检查；2026-09-08静态语法/格式检查，尚无本轮动态对局或回归结果。</x:v>
       </x:c>
       <x:c r="M35" s="99" t="str">
         <x:v>2026-09-06用户调整：连续分批完成全部已开发武将及AI的设计优先检查修改；保留测试用例和静态检查，中途不运行测试、不等待逐批签收，全部完成后统一测试。</x:v>
@@ -25103,40 +25355,40 @@
     </x:row>
     <x:row r="36" ht="84" hidden="0" customHeight="1">
       <x:c r="A36" s="99" t="str">
-        <x:v>excel_r126</x:v>
+        <x:v>fire_funeral</x:v>
       </x:c>
       <x:c r="B36" s="99" t="str">
-        <x:v>太阳神</x:v>
+        <x:v>火葬者</x:v>
       </x:c>
       <x:c r="C36" s="99" t="str">
-        <x:v>2026-09-06复核新10场：第7场已避开托尔致命反击陷阱，第5场审判击破两敌；933项回归本批仅剩一项测试沿用过期两格回避口径，现按技能索引一格规则修正测试与说明，待复跑。</x:v>
+        <x:v>2026-09-08完成规则、战斗、AI、预览及测试代码检查和修改；动态验证等待全部已开发武将完成后统一运行。</x:v>
       </x:c>
       <x:c r="D36" s="99" t="str">
         <x:v>AI</x:v>
       </x:c>
       <x:c r="E36" s="99" t="str">
-        <x:v>审判只在多目标、关键击杀、护盾/魔免突破或地形破局等高价值机会使用。</x:v>
+        <x:v>十字与终局须计算真实敌友影响、自身豁免、重复火区、降攻机会成本及无视魔免。</x:v>
       </x:c>
       <x:c r="F36" s="99" t="str">
-        <x:v>旧实测曾暴露低价值单体审判并加入破局评分；2026-09-03新批次进一步发现评分仍把声明时命中的敌人当作可靠收益，没有扣除其合法范围脱离反应。现从真实公开反应选项与预览落点识别回避、后撤射击、卡片移形、影反等区域脱离，并按可靠敌方击破与己方击破比较；己方阵亡数不少于可靠敌方阵亡数或价值不低于可靠敌损时拒绝审判。</x:v>
+        <x:v>ai.py::great_fire_funeral_score/skill_effect_units/probe_skill_damage_impact；原对已覆盖火区重复计分、自身算友伤，伤害探查遗漏无视魔免。</x:v>
       </x:c>
       <x:c r="G36" s="99" t="str">
-        <x:v>已修复待验证</x:v>
+        <x:v>已检查并修正，待统一动态验证</x:v>
       </x:c>
       <x:c r="H36" s="99" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="I36" s="99" t="str">
-        <x:v>保留一次性大范围破局评分，并复用通用区域脱离反应识别，以反应后的可靠收益决定是否交出审判。</x:v>
+        <x:v>新增火区才计算场地增益；降攻扣普攻机会成本并评价攻1阶段；排除自身虚假友伤；伤害探查共享无视魔免/不可回避钩子。</x:v>
       </x:c>
       <x:c r="J36" s="99" t="str">
-        <x:v>9月6日新第5场继续兑现两敌击破；按一格回避修正可逃出/封出口/无魔边界，待复测</x:v>
+        <x:v>代码与用例已更新；未运行动态测试</x:v>
       </x:c>
       <x:c r="K36" s="99" t="str">
-        <x:v>docs/武将设计思想.json#excel_r126</x:v>
+        <x:v>docs/武将设计思想.json#fire_funeral</x:v>
       </x:c>
       <x:c r="L36" s="99" t="str">
-        <x:v>9月4日新10场4胜5负、1场500步未决，自动高信号0；炮台7次、爆炎4次、审判7次、石墙19次。第5场步骤19爆炎、22审判，击破咏唱者与蝴蝶刺客；蕾米阵亡带走蝙蝠。第7场17审判、18托尔反击、19太阳神先阵亡，审判未结算。第2场末尾为盖泽尔与李持续交战，不能归为太阳神卡死。929项回归32条失败/错误，本批1条为审判选区测试缺陷，其余31条为既有战略/房间/前端/军团炮/时间停止范围。</x:v>
+        <x:v>本轮依据源码和既有测试代码逐项检查；2026-09-08静态语法/格式检查，尚无本轮动态对局或回归结果。</x:v>
       </x:c>
       <x:c r="M36" s="99" t="str">
         <x:v>2026-09-06用户调整：连续分批完成全部已开发武将及AI的设计优先检查修改；保留测试用例和静态检查，中途不运行测试、不等待逐批签收，全部完成后统一测试。</x:v>
@@ -25144,40 +25396,40 @@
     </x:row>
     <x:row r="37" ht="84" hidden="0" customHeight="1">
       <x:c r="A37" s="99" t="str">
-        <x:v>excel_r126</x:v>
+        <x:v>fire_funeral</x:v>
       </x:c>
       <x:c r="B37" s="99" t="str">
-        <x:v>太阳神</x:v>
+        <x:v>火葬者</x:v>
       </x:c>
       <x:c r="C37" s="99" t="str">
-        <x:v>2026-09-06复核新10场：第7场已避开托尔致命反击陷阱，第5场审判击破两敌；933项回归本批仅剩一项测试沿用过期两格回避口径，现按技能索引一格规则修正测试与说明，待复跑。</x:v>
+        <x:v>2026-09-08完成规则、战斗、AI、预览及测试代码检查和修改；动态验证等待全部已开发武将完成后统一运行。</x:v>
       </x:c>
       <x:c r="D37" s="99" t="str">
-        <x:v>AI</x:v>
+        <x:v>测试</x:v>
       </x:c>
       <x:c r="E37" s="99" t="str">
-        <x:v>炮台落点要评估安全、下回合生存、未来3×3火力覆盖和友伤，而不是只看敌人是否在7格。</x:v>
+        <x:v>公式、并列豁免、护盾、声明后资源/位置变化、独立武将回合、伤害探查不改变真实状态。</x:v>
       </x:c>
       <x:c r="F37" s="99" t="str">
-        <x:v>审查时sphinx_cannon_score只统计敌人与落点距离和简单安全分；现已枚举落点未来可声明的3×3，计入敌方价值、多格命中、己方友伤、地形收益、近敌危险和已有炮位间距。</x:v>
+        <x:v>test_behavior.py::DevelopedHeroReviewR01BehaviorTests；test_battle.py既有great_fire_funeral/judgment_fire/knockback/pierce用例。</x:v>
       </x:c>
       <x:c r="G37" s="99" t="str">
-        <x:v>已改进待验证</x:v>
+        <x:v>已检查并修正，待统一动态验证</x:v>
       </x:c>
       <x:c r="H37" s="99" t="str">
         <x:v>P2</x:v>
       </x:c>
       <x:c r="I37" s="99" t="str">
-        <x:v>加入未来3×3覆盖价值、友伤和敌方地形价值；继续保留近敌危险惩罚。</x:v>
+        <x:v>新增高防公式、并列最低、声明后能力变化仍打原格、护盾禁疗边界、施法者位移不改变十字、多人余烬和魔免探查回滚。未执行动态测试。</x:v>
       </x:c>
       <x:c r="J37" s="99" t="str">
-        <x:v>待用户统一测试</x:v>
+        <x:v>代码与用例已更新；未运行动态测试</x:v>
       </x:c>
       <x:c r="K37" s="99" t="str">
-        <x:v>docs/武将设计思想.json#excel_r126</x:v>
+        <x:v>docs/武将设计思想.json#fire_funeral</x:v>
       </x:c>
       <x:c r="L37" s="99" t="str">
-        <x:v>9月4日新10场4胜5负、1场500步未决，自动高信号0；炮台7次、爆炎4次、审判7次、石墙19次。第5场步骤19爆炎、22审判，击破咏唱者与蝴蝶刺客；蕾米阵亡带走蝙蝠。第7场17审判、18托尔反击、19太阳神先阵亡，审判未结算。第2场末尾为盖泽尔与李持续交战，不能归为太阳神卡死。929项回归32条失败/错误，本批1条为审判选区测试缺陷，其余31条为既有战略/房间/前端/军团炮/时间停止范围。</x:v>
+        <x:v>本轮依据源码和既有测试代码逐项检查；2026-09-08静态语法/格式检查，尚无本轮动态对局或回归结果。</x:v>
       </x:c>
       <x:c r="M37" s="99" t="str">
         <x:v>2026-09-06用户调整：连续分批完成全部已开发武将及AI的设计优先检查修改；保留测试用例和静态检查，中途不运行测试、不等待逐批签收，全部完成后统一测试。</x:v>
@@ -25194,13 +25446,13 @@
         <x:v>2026-09-06复核新10场：第7场已避开托尔致命反击陷阱，第5场审判击破两敌；933项回归本批仅剩一项测试沿用过期两格回避口径，现按技能索引一格规则修正测试与说明，待复跑。</x:v>
       </x:c>
       <x:c r="D38" s="99" t="str">
-        <x:v>AI</x:v>
+        <x:v>战斗实现</x:v>
       </x:c>
       <x:c r="E38" s="99" t="str">
-        <x:v>炮台到达可行动回合后应由通用回合束AI正常操作3×3普攻。</x:v>
+        <x:v>基础面板、石墙、爆炎、斯芬克斯炮和审判必须完整映射源表。</x:v>
       </x:c>
       <x:c r="F38" s="99" t="str">
-        <x:v>choose_turn_bundle_action遍历太阳神及其召唤物；炮台的pattern_cells候选经过效果与伤害评分。唯一生存到机会的实测炮台生成132个原始区域、9个合法有效候选并正常攻击。</x:v>
+        <x:v>src/wujiang/tactical/heroes/excel_roster.py::_special_skill_factory、SolarFlameSkill、SphinxCannonSkill、SolarJudgmentSkill；通用石墙由技能映射生成。</x:v>
       </x:c>
       <x:c r="G38" s="99" t="str">
         <x:v>符合</x:v>
@@ -25209,10 +25461,10 @@
         <x:v>P3</x:v>
       </x:c>
       <x:c r="I38" s="99" t="str">
-        <x:v>不改回合束；增加‘有行动机会但未行动’机会指标，避免把提前消散误判成AI闲置。</x:v>
+        <x:v>不改规则数值；补足分层测试。</x:v>
       </x:c>
       <x:c r="J38" s="99" t="str">
-        <x:v>机会决策点指标已加入，待用户统一测试</x:v>
+        <x:v>已审查</x:v>
       </x:c>
       <x:c r="K38" s="99" t="str">
         <x:v>docs/武将设计思想.json#excel_r126</x:v>
@@ -25235,25 +25487,25 @@
         <x:v>2026-09-06复核新10场：第7场已避开托尔致命反击陷阱，第5场审判击破两敌；933项回归本批仅剩一项测试沿用过期两格回避口径，现按技能索引一格规则修正测试与说明，待复跑。</x:v>
       </x:c>
       <x:c r="D39" s="99" t="str">
-        <x:v>前端/预览</x:v>
+        <x:v>AI</x:v>
       </x:c>
       <x:c r="E39" s="99" t="str">
-        <x:v>炮台3×3普攻既然会伤及双方，预览必须把范围内友军也列为受影响对象，不能只用格子暗示友伤。</x:v>
+        <x:v>审判应先判断当前合法反击能否在原动作结算前击破施法者；不能把无法兑现的范围伤害当作收益。</x:v>
       </x:c>
       <x:c r="F39" s="99" t="str">
-        <x:v>SphinxCannonAreaAttackTrait原预览只从enemy_units收集target_unit_ids，实际结算却由basic_attack_area_affects_allies包含友军；现改为从全部在场单位收集并排除炮台自身。</x:v>
+        <x:v>9月4日第7场曾向托尔交出审判后被反击先击破；9月6日新第7场不再使用审判，改用爆炎和普攻。933项用户回归中，致命反击、护盾/物免、射程/目标和探查回滚相关新增测试未列入失败。</x:v>
       </x:c>
       <x:c r="G39" s="99" t="str">
-        <x:v>已修复待验证</x:v>
+        <x:v>修复获用户复测支持</x:v>
       </x:c>
       <x:c r="H39" s="99" t="str">
-        <x:v>P2</x:v>
+        <x:v>P1</x:v>
       </x:c>
       <x:c r="I39" s="99" t="str">
-        <x:v>已补炮台预览同时列出敌友目标的定向断言。</x:v>
+        <x:v>9月5日已加入公开合法反击的可回滚探查；已有护盾、物免、射程之外或未被选区影响的敌人不会导致错误禁用。补致命反击、反向边界及探查不改状态的行为测试。</x:v>
       </x:c>
       <x:c r="J39" s="99" t="str">
-        <x:v>待用户当前批次测试</x:v>
+        <x:v>本项复测未见原缺陷；本批仍待太阳神回避边界测试复跑后签收</x:v>
       </x:c>
       <x:c r="K39" s="99" t="str">
         <x:v>docs/武将设计思想.json#excel_r126</x:v>
@@ -25276,25 +25528,25 @@
         <x:v>2026-09-06复核新10场：第7场已避开托尔致命反击陷阱，第5场审判击破两敌；933项回归本批仅剩一项测试沿用过期两格回避口径，现按技能索引一格规则修正测试与说明，待复跑。</x:v>
       </x:c>
       <x:c r="D40" s="99" t="str">
-        <x:v>测试</x:v>
+        <x:v>战斗实现</x:v>
       </x:c>
       <x:c r="E40" s="99" t="str">
-        <x:v>测试需逐项证明技能规则、AI决策、通用AI改动和关键交互边界。</x:v>
+        <x:v>爆炎按远程龙息：2魔、每回合2次、远程边界裁切2×2、当前攻、未指定阵营时可伤双方。</x:v>
       </x:c>
       <x:c r="F40" s="99" t="str">
-        <x:v>2026-09-06新回归933项，本批唯一失败是测试沿用旧说明的两格回避，合法预览实际为一格；按既定技能索引修正选区及落点，并保留真实连锁结算后的等量交换断言。其他太阳神、赤、犀牛专属测试未列入失败；三名尚未整批签收。</x:v>
+        <x:v>SolarFlameSkill继承RemoteDragonBreathSkill；DragonBreathSkill按所选格逐单位结算且仅排除施法者。</x:v>
       </x:c>
       <x:c r="G40" s="99" t="str">
-        <x:v>已补充待验证</x:v>
+        <x:v>符合</x:v>
       </x:c>
       <x:c r="H40" s="99" t="str">
-        <x:v>P1</x:v>
+        <x:v>P3</x:v>
       </x:c>
       <x:c r="I40" s="99" t="str">
-        <x:v>拆分/补充定向回归与AI测试；只写入统一总测试，不由开发代理运行。</x:v>
+        <x:v>新增太阳神专属回归断言，避免只依赖通用技能测试。</x:v>
       </x:c>
       <x:c r="J40" s="99" t="str">
-        <x:v>一格回避场景与旧说明已同步，待用户复跑当前批次</x:v>
+        <x:v>专属测试已加入统一总测试，待用户运行</x:v>
       </x:c>
       <x:c r="K40" s="99" t="str">
         <x:v>docs/武将设计思想.json#excel_r126</x:v>
@@ -25317,25 +25569,25 @@
         <x:v>2026-09-06复核新10场：第7场已避开托尔致命反击陷阱，第5场审判击破两敌；933项回归本批仅剩一项测试沿用过期两格回避口径，现按技能索引一格规则修正测试与说明，待复跑。</x:v>
       </x:c>
       <x:c r="D41" s="99" t="str">
-        <x:v>审计工具</x:v>
+        <x:v>战斗实现</x:v>
       </x:c>
       <x:c r="E41" s="99" t="str">
-        <x:v>随机对局只有在出现对应机会时才应报告条件性日志缺失。</x:v>
+        <x:v>斯芬克斯炮2轮一次，攻4守5速1范7；召唤物默认入场回合不能行动、随召唤者离场。</x:v>
       </x:c>
       <x:c r="F41" s="99" t="str">
-        <x:v>旧审计把‘破坏了地形’列为无条件日志并曾误报；本轮又确认仅记录技能可用不足以判断错失，且他人同名动作/日志可能串入目标武将。现把‘存在有效候选但未选’列为高优先级错失，把‘可用但无有效候选’列为覆盖缺口，并按事件中的动作来源、目标和相关单位归因。</x:v>
+        <x:v>SphinxCannonSkill cooldown_turns=2；SphinxCannonSummon面板正确；Battle.summon_unit令turn_ready=false；下一次所属回合refresh后可行动；cleanup_dead_units清除召唤者遗留召唤物。实测4次召唤中3次随太阳神提前阵亡，1次下回合正常行动。</x:v>
       </x:c>
       <x:c r="G41" s="99" t="str">
-        <x:v>已修复待验证</x:v>
+        <x:v>符合</x:v>
       </x:c>
       <x:c r="H41" s="99" t="str">
-        <x:v>P1</x:v>
+        <x:v>P3</x:v>
       </x:c>
       <x:c r="I41" s="99" t="str">
-        <x:v>保留条件日志与召唤生命周期指标；新增有效机会分类和跨武将日志隔离。</x:v>
+        <x:v>新增入场禁动、下回合可动及随召唤者消散测试；审计中把‘召唤后未行动’与‘存活到行动机会仍未行动’分开。</x:v>
       </x:c>
       <x:c r="J41" s="99" t="str">
-        <x:v>审计分类与归因已二次修正，待用户复跑当前批次</x:v>
+        <x:v>测试与审计决策点指标已加入，待用户统一测试</x:v>
       </x:c>
       <x:c r="K41" s="99" t="str">
         <x:v>docs/武将设计思想.json#excel_r126</x:v>
@@ -25349,22 +25601,22 @@
     </x:row>
     <x:row r="42" ht="84" customHeight="1">
       <x:c r="A42" s="99" t="str">
-        <x:v>excel_r142</x:v>
+        <x:v>excel_r126</x:v>
       </x:c>
       <x:c r="B42" s="99" t="str">
-        <x:v>猫叔</x:v>
+        <x:v>太阳神</x:v>
       </x:c>
       <x:c r="C42" s="99" t="str">
-        <x:v>已完整验收：设计、5项设计推断、战斗实现、通用AI、测试与两轮用户日志均已逐层审查；同一范围动作重复反制已按声明动作token修复，2026-09-02复测30场中猫叔32次反制均为单token单触发</x:v>
+        <x:v>2026-09-06复核新10场：第7场已避开托尔致命反击陷阱，第5场审判击破两敌；933项回归本批仅剩一项测试沿用过期两格回避口径，现按技能索引一格规则修正测试与说明，待复跑。</x:v>
       </x:c>
       <x:c r="D42" s="99" t="str">
         <x:v>战斗实现</x:v>
       </x:c>
       <x:c r="E42" s="99" t="str">
-        <x:v>嘲讽之吼必须对周围7×7敌我双方造成当前攻4的破魔伤害，再给仍存活命中单位施加指定攻击。</x:v>
+        <x:v>炮台的3×3区域普攻未写敌方限定，按通用对象规则必须同时影响敌我；AI仍应强烈规避友伤。</x:v>
       </x:c>
       <x:c r="F42" s="99" t="str">
-        <x:v>旧CatTauntRoarSkill明确写成敌方、无伤害，只调用validate_target并加状态；现改为effect_units_at_cells双方取值、DamageContext当前攻、ignore_shield，并仅在伤害未取消且目标存活后加状态。</x:v>
+        <x:v>原Battle.basic_area_attack_with_payload统一过滤己方，导致太阳神的炮击不会伤到己方。现增加按武将组件声明的basic_attack_area_affects_allies钩子，并只为SphinxCannonAreaAttackTrait启用；AI区域评分原本已包含己方惩罚。</x:v>
       </x:c>
       <x:c r="G42" s="99" t="str">
         <x:v>已修复待验证</x:v>
@@ -25373,16 +25625,16 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="I42" s="99" t="str">
-        <x:v>已补敌我伤害、破盾和状态顺序的定向测试。</x:v>
+        <x:v>已加入炮台同一区域同时伤敌我、同时破坏墙体的定向回归测试。</x:v>
       </x:c>
       <x:c r="J42" s="99" t="str">
-        <x:v>待用户当前批次测试</x:v>
+        <x:v>待用户统一测试</x:v>
       </x:c>
       <x:c r="K42" s="99" t="str">
-        <x:v>docs/武将设计思想.json#excel_r142</x:v>
+        <x:v>docs/武将设计思想.json#excel_r126</x:v>
       </x:c>
       <x:c r="L42" s="99" t="str">
-        <x:v>reports/current-hero-deep-audit/excel_r142--excel_r198--excel_r206：2026-09-02全新复测10场、8胜2负、自动高信号0/P3；猫叔反制32次。人工扫描30份trace确认不存在同token重复rule_trigger，也不存在单步重复反制；原第10场龙范围普攻现只触发一次。当前三将专属测试未出现在919项回归的31个失败/错误中，其余失败已归类为战略、房间、前端、军团炮或时间停止等非本批范围。</x:v>
+        <x:v>9月4日新10场4胜5负、1场500步未决，自动高信号0；炮台7次、爆炎4次、审判7次、石墙19次。第5场步骤19爆炎、22审判，击破咏唱者与蝴蝶刺客；蕾米阵亡带走蝙蝠。第7场17审判、18托尔反击、19太阳神先阵亡，审判未结算。第2场末尾为盖泽尔与李持续交战，不能归为太阳神卡死。929项回归32条失败/错误，本批1条为审判选区测试缺陷，其余31条为既有战略/房间/前端/军团炮/时间停止范围。</x:v>
       </x:c>
       <x:c r="M42" s="99" t="str">
         <x:v>2026-09-06用户调整：连续分批完成全部已开发武将及AI的设计优先检查修改；保留测试用例和静态检查，中途不运行测试、不等待逐批签收，全部完成后统一测试。</x:v>
@@ -25390,40 +25642,40 @@
     </x:row>
     <x:row r="43" ht="84" customHeight="1">
       <x:c r="A43" s="99" t="str">
-        <x:v>excel_r142</x:v>
+        <x:v>excel_r126</x:v>
       </x:c>
       <x:c r="B43" s="99" t="str">
-        <x:v>猫叔</x:v>
+        <x:v>太阳神</x:v>
       </x:c>
       <x:c r="C43" s="99" t="str">
-        <x:v>已完整验收：设计、5项设计推断、战斗实现、通用AI、测试与两轮用户日志均已逐层审查；同一范围动作重复反制已按声明动作token修复，2026-09-02复测30场中猫叔32次反制均为单token单触发</x:v>
+        <x:v>2026-09-06复核新10场：第7场已避开托尔致命反击陷阱，第5场审判击破两敌；933项回归本批仅剩一项测试沿用过期两格回避口径，现按技能索引一格规则修正测试与说明，待复跑。</x:v>
       </x:c>
       <x:c r="D43" s="99" t="str">
-        <x:v>战斗实现</x:v>
+        <x:v>规则歧义</x:v>
       </x:c>
       <x:c r="E43" s="99" t="str">
-        <x:v>猫叔反制必须覆盖敌我普攻/技能以及直接区域伤害，并且一个声明动作只触发一次。</x:v>
+        <x:v>斯芬克斯炮只能在太阳神周围合法格部署；其普攻按范7自由声明边界可截断3×3，不要求以单位为中心。</x:v>
       </x:c>
       <x:c r="F43" s="99" t="str">
-        <x:v>第一版修复虽共享_trigger接入on_targeted/on_before_damage，但用回合、来源、动作名和动作序号去重；用户日志证明龙的一次范围普攻在伤害与后续效果使用不同动作名，仍重复触发。现Battle为每个已声明QueuedAction提供稳定resolution token，两个钩子按同一token去重；嵌套声明动作仍各有独立token。</x:v>
+        <x:v>源文没有远程部署词语，炮台自身已有范7；周围部署保留低速脆弱本体的布阵风险。通用远程区域规则规定未写‘身前’的3×3按范点格，且源文没有‘目标周围/以目标为中心’。当前实现与该设计推断一致。</x:v>
       </x:c>
       <x:c r="G43" s="99" t="str">
-        <x:v>再次修复待验证</x:v>
+        <x:v>设计推断已锁定，符合</x:v>
       </x:c>
       <x:c r="H43" s="99" t="str">
-        <x:v>P1</x:v>
+        <x:v>P2</x:v>
       </x:c>
       <x:c r="I43" s="99" t="str">
-        <x:v>已补友方直接区域技能触发，以及龙的范围普攻含后续效果时整次动作只反制一次的定向测试。</x:v>
+        <x:v>保留当前实现；补充邻接部署拒绝远格、自由区域不以目标居中的定向断言。</x:v>
       </x:c>
       <x:c r="J43" s="99" t="str">
-        <x:v>待用户重跑当前批次</x:v>
+        <x:v>已裁定并补测试，待用户当前批次复测</x:v>
       </x:c>
       <x:c r="K43" s="99" t="str">
-        <x:v>docs/武将设计思想.json#excel_r142</x:v>
+        <x:v>docs/武将设计思想.json#excel_r126</x:v>
       </x:c>
       <x:c r="L43" s="99" t="str">
-        <x:v>reports/current-hero-deep-audit/excel_r142--excel_r198--excel_r206：2026-09-02全新复测10场、8胜2负、自动高信号0/P3；猫叔反制32次。人工扫描30份trace确认不存在同token重复rule_trigger，也不存在单步重复反制；原第10场龙范围普攻现只触发一次。当前三将专属测试未出现在919项回归的31个失败/错误中，其余失败已归类为战略、房间、前端、军团炮或时间停止等非本批范围。</x:v>
+        <x:v>9月4日新10场4胜5负、1场500步未决，自动高信号0；炮台7次、爆炎4次、审判7次、石墙19次。第5场步骤19爆炎、22审判，击破咏唱者与蝴蝶刺客；蕾米阵亡带走蝙蝠。第7场17审判、18托尔反击、19太阳神先阵亡，审判未结算。第2场末尾为盖泽尔与李持续交战，不能归为太阳神卡死。929项回归32条失败/错误，本批1条为审判选区测试缺陷，其余31条为既有战略/房间/前端/军团炮/时间停止范围。</x:v>
       </x:c>
       <x:c r="M43" s="99" t="str">
         <x:v>2026-09-06用户调整：连续分批完成全部已开发武将及AI的设计优先检查修改；保留测试用例和静态检查，中途不运行测试、不等待逐批签收，全部完成后统一测试。</x:v>
@@ -25431,40 +25683,40 @@
     </x:row>
     <x:row r="44" ht="84" customHeight="1">
       <x:c r="A44" s="99" t="str">
-        <x:v>excel_r142</x:v>
+        <x:v>excel_r126</x:v>
       </x:c>
       <x:c r="B44" s="99" t="str">
-        <x:v>猫叔</x:v>
+        <x:v>太阳神</x:v>
       </x:c>
       <x:c r="C44" s="99" t="str">
-        <x:v>已完整验收：设计、5项设计推断、战斗实现、通用AI、测试与两轮用户日志均已逐层审查；同一范围动作重复反制已按声明动作token修复，2026-09-02复测30场中猫叔32次反制均为单token单触发</x:v>
+        <x:v>2026-09-06复核新10场：第7场已避开托尔致命反击陷阱，第5场审判击破两敌；933项回归本批仅剩一项测试沿用过期两格回避口径，现按技能索引一格规则修正测试与说明，待复跑。</x:v>
       </x:c>
       <x:c r="D44" s="99" t="str">
         <x:v>战斗实现</x:v>
       </x:c>
       <x:c r="E44" s="99" t="str">
-        <x:v>直线拉近应走到合法直线上距离猫叔最近的可达点，而不是找不到恰好邻接共线格就完全不移动。</x:v>
+        <x:v>炮击和审判应破坏范围内一切非单位地形，以及被定义为地形的单位。</x:v>
       </x:c>
       <x:c r="F44" s="99" t="str">
-        <x:v>旧_straight_destination_around只搜索与起点严格共线的邻接落点；现枚举八方向可达直线点，先取与猫叔距离最小者，再取达到同等最近距离所需步数最少者，障碍前停止。</x:v>
+        <x:v>审查时发现_destroy_terrain_in_cells只能清除地形单位与is_terrain场地效果，漏掉Battle.blocked_cells墙体；现已统一移除范围内墙体并记录具体坐标。</x:v>
       </x:c>
       <x:c r="G44" s="99" t="str">
         <x:v>已修复待验证</x:v>
       </x:c>
       <x:c r="H44" s="99" t="str">
-        <x:v>P2</x:v>
+        <x:v>P1</x:v>
       </x:c>
       <x:c r="I44" s="99" t="str">
-        <x:v>已补非共线起点仍沿直线显著拉近的定向测试。</x:v>
+        <x:v>让统一地形破坏函数同时移除范围内blocked_cells，并输出具体墙体坐标日志。</x:v>
       </x:c>
       <x:c r="J44" s="99" t="str">
-        <x:v>待用户当前批次测试</x:v>
+        <x:v>已修复待用户统一测试</x:v>
       </x:c>
       <x:c r="K44" s="99" t="str">
-        <x:v>docs/武将设计思想.json#excel_r142</x:v>
+        <x:v>docs/武将设计思想.json#excel_r126</x:v>
       </x:c>
       <x:c r="L44" s="99" t="str">
-        <x:v>reports/current-hero-deep-audit/excel_r142--excel_r198--excel_r206：2026-09-02全新复测10场、8胜2负、自动高信号0/P3；猫叔反制32次。人工扫描30份trace确认不存在同token重复rule_trigger，也不存在单步重复反制；原第10场龙范围普攻现只触发一次。当前三将专属测试未出现在919项回归的31个失败/错误中，其余失败已归类为战略、房间、前端、军团炮或时间停止等非本批范围。</x:v>
+        <x:v>9月4日新10场4胜5负、1场500步未决，自动高信号0；炮台7次、爆炎4次、审判7次、石墙19次。第5场步骤19爆炎、22审判，击破咏唱者与蝴蝶刺客；蕾米阵亡带走蝙蝠。第7场17审判、18托尔反击、19太阳神先阵亡，审判未结算。第2场末尾为盖泽尔与李持续交战，不能归为太阳神卡死。929项回归32条失败/错误，本批1条为审判选区测试缺陷，其余31条为既有战略/房间/前端/军团炮/时间停止范围。</x:v>
       </x:c>
       <x:c r="M44" s="99" t="str">
         <x:v>2026-09-06用户调整：连续分批完成全部已开发武将及AI的设计优先检查修改；保留测试用例和静态检查，中途不运行测试、不等待逐批签收，全部完成后统一测试。</x:v>
@@ -25472,40 +25724,40 @@
     </x:row>
     <x:row r="45" ht="84" customHeight="1">
       <x:c r="A45" s="99" t="str">
-        <x:v>excel_r142</x:v>
+        <x:v>excel_r126</x:v>
       </x:c>
       <x:c r="B45" s="99" t="str">
-        <x:v>猫叔</x:v>
+        <x:v>太阳神</x:v>
       </x:c>
       <x:c r="C45" s="99" t="str">
-        <x:v>已完整验收：设计、5项设计推断、战斗实现、通用AI、测试与两轮用户日志均已逐层审查；同一范围动作重复反制已按声明动作token修复，2026-09-02复测30场中猫叔32次反制均为单token单触发</x:v>
+        <x:v>2026-09-06复核新10场：第7场已避开托尔致命反击陷阱，第5场审判击破两敌；933项回归本批仅剩一项测试沿用过期两格回避口径，现按技能索引一格规则修正测试与说明，待复跑。</x:v>
       </x:c>
       <x:c r="D45" s="99" t="str">
-        <x:v>通用战斗规则</x:v>
+        <x:v>规则歧义</x:v>
       </x:c>
       <x:c r="E45" s="99" t="str">
-        <x:v>被双方区域嘲讽命中的己方单位必须能把己方猫叔作为合法强制普攻目标。</x:v>
+        <x:v>炮击与审判先结算单位伤害，再独立破坏声明区地形；个体伤害被防御取消仍破坏地形，整个动作取消/失效才不结算两者。</x:v>
       </x:c>
       <x:c r="F45" s="99" t="str">
-        <x:v>旧basic_attack_preview_for_payload只枚举enemy_units，造成友方指定目标不可执行；现Battle.forced_basic_attack_target把有效指定目标加入普攻预览，并在声明时冻结友方目标许可，单体和区域普攻结算均可完成契约。</x:v>
+        <x:v>‘破坏地形’与伤害并列而非写成‘造成伤害后’条件；审判文字先列威力/穿透、后列破坏地形。先伤害后拆地形避免同一effect中途改变本次伤害环境。当前炮台结束回调与审判逐单位伤害后的地形清理符合。</x:v>
       </x:c>
       <x:c r="G45" s="99" t="str">
-        <x:v>已修复待验证</x:v>
+        <x:v>设计推断已锁定，符合</x:v>
       </x:c>
       <x:c r="H45" s="99" t="str">
-        <x:v>P1</x:v>
+        <x:v>P2</x:v>
       </x:c>
       <x:c r="I45" s="99" t="str">
-        <x:v>通用指定攻击目标动作生成与AI候选均已支持己方强制目标。</x:v>
+        <x:v>保留当前实现；补充伤害日志先于地形日志、无单位受伤仍能清地形的定向断言。</x:v>
       </x:c>
       <x:c r="J45" s="99" t="str">
-        <x:v>待用户当前批次测试</x:v>
+        <x:v>已裁定并补测试，待用户当前批次复测</x:v>
       </x:c>
       <x:c r="K45" s="99" t="str">
-        <x:v>docs/武将设计思想.json#excel_r142</x:v>
+        <x:v>docs/武将设计思想.json#excel_r126</x:v>
       </x:c>
       <x:c r="L45" s="99" t="str">
-        <x:v>reports/current-hero-deep-audit/excel_r142--excel_r198--excel_r206：2026-09-02全新复测10场、8胜2负、自动高信号0/P3；猫叔反制32次。人工扫描30份trace确认不存在同token重复rule_trigger，也不存在单步重复反制；原第10场龙范围普攻现只触发一次。当前三将专属测试未出现在919项回归的31个失败/错误中，其余失败已归类为战略、房间、前端、军团炮或时间停止等非本批范围。</x:v>
+        <x:v>9月4日新10场4胜5负、1场500步未决，自动高信号0；炮台7次、爆炎4次、审判7次、石墙19次。第5场步骤19爆炎、22审判，击破咏唱者与蝴蝶刺客；蕾米阵亡带走蝙蝠。第7场17审判、18托尔反击、19太阳神先阵亡，审判未结算。第2场末尾为盖泽尔与李持续交战，不能归为太阳神卡死。929项回归32条失败/错误，本批1条为审判选区测试缺陷，其余31条为既有战略/房间/前端/军团炮/时间停止范围。</x:v>
       </x:c>
       <x:c r="M45" s="99" t="str">
         <x:v>2026-09-06用户调整：连续分批完成全部已开发武将及AI的设计优先检查修改；保留测试用例和静态检查，中途不运行测试、不等待逐批签收，全部完成后统一测试。</x:v>
@@ -25513,40 +25765,40 @@
     </x:row>
     <x:row r="46" ht="84" customHeight="1">
       <x:c r="A46" s="99" t="str">
-        <x:v>excel_r142</x:v>
+        <x:v>excel_r126</x:v>
       </x:c>
       <x:c r="B46" s="99" t="str">
-        <x:v>猫叔</x:v>
+        <x:v>太阳神</x:v>
       </x:c>
       <x:c r="C46" s="99" t="str">
-        <x:v>已完整验收：设计、5项设计推断、战斗实现、通用AI、测试与两轮用户日志均已逐层审查；同一范围动作重复反制已按声明动作token修复，2026-09-02复测30场中猫叔32次反制均为单token单触发</x:v>
+        <x:v>2026-09-06复核新10场：第7场已避开托尔致命反击陷阱，第5场审判击破两敌；933项回归本批仅剩一项测试沿用过期两格回避口径，现按技能索引一格规则修正测试与说明，待复跑。</x:v>
       </x:c>
       <x:c r="D46" s="99" t="str">
-        <x:v>AI</x:v>
+        <x:v>战斗实现</x:v>
       </x:c>
       <x:c r="E46" s="99" t="str">
-        <x:v>猫叔AI必须把怒吼的攻4伤害、控制收益、友伤、队友强制攻击和自身未来承伤放在同一净值中。</x:v>
+        <x:v>审判每场一次、远程边界裁切10×10、威力6、半破魔、无视魔免、同时影响敌我。</x:v>
       </x:c>
       <x:c r="F46" s="99" t="str">
-        <x:v>旧taunt_control_score只统计敌方控制数量；现用真实技能伤害探针计算敌我伤害与破盾，敌方控制扣除预计反打，友方加入伤害及攻击资源浪费惩罚。</x:v>
+        <x:v>SolarJudgmentSkill max_uses_per_battle=1；patterns使用remote_rectangle_patterns；DamageContext固定6、half_ignore_shield与ignore_magic_immunity；units_at_cells不按阵营过滤。</x:v>
       </x:c>
       <x:c r="G46" s="99" t="str">
-        <x:v>已修复待验证</x:v>
+        <x:v>符合</x:v>
       </x:c>
       <x:c r="H46" s="99" t="str">
-        <x:v>P1</x:v>
+        <x:v>P3</x:v>
       </x:c>
       <x:c r="I46" s="99" t="str">
-        <x:v>已补两名队友在范围内时拒绝怒吼的AI测试。</x:v>
+        <x:v>保留实现；把一次/场、友伤、边界裁切与防御交互拆成明确测试。</x:v>
       </x:c>
       <x:c r="J46" s="99" t="str">
-        <x:v>待用户当前批次测试</x:v>
+        <x:v>防御交互、墙体与每场一次断言已加入，待用户统一测试</x:v>
       </x:c>
       <x:c r="K46" s="99" t="str">
-        <x:v>docs/武将设计思想.json#excel_r142</x:v>
+        <x:v>docs/武将设计思想.json#excel_r126</x:v>
       </x:c>
       <x:c r="L46" s="99" t="str">
-        <x:v>reports/current-hero-deep-audit/excel_r142--excel_r198--excel_r206：2026-09-02全新复测10场、8胜2负、自动高信号0/P3；猫叔反制32次。人工扫描30份trace确认不存在同token重复rule_trigger，也不存在单步重复反制；原第10场龙范围普攻现只触发一次。当前三将专属测试未出现在919项回归的31个失败/错误中，其余失败已归类为战略、房间、前端、军团炮或时间停止等非本批范围。</x:v>
+        <x:v>9月4日新10场4胜5负、1场500步未决，自动高信号0；炮台7次、爆炎4次、审判7次、石墙19次。第5场步骤19爆炎、22审判，击破咏唱者与蝴蝶刺客；蕾米阵亡带走蝙蝠。第7场17审判、18托尔反击、19太阳神先阵亡，审判未结算。第2场末尾为盖泽尔与李持续交战，不能归为太阳神卡死。929项回归32条失败/错误，本批1条为审判选区测试缺陷，其余31条为既有战略/房间/前端/军团炮/时间停止范围。</x:v>
       </x:c>
       <x:c r="M46" s="99" t="str">
         <x:v>2026-09-06用户调整：连续分批完成全部已开发武将及AI的设计优先检查修改；保留测试用例和静态检查，中途不运行测试、不等待逐批签收，全部完成后统一测试。</x:v>
@@ -25554,22 +25806,22 @@
     </x:row>
     <x:row r="47" ht="84" customHeight="1">
       <x:c r="A47" s="99" t="str">
-        <x:v>excel_r142</x:v>
+        <x:v>excel_r126</x:v>
       </x:c>
       <x:c r="B47" s="99" t="str">
-        <x:v>猫叔</x:v>
+        <x:v>太阳神</x:v>
       </x:c>
       <x:c r="C47" s="99" t="str">
-        <x:v>已完整验收：设计、5项设计推断、战斗实现、通用AI、测试与两轮用户日志均已逐层审查；同一范围动作重复反制已按声明动作token修复，2026-09-02复测30场中猫叔32次反制均为单token单触发</x:v>
+        <x:v>2026-09-06复核新10场：第7场已避开托尔致命反击陷阱，第5场审判击破两敌；933项回归本批仅剩一项测试沿用过期两格回避口径，现按技能索引一格规则修正测试与说明，待复跑。</x:v>
       </x:c>
       <x:c r="D47" s="99" t="str">
-        <x:v>通用AI</x:v>
+        <x:v>AI</x:v>
       </x:c>
       <x:c r="E47" s="99" t="str">
-        <x:v>所有单位选择攻击或技能影响猫叔时都要计入扣魔、被拉近和后续移动/主动技能锁定成本。</x:v>
+        <x:v>太阳神应管理石墙与爆炎共享的魔力，优先保住自身关键生存资源，避免对已有防御链的非致命盟友伤害重复投入。</x:v>
       </x:c>
       <x:c r="F47" s="99" t="str">
-        <x:v>旧攻击与技能评分没有猫叔反制成本；现build_attack_candidates/build_skill_candidates统一扣除猫叔反制机会成本，强制攻击以高契约分覆盖该惩罚。</x:v>
+        <x:v>用户实测10场石墙30次；多次与格挡、保护、光墙或震开叠加。审查时score_reaction_payload只看原始威胁且shield_targets_for_reaction按威胁升序截断；现已按致命性/威胁降序生成逐级目标组合，并在评分中计算已排队保护和主动伤害技能魔力储备。</x:v>
       </x:c>
       <x:c r="G47" s="99" t="str">
         <x:v>已修复待验证</x:v>
@@ -25578,16 +25830,16 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="I47" s="99" t="str">
-        <x:v>已补有暴露替代目标时通用AI避开猫叔、被嘲讽时仍正确攻击猫叔的测试。</x:v>
+        <x:v>改进通用护盾反应AI：按致命性/威胁降序选目标、识别已排队护盾保护、为可用主动技能保留资源，致命自保可突破保留线。</x:v>
       </x:c>
       <x:c r="J47" s="99" t="str">
-        <x:v>待用户当前批次测试</x:v>
+        <x:v>已修复待用户统一测试</x:v>
       </x:c>
       <x:c r="K47" s="99" t="str">
-        <x:v>docs/武将设计思想.json#excel_r142</x:v>
+        <x:v>docs/武将设计思想.json#excel_r126</x:v>
       </x:c>
       <x:c r="L47" s="99" t="str">
-        <x:v>reports/current-hero-deep-audit/excel_r142--excel_r198--excel_r206：2026-09-02全新复测10场、8胜2负、自动高信号0/P3；猫叔反制32次。人工扫描30份trace确认不存在同token重复rule_trigger，也不存在单步重复反制；原第10场龙范围普攻现只触发一次。当前三将专属测试未出现在919项回归的31个失败/错误中，其余失败已归类为战略、房间、前端、军团炮或时间停止等非本批范围。</x:v>
+        <x:v>9月4日新10场4胜5负、1场500步未决，自动高信号0；炮台7次、爆炎4次、审判7次、石墙19次。第5场步骤19爆炎、22审判，击破咏唱者与蝴蝶刺客；蕾米阵亡带走蝙蝠。第7场17审判、18托尔反击、19太阳神先阵亡，审判未结算。第2场末尾为盖泽尔与李持续交战，不能归为太阳神卡死。929项回归32条失败/错误，本批1条为审判选区测试缺陷，其余31条为既有战略/房间/前端/军团炮/时间停止范围。</x:v>
       </x:c>
       <x:c r="M47" s="99" t="str">
         <x:v>2026-09-06用户调整：连续分批完成全部已开发武将及AI的设计优先检查修改；保留测试用例和静态检查，中途不运行测试、不等待逐批签收，全部完成后统一测试。</x:v>
@@ -25595,40 +25847,40 @@
     </x:row>
     <x:row r="48" ht="84" customHeight="1">
       <x:c r="A48" s="99" t="str">
-        <x:v>excel_r142</x:v>
+        <x:v>excel_r126</x:v>
       </x:c>
       <x:c r="B48" s="99" t="str">
-        <x:v>猫叔</x:v>
+        <x:v>太阳神</x:v>
       </x:c>
       <x:c r="C48" s="99" t="str">
-        <x:v>已完整验收：设计、5项设计推断、战斗实现、通用AI、测试与两轮用户日志均已逐层审查；同一范围动作重复反制已按声明动作token修复，2026-09-02复测30场中猫叔32次反制均为单token单触发</x:v>
+        <x:v>2026-09-06复核新10场：第7场已避开托尔致命反击陷阱，第5场审判击破两敌；933项回归本批仅剩一项测试沿用过期两格回避口径，现按技能索引一格规则修正测试与说明，待复跑。</x:v>
       </x:c>
       <x:c r="D48" s="99" t="str">
-        <x:v>通用AI</x:v>
+        <x:v>AI</x:v>
       </x:c>
       <x:c r="E48" s="99" t="str">
-        <x:v>震开要计算推散已聚拢单位、损失后续近战接触与1魔资源的机会成本，致命防御时仍可使用。</x:v>
+        <x:v>审判只在多目标、关键击杀、护盾/魔免突破或地形破局等高价值机会使用。</x:v>
       </x:c>
       <x:c r="F48" s="99" t="str">
-        <x:v>旧knockback固定按威胁加分；现按周围敌人的未来近战价值、被推队友和低魔非紧急场景扣分，保留致命威胁的高紧急分。</x:v>
+        <x:v>旧实测曾暴露低价值单体审判并加入破局评分；2026-09-03新批次进一步发现评分仍把声明时命中的敌人当作可靠收益，没有扣除其合法范围脱离反应。现从真实公开反应选项与预览落点识别回避、后撤射击、卡片移形、影反等区域脱离，并按可靠敌方击破与己方击破比较；己方阵亡数不少于可靠敌方阵亡数或价值不低于可靠敌损时拒绝审判。</x:v>
       </x:c>
       <x:c r="G48" s="99" t="str">
-        <x:v>已改进待验证</x:v>
+        <x:v>已修复待验证</x:v>
       </x:c>
       <x:c r="H48" s="99" t="str">
-        <x:v>P2</x:v>
+        <x:v>P1</x:v>
       </x:c>
       <x:c r="I48" s="99" t="str">
-        <x:v>通过当前批次决策日志观察猫叔是否仍无条件震开。</x:v>
+        <x:v>保留一次性大范围破局评分，并复用通用区域脱离反应识别，以反应后的可靠收益决定是否交出审判。</x:v>
       </x:c>
       <x:c r="J48" s="99" t="str">
-        <x:v>待用户当前批次测试</x:v>
+        <x:v>9月6日新第5场继续兑现两敌击破；按一格回避修正可逃出/封出口/无魔边界，待复测</x:v>
       </x:c>
       <x:c r="K48" s="99" t="str">
-        <x:v>docs/武将设计思想.json#excel_r142</x:v>
+        <x:v>docs/武将设计思想.json#excel_r126</x:v>
       </x:c>
       <x:c r="L48" s="99" t="str">
-        <x:v>reports/current-hero-deep-audit/excel_r142--excel_r198--excel_r206：2026-09-02全新复测10场、8胜2负、自动高信号0/P3；猫叔反制32次。人工扫描30份trace确认不存在同token重复rule_trigger，也不存在单步重复反制；原第10场龙范围普攻现只触发一次。当前三将专属测试未出现在919项回归的31个失败/错误中，其余失败已归类为战略、房间、前端、军团炮或时间停止等非本批范围。</x:v>
+        <x:v>9月4日新10场4胜5负、1场500步未决，自动高信号0；炮台7次、爆炎4次、审判7次、石墙19次。第5场步骤19爆炎、22审判，击破咏唱者与蝴蝶刺客；蕾米阵亡带走蝙蝠。第7场17审判、18托尔反击、19太阳神先阵亡，审判未结算。第2场末尾为盖泽尔与李持续交战，不能归为太阳神卡死。929项回归32条失败/错误，本批1条为审判选区测试缺陷，其余31条为既有战略/房间/前端/军团炮/时间停止范围。</x:v>
       </x:c>
       <x:c r="M48" s="99" t="str">
         <x:v>2026-09-06用户调整：连续分批完成全部已开发武将及AI的设计优先检查修改；保留测试用例和静态检查，中途不运行测试、不等待逐批签收，全部完成后统一测试。</x:v>
@@ -25636,40 +25888,40 @@
     </x:row>
     <x:row r="49" ht="84" customHeight="1">
       <x:c r="A49" s="99" t="str">
-        <x:v>excel_r142</x:v>
+        <x:v>excel_r126</x:v>
       </x:c>
       <x:c r="B49" s="99" t="str">
-        <x:v>猫叔</x:v>
+        <x:v>太阳神</x:v>
       </x:c>
       <x:c r="C49" s="99" t="str">
-        <x:v>已完整验收：设计、5项设计推断、战斗实现、通用AI、测试与两轮用户日志均已逐层审查；同一范围动作重复反制已按声明动作token修复，2026-09-02复测30场中猫叔32次反制均为单token单触发</x:v>
+        <x:v>2026-09-06复核新10场：第7场已避开托尔致命反击陷阱，第5场审判击破两敌；933项回归本批仅剩一项测试沿用过期两格回避口径，现按技能索引一格规则修正测试与说明，待复跑。</x:v>
       </x:c>
       <x:c r="D49" s="99" t="str">
-        <x:v>审计工具</x:v>
+        <x:v>AI</x:v>
       </x:c>
       <x:c r="E49" s="99" t="str">
-        <x:v>自动审计必须把同一声明动作重复触发一次性反制识别为高信号，不能仅因对局无执行异常就给P3。</x:v>
+        <x:v>炮台落点要评估安全、下回合生存、未来3×3火力覆盖和友伤，而不是只看敌人是否在7格。</x:v>
       </x:c>
       <x:c r="F49" s="99" t="str">
-        <x:v>旧报告自动高信号为0，但同一步trace出现两条‘因攻击或技能猫叔失去’日志。现猫叔每次实际反制都会写入带action resolution token的结构化rule_trigger事件；match_audit按token检查一次性触发不变量，并以duplicate_once_per_action_trigger记录error；不同嵌套动作的token不同，不会误报。batch审计把该分类列入高信号。</x:v>
+        <x:v>审查时sphinx_cannon_score只统计敌人与落点距离和简单安全分；现已枚举落点未来可声明的3×3，计入敌方价值、多格命中、己方友伤、地形收益、近敌危险和已有炮位间距。</x:v>
       </x:c>
       <x:c r="G49" s="99" t="str">
-        <x:v>已修复待验证</x:v>
+        <x:v>已改进待验证</x:v>
       </x:c>
       <x:c r="H49" s="99" t="str">
-        <x:v>P1</x:v>
+        <x:v>P2</x:v>
       </x:c>
       <x:c r="I49" s="99" t="str">
-        <x:v>已补同一token重复事件必须报错、不同嵌套动作token不得误报的审计组件测试；重跑后该历史场景若复现，应进入suspected_defects而非P3。</x:v>
+        <x:v>加入未来3×3覆盖价值、友伤和敌方地形价值；继续保留近敌危险惩罚。</x:v>
       </x:c>
       <x:c r="J49" s="99" t="str">
-        <x:v>待用户重跑当前批次</x:v>
+        <x:v>待用户统一测试</x:v>
       </x:c>
       <x:c r="K49" s="99" t="str">
-        <x:v>docs/武将设计思想.json#excel_r142</x:v>
+        <x:v>docs/武将设计思想.json#excel_r126</x:v>
       </x:c>
       <x:c r="L49" s="99" t="str">
-        <x:v>reports/current-hero-deep-audit/excel_r142--excel_r198--excel_r206：2026-09-02全新复测10场、8胜2负、自动高信号0/P3；猫叔反制32次。人工扫描30份trace确认不存在同token重复rule_trigger，也不存在单步重复反制；原第10场龙范围普攻现只触发一次。当前三将专属测试未出现在919项回归的31个失败/错误中，其余失败已归类为战略、房间、前端、军团炮或时间停止等非本批范围。</x:v>
+        <x:v>9月4日新10场4胜5负、1场500步未决，自动高信号0；炮台7次、爆炎4次、审判7次、石墙19次。第5场步骤19爆炎、22审判，击破咏唱者与蝴蝶刺客；蕾米阵亡带走蝙蝠。第7场17审判、18托尔反击、19太阳神先阵亡，审判未结算。第2场末尾为盖泽尔与李持续交战，不能归为太阳神卡死。929项回归32条失败/错误，本批1条为审判选区测试缺陷，其余31条为既有战略/房间/前端/军团炮/时间停止范围。</x:v>
       </x:c>
       <x:c r="M49" s="99" t="str">
         <x:v>2026-09-06用户调整：连续分批完成全部已开发武将及AI的设计优先检查修改；保留测试用例和静态检查，中途不运行测试、不等待逐批签收，全部完成后统一测试。</x:v>
@@ -25677,40 +25929,40 @@
     </x:row>
     <x:row r="50" ht="84" customHeight="1">
       <x:c r="A50" s="99" t="str">
-        <x:v>excel_r142</x:v>
+        <x:v>excel_r126</x:v>
       </x:c>
       <x:c r="B50" s="99" t="str">
-        <x:v>猫叔</x:v>
+        <x:v>太阳神</x:v>
       </x:c>
       <x:c r="C50" s="99" t="str">
-        <x:v>已完整验收：设计、5项设计推断、战斗实现、通用AI、测试与两轮用户日志均已逐层审查；同一范围动作重复反制已按声明动作token修复，2026-09-02复测30场中猫叔32次反制均为单token单触发</x:v>
+        <x:v>2026-09-06复核新10场：第7场已避开托尔致命反击陷阱，第5场审判击破两敌；933项回归本批仅剩一项测试沿用过期两格回避口径，现按技能索引一格规则修正测试与说明，待复跑。</x:v>
       </x:c>
       <x:c r="D50" s="99" t="str">
-        <x:v>测试</x:v>
+        <x:v>AI</x:v>
       </x:c>
       <x:c r="E50" s="99" t="str">
-        <x:v>测试需覆盖伤害/阵营、破魔、指定攻击、友方强制目标、反制去重/范围触发、拉近和AI净值。</x:v>
+        <x:v>炮台到达可行动回合后应由通用回合束AI正常操作3×3普攻。</x:v>
       </x:c>
       <x:c r="F50" s="99" t="str">
-        <x:v>tests/test_battle.py与tests/test_behavior.py已加入对应定向用例；根据用户首轮结果修正了一个会在怒吼前杀死目标的AI测试夹具，以及一个把直线拉近等价落点写死的过度约束断言；本轮遵照流程不运行回合测试。</x:v>
+        <x:v>choose_turn_bundle_action遍历太阳神及其召唤物；炮台的pattern_cells候选经过效果与伤害评分。唯一生存到机会的实测炮台生成132个原始区域、9个合法有效候选并正常攻击。</x:v>
       </x:c>
       <x:c r="G50" s="99" t="str">
-        <x:v>已补充待验证</x:v>
+        <x:v>符合</x:v>
       </x:c>
       <x:c r="H50" s="99" t="str">
-        <x:v>P1</x:v>
+        <x:v>P3</x:v>
       </x:c>
       <x:c r="I50" s="99" t="str">
-        <x:v>由用户运行python detail_test_all_wujiangs.py --current统一执行。</x:v>
+        <x:v>不改回合束；增加‘有行动机会但未行动’机会指标，避免把提前消散误判成AI闲置。</x:v>
       </x:c>
       <x:c r="J50" s="99" t="str">
-        <x:v>待用户重跑</x:v>
+        <x:v>机会决策点指标已加入，待用户统一测试</x:v>
       </x:c>
       <x:c r="K50" s="99" t="str">
-        <x:v>docs/武将设计思想.json#excel_r142</x:v>
+        <x:v>docs/武将设计思想.json#excel_r126</x:v>
       </x:c>
       <x:c r="L50" s="99" t="str">
-        <x:v>reports/current-hero-deep-audit/excel_r142--excel_r198--excel_r206：2026-09-02全新复测10场、8胜2负、自动高信号0/P3；猫叔反制32次。人工扫描30份trace确认不存在同token重复rule_trigger，也不存在单步重复反制；原第10场龙范围普攻现只触发一次。当前三将专属测试未出现在919项回归的31个失败/错误中，其余失败已归类为战略、房间、前端、军团炮或时间停止等非本批范围。</x:v>
+        <x:v>9月4日新10场4胜5负、1场500步未决，自动高信号0；炮台7次、爆炎4次、审判7次、石墙19次。第5场步骤19爆炎、22审判，击破咏唱者与蝴蝶刺客；蕾米阵亡带走蝙蝠。第7场17审判、18托尔反击、19太阳神先阵亡，审判未结算。第2场末尾为盖泽尔与李持续交战，不能归为太阳神卡死。929项回归32条失败/错误，本批1条为审判选区测试缺陷，其余31条为既有战略/房间/前端/军团炮/时间停止范围。</x:v>
       </x:c>
       <x:c r="M50" s="99" t="str">
         <x:v>2026-09-06用户调整：连续分批完成全部已开发武将及AI的设计优先检查修改；保留测试用例和静态检查，中途不运行测试、不等待逐批签收，全部完成后统一测试。</x:v>
@@ -25718,40 +25970,40 @@
     </x:row>
     <x:row r="51" ht="84" customHeight="1">
       <x:c r="A51" s="99" t="str">
-        <x:v>excel_r198</x:v>
+        <x:v>excel_r126</x:v>
       </x:c>
       <x:c r="B51" s="99" t="str">
-        <x:v>三轮车人</x:v>
+        <x:v>太阳神</x:v>
       </x:c>
       <x:c r="C51" s="99" t="str">
-        <x:v>已完整验收：设计、5项设计推断、战斗实现、AI、测试与两轮用户日志均已逐层审查；召唤顺序、攻击后移动经济与AI重规划符合设计，2026-09-02复测未发现新缺陷</x:v>
+        <x:v>2026-09-06复核新10场：第7场已避开托尔致命反击陷阱，第5场审判击破两敌；933项回归本批仅剩一项测试沿用过期两格回避口径，现按技能索引一格规则修正测试与说明，待复跑。</x:v>
       </x:c>
       <x:c r="D51" s="99" t="str">
-        <x:v>战斗实现</x:v>
+        <x:v>前端/预览</x:v>
       </x:c>
       <x:c r="E51" s="99" t="str">
-        <x:v>本体每完成一次普攻，本回合普通移动上限独立+1，未命中也触发，技能不触发。</x:v>
+        <x:v>炮台3×3普攻既然会伤及双方，预览必须把范围内友军也列为受影响对象，不能只用格子暗示友伤。</x:v>
       </x:c>
       <x:c r="F51" s="99" t="str">
-        <x:v>ExtraMoveAfterAttackTrait以本回合attacks_used修改普通移动上限；攻击次数在普攻结算路径中增加，技能路径不增加，回合刷新后归零。</x:v>
+        <x:v>SphinxCannonAreaAttackTrait原预览只从enemy_units收集target_unit_ids，实际结算却由basic_attack_area_affects_allies包含友军；现改为从全部在场单位收集并排除炮台自身。</x:v>
       </x:c>
       <x:c r="G51" s="99" t="str">
-        <x:v>符合</x:v>
+        <x:v>已修复待验证</x:v>
       </x:c>
       <x:c r="H51" s="99" t="str">
-        <x:v>P3</x:v>
+        <x:v>P2</x:v>
       </x:c>
       <x:c r="I51" s="99" t="str">
-        <x:v>保留实现，补足多次与未命中边界测试。</x:v>
+        <x:v>已补炮台预览同时列出敌友目标的定向断言。</x:v>
       </x:c>
       <x:c r="J51" s="99" t="str">
         <x:v>待用户当前批次测试</x:v>
       </x:c>
       <x:c r="K51" s="99" t="str">
-        <x:v>docs/武将设计思想.json#excel_r198</x:v>
+        <x:v>docs/武将设计思想.json#excel_r126</x:v>
       </x:c>
       <x:c r="L51" s="99" t="str">
-        <x:v>reports/current-hero-deep-audit/excel_r142--excel_r198--excel_r206：2026-09-02全新复测10场、2胜8负、自动高信号0/P3；二轮车召唤10/13个有效机会，一轮车召唤1/1。人工逐步对照再次确认本体召唤→神速/移动→普攻→再次移动，以及二轮车召唤子车→移动→攻击；攻击后未再移动的代表场景随即结束战斗，不构成漏用。当前三将专属测试无失败，未发现实现或AI偏离设计。</x:v>
+        <x:v>9月4日新10场4胜5负、1场500步未决，自动高信号0；炮台7次、爆炎4次、审判7次、石墙19次。第5场步骤19爆炎、22审判，击破咏唱者与蝴蝶刺客；蕾米阵亡带走蝙蝠。第7场17审判、18托尔反击、19太阳神先阵亡，审判未结算。第2场末尾为盖泽尔与李持续交战，不能归为太阳神卡死。929项回归32条失败/错误，本批1条为审判选区测试缺陷，其余31条为既有战略/房间/前端/军团炮/时间停止范围。</x:v>
       </x:c>
       <x:c r="M51" s="99" t="str">
         <x:v>2026-09-06用户调整：连续分批完成全部已开发武将及AI的设计优先检查修改；保留测试用例和静态检查，中途不运行测试、不等待逐批签收，全部完成后统一测试。</x:v>
@@ -25759,40 +26011,40 @@
     </x:row>
     <x:row r="52" ht="84" customHeight="1">
       <x:c r="A52" s="99" t="str">
-        <x:v>excel_r198</x:v>
+        <x:v>excel_r126</x:v>
       </x:c>
       <x:c r="B52" s="99" t="str">
-        <x:v>三轮车人</x:v>
+        <x:v>太阳神</x:v>
       </x:c>
       <x:c r="C52" s="99" t="str">
-        <x:v>已完整验收：设计、5项设计推断、战斗实现、AI、测试与两轮用户日志均已逐层审查；召唤顺序、攻击后移动经济与AI重规划符合设计，2026-09-02复测未发现新缺陷</x:v>
+        <x:v>2026-09-06复核新10场：第7场已避开托尔致命反击陷阱，第5场审判击破两敌；933项回归本批仅剩一项测试沿用过期两格回避口径，现按技能索引一格规则修正测试与说明，待复跑。</x:v>
       </x:c>
       <x:c r="D52" s="99" t="str">
-        <x:v>战斗实现</x:v>
+        <x:v>测试</x:v>
       </x:c>
       <x:c r="E52" s="99" t="str">
-        <x:v>二轮车/一轮车完成普攻后重置普通移动次数和距离，不重置攻击、技能或神速。</x:v>
+        <x:v>测试需逐项证明技能规则、AI决策、通用AI改动和关键交互边界。</x:v>
       </x:c>
       <x:c r="F52" s="99" t="str">
-        <x:v>ResetMoveAfterAttackTrait只在on_basic_attack_finished清零move_used、normal_move_actions_used、normal_move_steps_used。</x:v>
+        <x:v>2026-09-06新回归933项，本批唯一失败是测试沿用旧说明的两格回避，合法预览实际为一格；按既定技能索引修正选区及落点，并保留真实连锁结算后的等量交换断言。其他太阳神、赤、犀牛专属测试未列入失败；三名尚未整批签收。</x:v>
       </x:c>
       <x:c r="G52" s="99" t="str">
-        <x:v>符合</x:v>
+        <x:v>已补充待验证</x:v>
       </x:c>
       <x:c r="H52" s="99" t="str">
-        <x:v>P3</x:v>
+        <x:v>P1</x:v>
       </x:c>
       <x:c r="I52" s="99" t="str">
-        <x:v>保留实现。</x:v>
+        <x:v>拆分/补充定向回归与AI测试；只写入统一总测试，不由开发代理运行。</x:v>
       </x:c>
       <x:c r="J52" s="99" t="str">
-        <x:v>待用户当前批次测试</x:v>
+        <x:v>一格回避场景与旧说明已同步，待用户复跑当前批次</x:v>
       </x:c>
       <x:c r="K52" s="99" t="str">
-        <x:v>docs/武将设计思想.json#excel_r198</x:v>
+        <x:v>docs/武将设计思想.json#excel_r126</x:v>
       </x:c>
       <x:c r="L52" s="99" t="str">
-        <x:v>reports/current-hero-deep-audit/excel_r142--excel_r198--excel_r206：2026-09-02全新复测10场、2胜8负、自动高信号0/P3；二轮车召唤10/13个有效机会，一轮车召唤1/1。人工逐步对照再次确认本体召唤→神速/移动→普攻→再次移动，以及二轮车召唤子车→移动→攻击；攻击后未再移动的代表场景随即结束战斗，不构成漏用。当前三将专属测试无失败，未发现实现或AI偏离设计。</x:v>
+        <x:v>9月4日新10场4胜5负、1场500步未决，自动高信号0；炮台7次、爆炎4次、审判7次、石墙19次。第5场步骤19爆炎、22审判，击破咏唱者与蝴蝶刺客；蕾米阵亡带走蝙蝠。第7场17审判、18托尔反击、19太阳神先阵亡，审判未结算。第2场末尾为盖泽尔与李持续交战，不能归为太阳神卡死。929项回归32条失败/错误，本批1条为审判选区测试缺陷，其余31条为既有战略/房间/前端/军团炮/时间停止范围。</x:v>
       </x:c>
       <x:c r="M52" s="99" t="str">
         <x:v>2026-09-06用户调整：连续分批完成全部已开发武将及AI的设计优先检查修改；保留测试用例和静态检查，中途不运行测试、不等待逐批签收，全部完成后统一测试。</x:v>
@@ -25800,40 +26052,40 @@
     </x:row>
     <x:row r="53" ht="84" customHeight="1">
       <x:c r="A53" s="99" t="str">
-        <x:v>excel_r198</x:v>
+        <x:v>excel_r126</x:v>
       </x:c>
       <x:c r="B53" s="99" t="str">
-        <x:v>三轮车人</x:v>
+        <x:v>太阳神</x:v>
       </x:c>
       <x:c r="C53" s="99" t="str">
-        <x:v>已完整验收：设计、5项设计推断、战斗实现、AI、测试与两轮用户日志均已逐层审查；召唤顺序、攻击后移动经济与AI重规划符合设计，2026-09-02复测未发现新缺陷</x:v>
+        <x:v>2026-09-06复核新10场：第7场已避开托尔致命反击陷阱，第5场审判击破两敌；933项回归本批仅剩一项测试沿用过期两格回避口径，现按技能索引一格规则修正测试与说明，待复跑。</x:v>
       </x:c>
       <x:c r="D53" s="99" t="str">
-        <x:v>战斗实现</x:v>
+        <x:v>审计工具</x:v>
       </x:c>
       <x:c r="E53" s="99" t="str">
-        <x:v>允许多座二轮车并存，每座独立召唤一轮车；所有召唤相邻部署、入场禁动。</x:v>
+        <x:v>随机对局只有在出现对应机会时才应报告条件性日志缺失。</x:v>
       </x:c>
       <x:c r="F53" s="99" t="str">
-        <x:v>两个召唤技能按各自actor周围合法格生成且无场上同名上限；每个BicycleSummon拥有独立SummonUnicycleSkill；Battle.summon_unit令turn_ready=false。</x:v>
+        <x:v>旧审计把‘破坏了地形’列为无条件日志并曾误报；本轮又确认仅记录技能可用不足以判断错失，且他人同名动作/日志可能串入目标武将。现把‘存在有效候选但未选’列为高优先级错失，把‘可用但无有效候选’列为覆盖缺口，并按事件中的动作来源、目标和相关单位归因。</x:v>
       </x:c>
       <x:c r="G53" s="99" t="str">
-        <x:v>符合</x:v>
+        <x:v>已修复待验证</x:v>
       </x:c>
       <x:c r="H53" s="99" t="str">
-        <x:v>P3</x:v>
+        <x:v>P1</x:v>
       </x:c>
       <x:c r="I53" s="99" t="str">
-        <x:v>新增两条并存分支及各自子召唤测试。</x:v>
+        <x:v>保留条件日志与召唤生命周期指标；新增有效机会分类和跨武将日志隔离。</x:v>
       </x:c>
       <x:c r="J53" s="99" t="str">
-        <x:v>待用户当前批次测试</x:v>
+        <x:v>审计分类与归因已二次修正，待用户复跑当前批次</x:v>
       </x:c>
       <x:c r="K53" s="99" t="str">
-        <x:v>docs/武将设计思想.json#excel_r198</x:v>
+        <x:v>docs/武将设计思想.json#excel_r126</x:v>
       </x:c>
       <x:c r="L53" s="99" t="str">
-        <x:v>reports/current-hero-deep-audit/excel_r142--excel_r198--excel_r206：2026-09-02全新复测10场、2胜8负、自动高信号0/P3；二轮车召唤10/13个有效机会，一轮车召唤1/1。人工逐步对照再次确认本体召唤→神速/移动→普攻→再次移动，以及二轮车召唤子车→移动→攻击；攻击后未再移动的代表场景随即结束战斗，不构成漏用。当前三将专属测试无失败，未发现实现或AI偏离设计。</x:v>
+        <x:v>9月4日新10场4胜5负、1场500步未决，自动高信号0；炮台7次、爆炎4次、审判7次、石墙19次。第5场步骤19爆炎、22审判，击破咏唱者与蝴蝶刺客；蕾米阵亡带走蝙蝠。第7场17审判、18托尔反击、19太阳神先阵亡，审判未结算。第2场末尾为盖泽尔与李持续交战，不能归为太阳神卡死。929项回归32条失败/错误，本批1条为审判选区测试缺陷，其余31条为既有战略/房间/前端/军团炮/时间停止范围。</x:v>
       </x:c>
       <x:c r="M53" s="99" t="str">
         <x:v>2026-09-06用户调整：连续分批完成全部已开发武将及AI的设计优先检查修改；保留测试用例和静态检查，中途不运行测试、不等待逐批签收，全部完成后统一测试。</x:v>
@@ -25841,40 +26093,40 @@
     </x:row>
     <x:row r="54" ht="84" customHeight="1">
       <x:c r="A54" s="99" t="str">
-        <x:v>excel_r198</x:v>
+        <x:v>excel_r142</x:v>
       </x:c>
       <x:c r="B54" s="99" t="str">
-        <x:v>三轮车人</x:v>
+        <x:v>猫叔</x:v>
       </x:c>
       <x:c r="C54" s="99" t="str">
-        <x:v>已完整验收：设计、5项设计推断、战斗实现、AI、测试与两轮用户日志均已逐层审查；召唤顺序、攻击后移动经济与AI重规划符合设计，2026-09-02复测未发现新缺陷</x:v>
+        <x:v>已完整验收：设计、5项设计推断、战斗实现、通用AI、测试与两轮用户日志均已逐层审查；同一范围动作重复反制已按声明动作token修复，2026-09-02复测30场中猫叔32次反制均为单token单触发</x:v>
       </x:c>
       <x:c r="D54" s="99" t="str">
         <x:v>战斗实现</x:v>
       </x:c>
       <x:c r="E54" s="99" t="str">
-        <x:v>召唤消散必须按直接召唤者分支级联。</x:v>
+        <x:v>嘲讽之吼必须对周围7×7敌我双方造成当前攻4的破魔伤害，再给仍存活命中单位施加指定攻击。</x:v>
       </x:c>
       <x:c r="F54" s="99" t="str">
-        <x:v>Battle.summon_unit记录直接summoner_id；cleanup_dead_units循环清理召唤者已死亡的单位，因此三轮车人→二轮车→一轮车逐层级联，单座二轮车死亡不影响另一分支。</x:v>
+        <x:v>旧CatTauntRoarSkill明确写成敌方、无伤害，只调用validate_target并加状态；现改为effect_units_at_cells双方取值、DamageContext当前攻、ignore_shield，并仅在伤害未取消且目标存活后加状态。</x:v>
       </x:c>
       <x:c r="G54" s="99" t="str">
-        <x:v>符合</x:v>
+        <x:v>已修复待验证</x:v>
       </x:c>
       <x:c r="H54" s="99" t="str">
-        <x:v>P3</x:v>
+        <x:v>P1</x:v>
       </x:c>
       <x:c r="I54" s="99" t="str">
-        <x:v>新增单分支清理、另一分支保留的测试。</x:v>
+        <x:v>已补敌我伤害、破盾和状态顺序的定向测试。</x:v>
       </x:c>
       <x:c r="J54" s="99" t="str">
         <x:v>待用户当前批次测试</x:v>
       </x:c>
       <x:c r="K54" s="99" t="str">
-        <x:v>docs/武将设计思想.json#excel_r198</x:v>
+        <x:v>docs/武将设计思想.json#excel_r142</x:v>
       </x:c>
       <x:c r="L54" s="99" t="str">
-        <x:v>reports/current-hero-deep-audit/excel_r142--excel_r198--excel_r206：2026-09-02全新复测10场、2胜8负、自动高信号0/P3；二轮车召唤10/13个有效机会，一轮车召唤1/1。人工逐步对照再次确认本体召唤→神速/移动→普攻→再次移动，以及二轮车召唤子车→移动→攻击；攻击后未再移动的代表场景随即结束战斗，不构成漏用。当前三将专属测试无失败，未发现实现或AI偏离设计。</x:v>
+        <x:v>reports/current-hero-deep-audit/excel_r142--excel_r198--excel_r206：2026-09-02全新复测10场、8胜2负、自动高信号0/P3；猫叔反制32次。人工扫描30份trace确认不存在同token重复rule_trigger，也不存在单步重复反制；原第10场龙范围普攻现只触发一次。当前三将专属测试未出现在919项回归的31个失败/错误中，其余失败已归类为战略、房间、前端、军团炮或时间停止等非本批范围。</x:v>
       </x:c>
       <x:c r="M54" s="99" t="str">
         <x:v>2026-09-06用户调整：连续分批完成全部已开发武将及AI的设计优先检查修改；保留测试用例和静态检查，中途不运行测试、不等待逐批签收，全部完成后统一测试。</x:v>
@@ -25882,40 +26134,40 @@
     </x:row>
     <x:row r="55" ht="84" customHeight="1">
       <x:c r="A55" s="99" t="str">
-        <x:v>excel_r198</x:v>
+        <x:v>excel_r142</x:v>
       </x:c>
       <x:c r="B55" s="99" t="str">
-        <x:v>三轮车人</x:v>
+        <x:v>猫叔</x:v>
       </x:c>
       <x:c r="C55" s="99" t="str">
-        <x:v>已完整验收：设计、5项设计推断、战斗实现、AI、测试与两轮用户日志均已逐层审查；召唤顺序、攻击后移动经济与AI重规划符合设计，2026-09-02复测未发现新缺陷</x:v>
+        <x:v>已完整验收：设计、5项设计推断、战斗实现、通用AI、测试与两轮用户日志均已逐层审查；同一范围动作重复反制已按声明动作token修复，2026-09-02复测30场中猫叔32次反制均为单token单触发</x:v>
       </x:c>
       <x:c r="D55" s="99" t="str">
-        <x:v>AI</x:v>
+        <x:v>战斗实现</x:v>
       </x:c>
       <x:c r="E55" s="99" t="str">
-        <x:v>二轮车落点应同时考虑入场暴露、下回合攻击接触和未来一轮车合法空位。</x:v>
+        <x:v>猫叔反制必须覆盖敌我普攻/技能以及直接区域伤害，并且一个声明动作只触发一次。</x:v>
       </x:c>
       <x:c r="F55" s="99" t="str">
-        <x:v>旧通用召唤评分只奖励接近敌人；现cycle_summon_score计算下一轮速5+范1接触、敌方可达威胁、过近惩罚，并让二轮车强烈保留邻接空格。</x:v>
+        <x:v>第一版修复虽共享_trigger接入on_targeted/on_before_damage，但用回合、来源、动作名和动作序号去重；用户日志证明龙的一次范围普攻在伤害与后续效果使用不同动作名，仍重复触发。现Battle为每个已声明QueuedAction提供稳定resolution token，两个钩子按同一token去重；嵌套声明动作仍各有独立token。</x:v>
       </x:c>
       <x:c r="G55" s="99" t="str">
-        <x:v>已改进待验证</x:v>
+        <x:v>再次修复待验证</x:v>
       </x:c>
       <x:c r="H55" s="99" t="str">
-        <x:v>P2</x:v>
+        <x:v>P1</x:v>
       </x:c>
       <x:c r="I55" s="99" t="str">
-        <x:v>已补受地形限制时仍选择保留子召唤空位的AI测试。</x:v>
+        <x:v>已补友方直接区域技能触发，以及龙的范围普攻含后续效果时整次动作只反制一次的定向测试。</x:v>
       </x:c>
       <x:c r="J55" s="99" t="str">
-        <x:v>待用户当前批次测试</x:v>
+        <x:v>待用户重跑当前批次</x:v>
       </x:c>
       <x:c r="K55" s="99" t="str">
-        <x:v>docs/武将设计思想.json#excel_r198</x:v>
+        <x:v>docs/武将设计思想.json#excel_r142</x:v>
       </x:c>
       <x:c r="L55" s="99" t="str">
-        <x:v>reports/current-hero-deep-audit/excel_r142--excel_r198--excel_r206：2026-09-02全新复测10场、2胜8负、自动高信号0/P3；二轮车召唤10/13个有效机会，一轮车召唤1/1。人工逐步对照再次确认本体召唤→神速/移动→普攻→再次移动，以及二轮车召唤子车→移动→攻击；攻击后未再移动的代表场景随即结束战斗，不构成漏用。当前三将专属测试无失败，未发现实现或AI偏离设计。</x:v>
+        <x:v>reports/current-hero-deep-audit/excel_r142--excel_r198--excel_r206：2026-09-02全新复测10场、8胜2负、自动高信号0/P3；猫叔反制32次。人工扫描30份trace确认不存在同token重复rule_trigger，也不存在单步重复反制；原第10场龙范围普攻现只触发一次。当前三将专属测试未出现在919项回归的31个失败/错误中，其余失败已归类为战略、房间、前端、军团炮或时间停止等非本批范围。</x:v>
       </x:c>
       <x:c r="M55" s="99" t="str">
         <x:v>2026-09-06用户调整：连续分批完成全部已开发武将及AI的设计优先检查修改；保留测试用例和静态检查，中途不运行测试、不等待逐批签收，全部完成后统一测试。</x:v>
@@ -25923,40 +26175,40 @@
     </x:row>
     <x:row r="56">
       <x:c r="A56" t="str">
-        <x:v>excel_r198</x:v>
+        <x:v>excel_r142</x:v>
       </x:c>
       <x:c r="B56" t="str">
-        <x:v>三轮车人</x:v>
+        <x:v>猫叔</x:v>
       </x:c>
       <x:c r="C56" t="str">
-        <x:v>已完整验收：设计、5项设计推断、战斗实现、AI、测试与两轮用户日志均已逐层审查；召唤顺序、攻击后移动经济与AI重规划符合设计，2026-09-02复测未发现新缺陷</x:v>
+        <x:v>已完整验收：设计、5项设计推断、战斗实现、通用AI、测试与两轮用户日志均已逐层审查；同一范围动作重复反制已按声明动作token修复，2026-09-02复测30场中猫叔32次反制均为单token单触发</x:v>
       </x:c>
       <x:c r="D56" t="str">
-        <x:v>通用AI</x:v>
+        <x:v>战斗实现</x:v>
       </x:c>
       <x:c r="E56" t="str">
-        <x:v>车体攻击重置移动后必须重新生成动作候选，实现移动→攻击→再移动。</x:v>
+        <x:v>直线拉近应走到合法直线上距离猫叔最近的可达点，而不是找不到恰好邻接共线格就完全不移动。</x:v>
       </x:c>
       <x:c r="F56" t="str">
-        <x:v>choose_turn_action/choose_turn_bundle_action每次行动后重新读取action_snapshot；ResetMoveAfterAttackTrait在普攻完成时立即清零移动使用量。新增测试锁定攻击后再次生成move。</x:v>
+        <x:v>旧_straight_destination_around只搜索与起点严格共线的邻接落点；现枚举八方向可达直线点，先取与猫叔距离最小者，再取达到同等最近距离所需步数最少者，障碍前停止。</x:v>
       </x:c>
       <x:c r="G56" t="str">
-        <x:v>符合并补测试</x:v>
+        <x:v>已修复待验证</x:v>
       </x:c>
       <x:c r="H56" t="str">
         <x:v>P2</x:v>
       </x:c>
       <x:c r="I56" t="str">
-        <x:v>保留动态重规划架构，观察当前批次日志中的攻击后移动机会采用率。</x:v>
+        <x:v>已补非共线起点仍沿直线显著拉近的定向测试。</x:v>
       </x:c>
       <x:c r="J56" t="str">
         <x:v>待用户当前批次测试</x:v>
       </x:c>
       <x:c r="K56" t="str">
-        <x:v>docs/武将设计思想.json#excel_r198</x:v>
+        <x:v>docs/武将设计思想.json#excel_r142</x:v>
       </x:c>
       <x:c r="L56" t="str">
-        <x:v>reports/current-hero-deep-audit/excel_r142--excel_r198--excel_r206：2026-09-02全新复测10场、2胜8负、自动高信号0/P3；二轮车召唤10/13个有效机会，一轮车召唤1/1。人工逐步对照再次确认本体召唤→神速/移动→普攻→再次移动，以及二轮车召唤子车→移动→攻击；攻击后未再移动的代表场景随即结束战斗，不构成漏用。当前三将专属测试无失败，未发现实现或AI偏离设计。</x:v>
+        <x:v>reports/current-hero-deep-audit/excel_r142--excel_r198--excel_r206：2026-09-02全新复测10场、8胜2负、自动高信号0/P3；猫叔反制32次。人工扫描30份trace确认不存在同token重复rule_trigger，也不存在单步重复反制；原第10场龙范围普攻现只触发一次。当前三将专属测试未出现在919项回归的31个失败/错误中，其余失败已归类为战略、房间、前端、军团炮或时间停止等非本批范围。</x:v>
       </x:c>
       <x:c r="M56" t="str">
         <x:v>2026-09-06用户调整：连续分批完成全部已开发武将及AI的设计优先检查修改；保留测试用例和静态检查，中途不运行测试、不等待逐批签收，全部完成后统一测试。</x:v>
@@ -25964,40 +26216,40 @@
     </x:row>
     <x:row r="57">
       <x:c r="A57" t="str">
-        <x:v>excel_r198</x:v>
+        <x:v>excel_r142</x:v>
       </x:c>
       <x:c r="B57" t="str">
-        <x:v>三轮车人</x:v>
+        <x:v>猫叔</x:v>
       </x:c>
       <x:c r="C57" t="str">
-        <x:v>已完整验收：设计、5项设计推断、战斗实现、AI、测试与两轮用户日志均已逐层审查；召唤顺序、攻击后移动经济与AI重规划符合设计，2026-09-02复测未发现新缺陷</x:v>
+        <x:v>已完整验收：设计、5项设计推断、战斗实现、通用AI、测试与两轮用户日志均已逐层审查；同一范围动作重复反制已按声明动作token修复，2026-09-02复测30场中猫叔32次反制均为单token单触发</x:v>
       </x:c>
       <x:c r="D57" t="str">
-        <x:v>测试</x:v>
+        <x:v>通用战斗规则</x:v>
       </x:c>
       <x:c r="E57" t="str">
-        <x:v>测试需覆盖独立召唤分支、入场禁动、移动增益/重置、级联和AI重规划。</x:v>
+        <x:v>被双方区域嘲讽命中的己方单位必须能把己方猫叔作为合法强制普攻目标。</x:v>
       </x:c>
       <x:c r="F57" t="str">
-        <x:v>tests/test_battle.py与tests/test_behavior.py已扩充上述场景；本轮不运行动态测试。</x:v>
+        <x:v>旧basic_attack_preview_for_payload只枚举enemy_units，造成友方指定目标不可执行；现Battle.forced_basic_attack_target把有效指定目标加入普攻预览，并在声明时冻结友方目标许可，单体和区域普攻结算均可完成契约。</x:v>
       </x:c>
       <x:c r="G57" t="str">
-        <x:v>已补充待验证</x:v>
+        <x:v>已修复待验证</x:v>
       </x:c>
       <x:c r="H57" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="I57" t="str">
-        <x:v>由用户运行当前批次统一测试。</x:v>
+        <x:v>通用指定攻击目标动作生成与AI候选均已支持己方强制目标。</x:v>
       </x:c>
       <x:c r="J57" t="str">
-        <x:v>首轮日志符合，待统一回归重跑</x:v>
+        <x:v>待用户当前批次测试</x:v>
       </x:c>
       <x:c r="K57" t="str">
-        <x:v>docs/武将设计思想.json#excel_r198</x:v>
+        <x:v>docs/武将设计思想.json#excel_r142</x:v>
       </x:c>
       <x:c r="L57" t="str">
-        <x:v>reports/current-hero-deep-audit/excel_r142--excel_r198--excel_r206：2026-09-02全新复测10场、2胜8负、自动高信号0/P3；二轮车召唤10/13个有效机会，一轮车召唤1/1。人工逐步对照再次确认本体召唤→神速/移动→普攻→再次移动，以及二轮车召唤子车→移动→攻击；攻击后未再移动的代表场景随即结束战斗，不构成漏用。当前三将专属测试无失败，未发现实现或AI偏离设计。</x:v>
+        <x:v>reports/current-hero-deep-audit/excel_r142--excel_r198--excel_r206：2026-09-02全新复测10场、8胜2负、自动高信号0/P3；猫叔反制32次。人工扫描30份trace确认不存在同token重复rule_trigger，也不存在单步重复反制；原第10场龙范围普攻现只触发一次。当前三将专属测试未出现在919项回归的31个失败/错误中，其余失败已归类为战略、房间、前端、军团炮或时间停止等非本批范围。</x:v>
       </x:c>
       <x:c r="M57" t="str">
         <x:v>2026-09-06用户调整：连续分批完成全部已开发武将及AI的设计优先检查修改；保留测试用例和静态检查，中途不运行测试、不等待逐批签收，全部完成后统一测试。</x:v>
@@ -26005,22 +26257,22 @@
     </x:row>
     <x:row r="58">
       <x:c r="A58" t="str">
-        <x:v>excel_r206</x:v>
+        <x:v>excel_r142</x:v>
       </x:c>
       <x:c r="B58" t="str">
-        <x:v>反击拳手</x:v>
+        <x:v>猫叔</x:v>
       </x:c>
       <x:c r="C58" t="str">
-        <x:v>已完整验收：设计、6项设计推断、战斗实现、通用AI、测试与两轮用户日志均已逐层审查；嘲讽服从、反应选择、临时防御与吸血符合设计，2026-09-02复测未发现新缺陷</x:v>
+        <x:v>已完整验收：设计、5项设计推断、战斗实现、通用AI、测试与两轮用户日志均已逐层审查；同一范围动作重复反制已按声明动作token修复，2026-09-02复测30场中猫叔32次反制均为单token单触发</x:v>
       </x:c>
       <x:c r="D58" t="str">
-        <x:v>战斗实现</x:v>
+        <x:v>AI</x:v>
       </x:c>
       <x:c r="E58" t="str">
-        <x:v>擂台嘲讽必须对周围8格敌我双方造成当前攻3破魔伤害，再给存活命中单位施加指定攻击。</x:v>
+        <x:v>猫叔AI必须把怒吼的攻4伤害、控制收益、友伤、队友强制攻击和自身未来承伤放在同一净值中。</x:v>
       </x:c>
       <x:c r="F58" t="str">
-        <x:v>旧RingTauntSkill明确实现为敌方、无伤害；现改为双方区域DamageContext、当前攻、ignore_shield，伤害成功且存活后才加状态。</x:v>
+        <x:v>旧taunt_control_score只统计敌方控制数量；现用真实技能伤害探针计算敌我伤害与破盾，敌方控制扣除预计反打，友方加入伤害及攻击资源浪费惩罚。</x:v>
       </x:c>
       <x:c r="G58" t="str">
         <x:v>已修复待验证</x:v>
@@ -26029,16 +26281,16 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="I58" t="str">
-        <x:v>已补敌我伤害、破盾与控制顺序测试。</x:v>
+        <x:v>已补两名队友在范围内时拒绝怒吼的AI测试。</x:v>
       </x:c>
       <x:c r="J58" t="str">
         <x:v>待用户当前批次测试</x:v>
       </x:c>
       <x:c r="K58" t="str">
-        <x:v>docs/武将设计思想.json#excel_r206</x:v>
+        <x:v>docs/武将设计思想.json#excel_r142</x:v>
       </x:c>
       <x:c r="L58" t="str">
-        <x:v>reports/current-hero-deep-audit/excel_r142--excel_r198--excel_r206：2026-09-02全新复测10场、8胜2负、自动高信号0/P3；擂台嘲讽7/37，组合格挡反击33/35，保护3次、普通格挡4次。人工逐步对照再次确认被嘲讽单位服从指定攻击，组合反击先结算、临时守链尾清除、实际伤害触发吸血，AI会按威胁切换保护/格挡。普通反击因组合通常严格占优而未采用，合法候选与定向测试均保留；当前三将专属测试无失败，未发现新缺陷。</x:v>
+        <x:v>reports/current-hero-deep-audit/excel_r142--excel_r198--excel_r206：2026-09-02全新复测10场、8胜2负、自动高信号0/P3；猫叔反制32次。人工扫描30份trace确认不存在同token重复rule_trigger，也不存在单步重复反制；原第10场龙范围普攻现只触发一次。当前三将专属测试未出现在919项回归的31个失败/错误中，其余失败已归类为战略、房间、前端、军团炮或时间停止等非本批范围。</x:v>
       </x:c>
       <x:c r="M58" t="str">
         <x:v>2026-09-06用户调整：连续分批完成全部已开发武将及AI的设计优先检查修改；保留测试用例和静态检查，中途不运行测试、不等待逐批签收，全部完成后统一测试。</x:v>
@@ -26046,40 +26298,40 @@
     </x:row>
     <x:row r="59">
       <x:c r="A59" t="str">
-        <x:v>excel_r206</x:v>
+        <x:v>excel_r142</x:v>
       </x:c>
       <x:c r="B59" t="str">
-        <x:v>反击拳手</x:v>
+        <x:v>猫叔</x:v>
       </x:c>
       <x:c r="C59" t="str">
-        <x:v>已完整验收：设计、6项设计推断、战斗实现、通用AI、测试与两轮用户日志均已逐层审查；嘲讽服从、反应选择、临时防御与吸血符合设计，2026-09-02复测未发现新缺陷</x:v>
+        <x:v>已完整验收：设计、5项设计推断、战斗实现、通用AI、测试与两轮用户日志均已逐层审查；同一范围动作重复反制已按声明动作token修复，2026-09-02复测30场中猫叔32次反制均为单token单触发</x:v>
       </x:c>
       <x:c r="D59" t="str">
-        <x:v>战斗实现</x:v>
+        <x:v>通用AI</x:v>
       </x:c>
       <x:c r="E59" t="str">
-        <x:v>目标下回合有普攻资源时才激活指定攻击；声明消耗正常次数并解除，拳手离场/回合结束清除。</x:v>
+        <x:v>所有单位选择攻击或技能影响猫叔时都要计入扣魔、被拉近和后续移动/主动技能锁定成本。</x:v>
       </x:c>
       <x:c r="F59" t="str">
-        <x:v>RequiredAttackStatus已实现声明解除、来源失效、owner_turn_end过期与最新覆盖；BoxerTauntStatus补充无可用攻击次数时不激活。</x:v>
+        <x:v>旧攻击与技能评分没有猫叔反制成本；现build_attack_candidates/build_skill_candidates统一扣除猫叔反制机会成本，强制攻击以高契约分覆盖该惩罚。</x:v>
       </x:c>
       <x:c r="G59" t="str">
         <x:v>已修复待验证</x:v>
       </x:c>
       <x:c r="H59" t="str">
-        <x:v>P2</x:v>
+        <x:v>P1</x:v>
       </x:c>
       <x:c r="I59" t="str">
-        <x:v>补充无攻击数和友方强制目标测试。</x:v>
+        <x:v>已补有暴露替代目标时通用AI避开猫叔、被嘲讽时仍正确攻击猫叔的测试。</x:v>
       </x:c>
       <x:c r="J59" t="str">
         <x:v>待用户当前批次测试</x:v>
       </x:c>
       <x:c r="K59" t="str">
-        <x:v>docs/武将设计思想.json#excel_r206</x:v>
+        <x:v>docs/武将设计思想.json#excel_r142</x:v>
       </x:c>
       <x:c r="L59" t="str">
-        <x:v>reports/current-hero-deep-audit/excel_r142--excel_r198--excel_r206：2026-09-02全新复测10场、8胜2负、自动高信号0/P3；擂台嘲讽7/37，组合格挡反击33/35，保护3次、普通格挡4次。人工逐步对照再次确认被嘲讽单位服从指定攻击，组合反击先结算、临时守链尾清除、实际伤害触发吸血，AI会按威胁切换保护/格挡。普通反击因组合通常严格占优而未采用，合法候选与定向测试均保留；当前三将专属测试无失败，未发现新缺陷。</x:v>
+        <x:v>reports/current-hero-deep-audit/excel_r142--excel_r198--excel_r206：2026-09-02全新复测10场、8胜2负、自动高信号0/P3；猫叔反制32次。人工扫描30份trace确认不存在同token重复rule_trigger，也不存在单步重复反制；原第10场龙范围普攻现只触发一次。当前三将专属测试未出现在919项回归的31个失败/错误中，其余失败已归类为战略、房间、前端、军团炮或时间停止等非本批范围。</x:v>
       </x:c>
       <x:c r="M59" t="str">
         <x:v>2026-09-06用户调整：连续分批完成全部已开发武将及AI的设计优先检查修改；保留测试用例和静态检查，中途不运行测试、不等待逐批签收，全部完成后统一测试。</x:v>
@@ -26087,40 +26339,40 @@
     </x:row>
     <x:row r="60">
       <x:c r="A60" t="str">
-        <x:v>excel_r206</x:v>
+        <x:v>excel_r142</x:v>
       </x:c>
       <x:c r="B60" t="str">
-        <x:v>反击拳手</x:v>
+        <x:v>猫叔</x:v>
       </x:c>
       <x:c r="C60" t="str">
-        <x:v>已完整验收：设计、6项设计推断、战斗实现、通用AI、测试与两轮用户日志均已逐层审查；嘲讽服从、反应选择、临时防御与吸血符合设计，2026-09-02复测未发现新缺陷</x:v>
+        <x:v>已完整验收：设计、5项设计推断、战斗实现、通用AI、测试与两轮用户日志均已逐层审查；同一范围动作重复反制已按声明动作token修复，2026-09-02复测30场中猫叔32次反制均为单token单触发</x:v>
       </x:c>
       <x:c r="D60" t="str">
-        <x:v>通用战斗规则</x:v>
+        <x:v>通用AI</x:v>
       </x:c>
       <x:c r="E60" t="str">
-        <x:v>被擂台嘲讽命中的己方单位必须能合法普攻己方拳手。</x:v>
+        <x:v>震开要计算推散已聚拢单位、损失后续近战接触与1魔资源的机会成本，致命防御时仍可使用。</x:v>
       </x:c>
       <x:c r="F60" t="str">
-        <x:v>Battle.forced_basic_attack_target及声明冻结许可同时服务猫叔与反击拳手；AI候选也允许只为完成契约而攻击指定己方目标。</x:v>
+        <x:v>旧knockback固定按威胁加分；现按周围敌人的未来近战价值、被推队友和低魔非紧急场景扣分，保留致命威胁的高紧急分。</x:v>
       </x:c>
       <x:c r="G60" t="str">
-        <x:v>已修复待验证</x:v>
+        <x:v>已改进待验证</x:v>
       </x:c>
       <x:c r="H60" t="str">
-        <x:v>P1</x:v>
+        <x:v>P2</x:v>
       </x:c>
       <x:c r="I60" t="str">
-        <x:v>复用通用指定攻击测试。</x:v>
+        <x:v>通过当前批次决策日志观察猫叔是否仍无条件震开。</x:v>
       </x:c>
       <x:c r="J60" t="str">
         <x:v>待用户当前批次测试</x:v>
       </x:c>
       <x:c r="K60" t="str">
-        <x:v>docs/武将设计思想.json#excel_r206</x:v>
+        <x:v>docs/武将设计思想.json#excel_r142</x:v>
       </x:c>
       <x:c r="L60" t="str">
-        <x:v>reports/current-hero-deep-audit/excel_r142--excel_r198--excel_r206：2026-09-02全新复测10场、8胜2负、自动高信号0/P3；擂台嘲讽7/37，组合格挡反击33/35，保护3次、普通格挡4次。人工逐步对照再次确认被嘲讽单位服从指定攻击，组合反击先结算、临时守链尾清除、实际伤害触发吸血，AI会按威胁切换保护/格挡。普通反击因组合通常严格占优而未采用，合法候选与定向测试均保留；当前三将专属测试无失败，未发现新缺陷。</x:v>
+        <x:v>reports/current-hero-deep-audit/excel_r142--excel_r198--excel_r206：2026-09-02全新复测10场、8胜2负、自动高信号0/P3；猫叔反制32次。人工扫描30份trace确认不存在同token重复rule_trigger，也不存在单步重复反制；原第10场龙范围普攻现只触发一次。当前三将专属测试未出现在919项回归的31个失败/错误中，其余失败已归类为战略、房间、前端、军团炮或时间停止等非本批范围。</x:v>
       </x:c>
       <x:c r="M60" t="str">
         <x:v>2026-09-06用户调整：连续分批完成全部已开发武将及AI的设计优先检查修改；保留测试用例和静态检查，中途不运行测试、不等待逐批签收，全部完成后统一测试。</x:v>
@@ -26128,40 +26380,40 @@
     </x:row>
     <x:row r="61">
       <x:c r="A61" t="str">
-        <x:v>excel_r206</x:v>
+        <x:v>excel_r142</x:v>
       </x:c>
       <x:c r="B61" t="str">
-        <x:v>反击拳手</x:v>
+        <x:v>猫叔</x:v>
       </x:c>
       <x:c r="C61" t="str">
-        <x:v>已完整验收：设计、6项设计推断、战斗实现、通用AI、测试与两轮用户日志均已逐层审查；嘲讽服从、反应选择、临时防御与吸血符合设计，2026-09-02复测未发现新缺陷</x:v>
+        <x:v>已完整验收：设计、5项设计推断、战斗实现、通用AI、测试与两轮用户日志均已逐层审查；同一范围动作重复反制已按声明动作token修复，2026-09-02复测30场中猫叔32次反制均为单token单触发</x:v>
       </x:c>
       <x:c r="D61" t="str">
-        <x:v>战斗实现</x:v>
+        <x:v>审计工具</x:v>
       </x:c>
       <x:c r="E61" t="str">
-        <x:v>普通格挡、普通反击和组合格挡反击必须同时保留；组合只对敌方速度1、来源在范围的动作开放。</x:v>
+        <x:v>自动审计必须把同一声明动作重复触发一次性反制识别为高信号，不能仅因对局无执行异常就给P3。</x:v>
       </x:c>
       <x:c r="F61" t="str">
-        <x:v>BlockCounterTrait提供普通两个候选；BoxerBlockCounterSkill为额外被动技能，can_react_to检查敌方、速度与attack_target_allowed范围。</x:v>
+        <x:v>旧报告自动高信号为0，但同一步trace出现两条‘因攻击或技能猫叔失去’日志。现猫叔每次实际反制都会写入带action resolution token的结构化rule_trigger事件；match_audit按token检查一次性触发不变量，并以duplicate_once_per_action_trigger记录error；不同嵌套动作的token不同，不会误报。batch审计把该分类列入高信号。</x:v>
       </x:c>
       <x:c r="G61" t="str">
-        <x:v>符合</x:v>
+        <x:v>已修复待验证</x:v>
       </x:c>
       <x:c r="H61" t="str">
-        <x:v>P3</x:v>
+        <x:v>P1</x:v>
       </x:c>
       <x:c r="I61" t="str">
-        <x:v>保留实现，补远程来源不生成组合测试。</x:v>
+        <x:v>已补同一token重复事件必须报错、不同嵌套动作token不得误报的审计组件测试；重跑后该历史场景若复现，应进入suspected_defects而非P3。</x:v>
       </x:c>
       <x:c r="J61" t="str">
-        <x:v>待用户当前批次测试</x:v>
+        <x:v>待用户重跑当前批次</x:v>
       </x:c>
       <x:c r="K61" t="str">
-        <x:v>docs/武将设计思想.json#excel_r206</x:v>
+        <x:v>docs/武将设计思想.json#excel_r142</x:v>
       </x:c>
       <x:c r="L61" t="str">
-        <x:v>reports/current-hero-deep-audit/excel_r142--excel_r198--excel_r206：2026-09-02全新复测10场、8胜2负、自动高信号0/P3；擂台嘲讽7/37，组合格挡反击33/35，保护3次、普通格挡4次。人工逐步对照再次确认被嘲讽单位服从指定攻击，组合反击先结算、临时守链尾清除、实际伤害触发吸血，AI会按威胁切换保护/格挡。普通反击因组合通常严格占优而未采用，合法候选与定向测试均保留；当前三将专属测试无失败，未发现新缺陷。</x:v>
+        <x:v>reports/current-hero-deep-audit/excel_r142--excel_r198--excel_r206：2026-09-02全新复测10场、8胜2负、自动高信号0/P3；猫叔反制32次。人工扫描30份trace确认不存在同token重复rule_trigger，也不存在单步重复反制；原第10场龙范围普攻现只触发一次。当前三将专属测试未出现在919项回归的31个失败/错误中，其余失败已归类为战略、房间、前端、军团炮或时间停止等非本批范围。</x:v>
       </x:c>
       <x:c r="M61" t="str">
         <x:v>2026-09-06用户调整：连续分批完成全部已开发武将及AI的设计优先检查修改；保留测试用例和静态检查，中途不运行测试、不等待逐批签收，全部完成后统一测试。</x:v>
@@ -26169,40 +26421,40 @@
     </x:row>
     <x:row r="62">
       <x:c r="A62" t="str">
-        <x:v>excel_r206</x:v>
+        <x:v>excel_r142</x:v>
       </x:c>
       <x:c r="B62" t="str">
-        <x:v>反击拳手</x:v>
+        <x:v>猫叔</x:v>
       </x:c>
       <x:c r="C62" t="str">
-        <x:v>已完整验收：设计、6项设计推断、战斗实现、通用AI、测试与两轮用户日志均已逐层审查；嘲讽服从、反应选择、临时防御与吸血符合设计，2026-09-02复测未发现新缺陷</x:v>
+        <x:v>已完整验收：设计、5项设计推断、战斗实现、通用AI、测试与两轮用户日志均已逐层审查；同一范围动作重复反制已按声明动作token修复，2026-09-02复测30场中猫叔32次反制均为单token单触发</x:v>
       </x:c>
       <x:c r="D62" t="str">
-        <x:v>战斗实现</x:v>
+        <x:v>测试</x:v>
       </x:c>
       <x:c r="E62" t="str">
-        <x:v>组合反应先临时守+1、再进行普攻式反击，链尾清除；反击伤害触发吸血。</x:v>
+        <x:v>测试需覆盖伤害/阵营、破魔、指定攻击、友方强制目标、反制去重/范围触发、拉近和AI净值。</x:v>
       </x:c>
       <x:c r="F62" t="str">
-        <x:v>react先加expire_with_chain TemporaryDefenseStatus，再resolve_attack_damage；该上下文is_skill=false且带attack标签，AttackLifeStealTrait会在实际伤害后回复，finalize_reaction_window清除临时守。</x:v>
+        <x:v>tests/test_battle.py与tests/test_behavior.py已加入对应定向用例；根据用户首轮结果修正了一个会在怒吼前杀死目标的AI测试夹具，以及一个把直线拉近等价落点写死的过度约束断言；本轮遵照流程不运行回合测试。</x:v>
       </x:c>
       <x:c r="G62" t="str">
-        <x:v>符合</x:v>
+        <x:v>已补充待验证</x:v>
       </x:c>
       <x:c r="H62" t="str">
-        <x:v>P3</x:v>
+        <x:v>P1</x:v>
       </x:c>
       <x:c r="I62" t="str">
-        <x:v>补足吸血、链尾清理和穿刺不吸血断言。</x:v>
+        <x:v>由用户运行python detail_test_all_wujiangs.py --current统一执行。</x:v>
       </x:c>
       <x:c r="J62" t="str">
-        <x:v>待用户当前批次测试</x:v>
+        <x:v>待用户重跑</x:v>
       </x:c>
       <x:c r="K62" t="str">
-        <x:v>docs/武将设计思想.json#excel_r206</x:v>
+        <x:v>docs/武将设计思想.json#excel_r142</x:v>
       </x:c>
       <x:c r="L62" t="str">
-        <x:v>reports/current-hero-deep-audit/excel_r142--excel_r198--excel_r206：2026-09-02全新复测10场、8胜2负、自动高信号0/P3；擂台嘲讽7/37，组合格挡反击33/35，保护3次、普通格挡4次。人工逐步对照再次确认被嘲讽单位服从指定攻击，组合反击先结算、临时守链尾清除、实际伤害触发吸血，AI会按威胁切换保护/格挡。普通反击因组合通常严格占优而未采用，合法候选与定向测试均保留；当前三将专属测试无失败，未发现新缺陷。</x:v>
+        <x:v>reports/current-hero-deep-audit/excel_r142--excel_r198--excel_r206：2026-09-02全新复测10场、8胜2负、自动高信号0/P3；猫叔反制32次。人工扫描30份trace确认不存在同token重复rule_trigger，也不存在单步重复反制；原第10场龙范围普攻现只触发一次。当前三将专属测试未出现在919项回归的31个失败/错误中，其余失败已归类为战略、房间、前端、军团炮或时间停止等非本批范围。</x:v>
       </x:c>
       <x:c r="M62" t="str">
         <x:v>2026-09-06用户调整：连续分批完成全部已开发武将及AI的设计优先检查修改；保留测试用例和静态检查，中途不运行测试、不等待逐批签收，全部完成后统一测试。</x:v>
@@ -26210,40 +26462,40 @@
     </x:row>
     <x:row r="63">
       <x:c r="A63" t="str">
-        <x:v>excel_r206</x:v>
+        <x:v>excel_r198</x:v>
       </x:c>
       <x:c r="B63" t="str">
-        <x:v>反击拳手</x:v>
+        <x:v>三轮车人</x:v>
       </x:c>
       <x:c r="C63" t="str">
-        <x:v>已完整验收：设计、6项设计推断、战斗实现、通用AI、测试与两轮用户日志均已逐层审查；嘲讽服从、反应选择、临时防御与吸血符合设计，2026-09-02复测未发现新缺陷</x:v>
+        <x:v>已完整验收：设计、5项设计推断、战斗实现、AI、测试与两轮用户日志均已逐层审查；召唤顺序、攻击后移动经济与AI重规划符合设计，2026-09-02复测未发现新缺陷</x:v>
       </x:c>
       <x:c r="D63" t="str">
-        <x:v>AI</x:v>
+        <x:v>战斗实现</x:v>
       </x:c>
       <x:c r="E63" t="str">
-        <x:v>嘲讽评分必须同时计算攻3伤害、友伤、控制价值、预计承伤、可反击与吸血收益。</x:v>
+        <x:v>本体每完成一次普攻，本回合普通移动上限独立+1，未命中也触发，技能不触发。</x:v>
       </x:c>
       <x:c r="F63" t="str">
-        <x:v>旧taunt_control_score只数敌方控制；现按真实技能伤害探针、敌我阵营、未来攻击资源、预计敌方伤害和拳手反击伤害综合评分。</x:v>
+        <x:v>ExtraMoveAfterAttackTrait以本回合attacks_used修改普通移动上限；攻击次数在普攻结算路径中增加，技能路径不增加，回合刷新后归零。</x:v>
       </x:c>
       <x:c r="G63" t="str">
-        <x:v>已修复待验证</x:v>
+        <x:v>符合</x:v>
       </x:c>
       <x:c r="H63" t="str">
-        <x:v>P1</x:v>
+        <x:v>P3</x:v>
       </x:c>
       <x:c r="I63" t="str">
-        <x:v>已补两名队友邻接时拒绝擂台嘲讽的AI测试。</x:v>
+        <x:v>保留实现，补足多次与未命中边界测试。</x:v>
       </x:c>
       <x:c r="J63" t="str">
         <x:v>待用户当前批次测试</x:v>
       </x:c>
       <x:c r="K63" t="str">
-        <x:v>docs/武将设计思想.json#excel_r206</x:v>
+        <x:v>docs/武将设计思想.json#excel_r198</x:v>
       </x:c>
       <x:c r="L63" t="str">
-        <x:v>reports/current-hero-deep-audit/excel_r142--excel_r198--excel_r206：2026-09-02全新复测10场、8胜2负、自动高信号0/P3；擂台嘲讽7/37，组合格挡反击33/35，保护3次、普通格挡4次。人工逐步对照再次确认被嘲讽单位服从指定攻击，组合反击先结算、临时守链尾清除、实际伤害触发吸血，AI会按威胁切换保护/格挡。普通反击因组合通常严格占优而未采用，合法候选与定向测试均保留；当前三将专属测试无失败，未发现新缺陷。</x:v>
+        <x:v>reports/current-hero-deep-audit/excel_r142--excel_r198--excel_r206：2026-09-02全新复测10场、2胜8负、自动高信号0/P3；二轮车召唤10/13个有效机会，一轮车召唤1/1。人工逐步对照再次确认本体召唤→神速/移动→普攻→再次移动，以及二轮车召唤子车→移动→攻击；攻击后未再移动的代表场景随即结束战斗，不构成漏用。当前三将专属测试无失败，未发现实现或AI偏离设计。</x:v>
       </x:c>
       <x:c r="M63" t="str">
         <x:v>2026-09-06用户调整：连续分批完成全部已开发武将及AI的设计优先检查修改；保留测试用例和静态检查，中途不运行测试、不等待逐批签收，全部完成后统一测试。</x:v>
@@ -26251,40 +26503,40 @@
     </x:row>
     <x:row r="64">
       <x:c r="A64" t="str">
-        <x:v>excel_r206</x:v>
+        <x:v>excel_r198</x:v>
       </x:c>
       <x:c r="B64" t="str">
-        <x:v>反击拳手</x:v>
+        <x:v>三轮车人</x:v>
       </x:c>
       <x:c r="C64" t="str">
-        <x:v>已完整验收：设计、6项设计推断、战斗实现、通用AI、测试与两轮用户日志均已逐层审查；嘲讽服从、反应选择、临时防御与吸血符合设计，2026-09-02复测未发现新缺陷</x:v>
+        <x:v>已完整验收：设计、5项设计推断、战斗实现、AI、测试与两轮用户日志均已逐层审查；召唤顺序、攻击后移动经济与AI重规划符合设计，2026-09-02复测未发现新缺陷</x:v>
       </x:c>
       <x:c r="D64" t="str">
-        <x:v>通用AI</x:v>
+        <x:v>战斗实现</x:v>
       </x:c>
       <x:c r="E64" t="str">
-        <x:v>格挡类AI要按守+1实际减少的伤害评分，不能把破魔误当成无视防御；组合还要计算反击击杀与吸血。</x:v>
+        <x:v>二轮车/一轮车完成普攻后重置普通移动次数和距离，不重置攻击、技能或神速。</x:v>
       </x:c>
       <x:c r="F64" t="str">
-        <x:v>旧block分支遇ignore_shield直接否决，混淆破魔与守+1；现temporary_defense_prevention_score在回滚探针内比较守+1前后威胁，组合评分再加入反击、击杀与缺血吸血价值。</x:v>
+        <x:v>ResetMoveAfterAttackTrait只在on_basic_attack_finished清零move_used、normal_move_actions_used、normal_move_steps_used。</x:v>
       </x:c>
       <x:c r="G64" t="str">
-        <x:v>已修复待验证</x:v>
+        <x:v>符合</x:v>
       </x:c>
       <x:c r="H64" t="str">
-        <x:v>P1</x:v>
+        <x:v>P3</x:v>
       </x:c>
       <x:c r="I64" t="str">
-        <x:v>保留普通格挡/反击作为合法替代，当前批次观察组合采用质量。</x:v>
+        <x:v>保留实现。</x:v>
       </x:c>
       <x:c r="J64" t="str">
         <x:v>待用户当前批次测试</x:v>
       </x:c>
       <x:c r="K64" t="str">
-        <x:v>docs/武将设计思想.json#excel_r206</x:v>
+        <x:v>docs/武将设计思想.json#excel_r198</x:v>
       </x:c>
       <x:c r="L64" t="str">
-        <x:v>reports/current-hero-deep-audit/excel_r142--excel_r198--excel_r206：2026-09-02全新复测10场、8胜2负、自动高信号0/P3；擂台嘲讽7/37，组合格挡反击33/35，保护3次、普通格挡4次。人工逐步对照再次确认被嘲讽单位服从指定攻击，组合反击先结算、临时守链尾清除、实际伤害触发吸血，AI会按威胁切换保护/格挡。普通反击因组合通常严格占优而未采用，合法候选与定向测试均保留；当前三将专属测试无失败，未发现新缺陷。</x:v>
+        <x:v>reports/current-hero-deep-audit/excel_r142--excel_r198--excel_r206：2026-09-02全新复测10场、2胜8负、自动高信号0/P3；二轮车召唤10/13个有效机会，一轮车召唤1/1。人工逐步对照再次确认本体召唤→神速/移动→普攻→再次移动，以及二轮车召唤子车→移动→攻击；攻击后未再移动的代表场景随即结束战斗，不构成漏用。当前三将专属测试无失败，未发现实现或AI偏离设计。</x:v>
       </x:c>
       <x:c r="M64" t="str">
         <x:v>2026-09-06用户调整：连续分批完成全部已开发武将及AI的设计优先检查修改；保留测试用例和静态检查，中途不运行测试、不等待逐批签收，全部完成后统一测试。</x:v>
@@ -26292,40 +26544,40 @@
     </x:row>
     <x:row r="65">
       <x:c r="A65" t="str">
-        <x:v>excel_r206</x:v>
+        <x:v>excel_r198</x:v>
       </x:c>
       <x:c r="B65" t="str">
-        <x:v>反击拳手</x:v>
+        <x:v>三轮车人</x:v>
       </x:c>
       <x:c r="C65" t="str">
-        <x:v>已完整验收：设计、6项设计推断、战斗实现、通用AI、测试与两轮用户日志均已逐层审查；嘲讽服从、反应选择、临时防御与吸血符合设计，2026-09-02复测未发现新缺陷</x:v>
+        <x:v>已完整验收：设计、5项设计推断、战斗实现、AI、测试与两轮用户日志均已逐层审查；召唤顺序、攻击后移动经济与AI重规划符合设计，2026-09-02复测未发现新缺陷</x:v>
       </x:c>
       <x:c r="D65" t="str">
-        <x:v>测试</x:v>
+        <x:v>战斗实现</x:v>
       </x:c>
       <x:c r="E65" t="str">
-        <x:v>测试需覆盖双方嘲讽、普攻资源门槛、三个反应候选、临时守、反击吸血与AI选择。</x:v>
+        <x:v>允许多座二轮车并存，每座独立召唤一轮车；所有召唤相邻部署、入场禁动。</x:v>
       </x:c>
       <x:c r="F65" t="str">
-        <x:v>tests/test_battle.py与tests/test_behavior.py已扩充对应场景；本轮只做静态编译。</x:v>
+        <x:v>两个召唤技能按各自actor周围合法格生成且无场上同名上限；每个BicycleSummon拥有独立SummonUnicycleSkill；Battle.summon_unit令turn_ready=false。</x:v>
       </x:c>
       <x:c r="G65" t="str">
-        <x:v>已补充待验证</x:v>
+        <x:v>符合</x:v>
       </x:c>
       <x:c r="H65" t="str">
-        <x:v>P1</x:v>
+        <x:v>P3</x:v>
       </x:c>
       <x:c r="I65" t="str">
-        <x:v>由用户运行当前批次统一测试。</x:v>
+        <x:v>新增两条并存分支及各自子召唤测试。</x:v>
       </x:c>
       <x:c r="J65" t="str">
-        <x:v>首轮日志符合，待统一回归重跑</x:v>
+        <x:v>待用户当前批次测试</x:v>
       </x:c>
       <x:c r="K65" t="str">
-        <x:v>docs/武将设计思想.json#excel_r206</x:v>
+        <x:v>docs/武将设计思想.json#excel_r198</x:v>
       </x:c>
       <x:c r="L65" t="str">
-        <x:v>reports/current-hero-deep-audit/excel_r142--excel_r198--excel_r206：2026-09-02全新复测10场、8胜2负、自动高信号0/P3；擂台嘲讽7/37，组合格挡反击33/35，保护3次、普通格挡4次。人工逐步对照再次确认被嘲讽单位服从指定攻击，组合反击先结算、临时守链尾清除、实际伤害触发吸血，AI会按威胁切换保护/格挡。普通反击因组合通常严格占优而未采用，合法候选与定向测试均保留；当前三将专属测试无失败，未发现新缺陷。</x:v>
+        <x:v>reports/current-hero-deep-audit/excel_r142--excel_r198--excel_r206：2026-09-02全新复测10场、2胜8负、自动高信号0/P3；二轮车召唤10/13个有效机会，一轮车召唤1/1。人工逐步对照再次确认本体召唤→神速/移动→普攻→再次移动，以及二轮车召唤子车→移动→攻击；攻击后未再移动的代表场景随即结束战斗，不构成漏用。当前三将专属测试无失败，未发现实现或AI偏离设计。</x:v>
       </x:c>
       <x:c r="M65" t="str">
         <x:v>2026-09-06用户调整：连续分批完成全部已开发武将及AI的设计优先检查修改；保留测试用例和静态检查，中途不运行测试、不等待逐批签收，全部完成后统一测试。</x:v>
@@ -26333,22 +26585,22 @@
     </x:row>
     <x:row r="66">
       <x:c r="A66" t="str">
-        <x:v>excel_r291</x:v>
+        <x:v>excel_r198</x:v>
       </x:c>
       <x:c r="B66" t="str">
-        <x:v>机甲忍者。赤</x:v>
+        <x:v>三轮车人</x:v>
       </x:c>
       <x:c r="C66" t="str">
-        <x:v>2026-09-06复核新10场：45次声明逐条对应45条公开随机破魔日志，无遗漏或重复；专属测试未列入失败。本批随太阳神测试修正保持待复测。</x:v>
+        <x:v>已完整验收：设计、5项设计推断、战斗实现、AI、测试与两轮用户日志均已逐层审查；召唤顺序、攻击后移动经济与AI重规划符合设计，2026-09-02复测未发现新缺陷</x:v>
       </x:c>
       <x:c r="D66" t="str">
         <x:v>战斗实现</x:v>
       </x:c>
       <x:c r="E66" t="str">
-        <x:v>面板及回避、吸魔、铁锁路径必须映射源表；铁锁每回合首发免费、后续0.5魔且无次数上限，只伤敌方并固定破魔。</x:v>
+        <x:v>召唤消散必须按直接召唤者分支级联。</x:v>
       </x:c>
       <x:c r="F66" t="str">
-        <x:v>excel_r291专用工厂映射IronChainPathSkill与RedDrainManaSkill；通用回避保留。mana_cost_for_payload按uses_this_turn首发归零，后续回到0.5；max_uses_per_turn未设置；affected_units过滤友军，resolve_hit固定ignore_shield。</x:v>
+        <x:v>Battle.summon_unit记录直接summoner_id；cleanup_dead_units循环清理召唤者已死亡的单位，因此三轮车人→二轮车→一轮车逐层级联，单座二轮车死亡不影响另一分支。</x:v>
       </x:c>
       <x:c r="G66" t="str">
         <x:v>符合</x:v>
@@ -26357,16 +26609,16 @@
         <x:v>P3</x:v>
       </x:c>
       <x:c r="I66" t="str">
-        <x:v>保留数值与资源规则，补首发/后续费用、敌友过滤和固定破魔断言。</x:v>
+        <x:v>新增单分支清理、另一分支保留的测试。</x:v>
       </x:c>
       <x:c r="J66" t="str">
-        <x:v>已审查，待用户当前批次测试</x:v>
+        <x:v>待用户当前批次测试</x:v>
       </x:c>
       <x:c r="K66" t="str">
-        <x:v>docs/武将设计思想.json#excel_r291</x:v>
+        <x:v>docs/武将设计思想.json#excel_r198</x:v>
       </x:c>
       <x:c r="L66" t="str">
-        <x:v>9月4日新10场3胜7负、铁锁7次、吸魔3次、回避27次。逐场声明/公开随机日志数为2/2、6/6、7/7、2/2、2/2、6/6、2/2、6/6、10/10、2/2，共45/45；每次声明同一步均有对应结果。929项回归没有赤专属失败。</x:v>
+        <x:v>reports/current-hero-deep-audit/excel_r142--excel_r198--excel_r206：2026-09-02全新复测10场、2胜8负、自动高信号0/P3；二轮车召唤10/13个有效机会，一轮车召唤1/1。人工逐步对照再次确认本体召唤→神速/移动→普攻→再次移动，以及二轮车召唤子车→移动→攻击；攻击后未再移动的代表场景随即结束战斗，不构成漏用。当前三将专属测试无失败，未发现实现或AI偏离设计。</x:v>
       </x:c>
       <x:c r="M66" t="str">
         <x:v>2026-09-06用户调整：连续分批完成全部已开发武将及AI的设计优先检查修改；保留测试用例和静态检查，中途不运行测试、不等待逐批签收，全部完成后统一测试。</x:v>
@@ -26374,40 +26626,40 @@
     </x:row>
     <x:row r="67">
       <x:c r="A67" t="str">
-        <x:v>excel_r291</x:v>
+        <x:v>excel_r198</x:v>
       </x:c>
       <x:c r="B67" t="str">
-        <x:v>机甲忍者。赤</x:v>
+        <x:v>三轮车人</x:v>
       </x:c>
       <x:c r="C67" t="str">
-        <x:v>2026-09-06复核新10场：45次声明逐条对应45条公开随机破魔日志，无遗漏或重复；专属测试未列入失败。本批随太阳神测试修正保持待复测。</x:v>
+        <x:v>已完整验收：设计、5项设计推断、战斗实现、AI、测试与两轮用户日志均已逐层审查；召唤顺序、攻击后移动经济与AI重规划符合设计，2026-09-02复测未发现新缺陷</x:v>
       </x:c>
       <x:c r="D67" t="str">
-        <x:v>战斗实现</x:v>
+        <x:v>AI</x:v>
       </x:c>
       <x:c r="E67" t="str">
-        <x:v>铁锁必须把纯墙体、地形场和地形单位纳入最近锚点；地形只移动，不产生追击。</x:v>
+        <x:v>二轮车落点应同时考虑入场暴露、下回合攻击接触和未来一轮车合法空位。</x:v>
       </x:c>
       <x:c r="F67" t="str">
-        <x:v>旧anchor_for_cells只检查units_at，纯blocked_cells墙体和is_terrain场地无法成为锚。现按声明线近到远检查稳定单位、墙体和地形场；带地形语义的单位归类为terrain，不创建RedNextDamageStatus。</x:v>
+        <x:v>旧通用召唤评分只奖励接近敌人；现cycle_summon_score计算下一轮速5+范1接触、敌方可达威胁、过近惩罚，并让二轮车强烈保留邻接空格。</x:v>
       </x:c>
       <x:c r="G67" t="str">
-        <x:v>已修复待验证</x:v>
+        <x:v>已改进待验证</x:v>
       </x:c>
       <x:c r="H67" t="str">
-        <x:v>P1</x:v>
+        <x:v>P2</x:v>
       </x:c>
       <x:c r="I67" t="str">
-        <x:v>已加入墙体位于敌人之前时优先锁墙、只伤敌人并且无追击状态的定向测试。</x:v>
+        <x:v>已补受地形限制时仍选择保留子召唤空位的AI测试。</x:v>
       </x:c>
       <x:c r="J67" t="str">
         <x:v>待用户当前批次测试</x:v>
       </x:c>
       <x:c r="K67" t="str">
-        <x:v>docs/武将设计思想.json#excel_r291</x:v>
+        <x:v>docs/武将设计思想.json#excel_r198</x:v>
       </x:c>
       <x:c r="L67" t="str">
-        <x:v>9月4日新10场3胜7负、铁锁7次、吸魔3次、回避27次。逐场声明/公开随机日志数为2/2、6/6、7/7、2/2、2/2、6/6、2/2、6/6、10/10、2/2，共45/45；每次声明同一步均有对应结果。929项回归没有赤专属失败。</x:v>
+        <x:v>reports/current-hero-deep-audit/excel_r142--excel_r198--excel_r206：2026-09-02全新复测10场、2胜8负、自动高信号0/P3；二轮车召唤10/13个有效机会，一轮车召唤1/1。人工逐步对照再次确认本体召唤→神速/移动→普攻→再次移动，以及二轮车召唤子车→移动→攻击；攻击后未再移动的代表场景随即结束战斗，不构成漏用。当前三将专属测试无失败，未发现实现或AI偏离设计。</x:v>
       </x:c>
       <x:c r="M67" t="str">
         <x:v>2026-09-06用户调整：连续分批完成全部已开发武将及AI的设计优先检查修改；保留测试用例和静态检查，中途不运行测试、不等待逐批签收，全部完成后统一测试。</x:v>
@@ -26415,40 +26667,40 @@
     </x:row>
     <x:row r="68">
       <x:c r="A68" t="str">
-        <x:v>excel_r291</x:v>
+        <x:v>excel_r198</x:v>
       </x:c>
       <x:c r="B68" t="str">
-        <x:v>机甲忍者。赤</x:v>
+        <x:v>三轮车人</x:v>
       </x:c>
       <x:c r="C68" t="str">
-        <x:v>2026-09-06复核新10场：45次声明逐条对应45条公开随机破魔日志，无遗漏或重复；专属测试未列入失败。本批随太阳神测试修正保持待复测。</x:v>
+        <x:v>已完整验收：设计、5项设计推断、战斗实现、AI、测试与两轮用户日志均已逐层审查；召唤顺序、攻击后移动经济与AI重规划符合设计，2026-09-02复测未发现新缺陷</x:v>
       </x:c>
       <x:c r="D68" t="str">
-        <x:v>战斗实现</x:v>
+        <x:v>通用AI</x:v>
       </x:c>
       <x:c r="E68" t="str">
-        <x:v>锚点在伤害前锁定；位移只能在5格内沿一条直线到达锚点真正周围，失败不回滚伤害或单位追击。</x:v>
+        <x:v>车体攻击重置移动后必须重新生成动作候选，实现移动→攻击→再移动。</x:v>
       </x:c>
       <x:c r="F68" t="str">
-        <x:v>旧实现只有活着且仍有position的单位锚才能继续，并调用可跨全图且只求最近距离的通用拉近函数。现先保存锚点及占格，再结算伤害；destination_for_anchor仅枚举5格直线可达点并要求与锚占格距离恰为1；失败后仍建立单位追击。</x:v>
+        <x:v>choose_turn_action/choose_turn_bundle_action每次行动后重新读取action_snapshot；ResetMoveAfterAttackTrait在普攻完成时立即清零移动使用量。新增测试锁定攻击后再次生成move。</x:v>
       </x:c>
       <x:c r="G68" t="str">
-        <x:v>已修复待验证</x:v>
+        <x:v>符合并补测试</x:v>
       </x:c>
       <x:c r="H68" t="str">
-        <x:v>P1</x:v>
+        <x:v>P2</x:v>
       </x:c>
       <x:c r="I68" t="str">
-        <x:v>已补锚点被本发击破后仍保留追击，以及墙体阻路只到合法邻格的测试。</x:v>
+        <x:v>保留动态重规划架构，观察当前批次日志中的攻击后移动机会采用率。</x:v>
       </x:c>
       <x:c r="J68" t="str">
         <x:v>待用户当前批次测试</x:v>
       </x:c>
       <x:c r="K68" t="str">
-        <x:v>docs/武将设计思想.json#excel_r291</x:v>
+        <x:v>docs/武将设计思想.json#excel_r198</x:v>
       </x:c>
       <x:c r="L68" t="str">
-        <x:v>9月4日新10场3胜7负、铁锁7次、吸魔3次、回避27次。逐场声明/公开随机日志数为2/2、6/6、7/7、2/2、2/2、6/6、2/2、6/6、10/10、2/2，共45/45；每次声明同一步均有对应结果。929项回归没有赤专属失败。</x:v>
+        <x:v>reports/current-hero-deep-audit/excel_r142--excel_r198--excel_r206：2026-09-02全新复测10场、2胜8负、自动高信号0/P3；二轮车召唤10/13个有效机会，一轮车召唤1/1。人工逐步对照再次确认本体召唤→神速/移动→普攻→再次移动，以及二轮车召唤子车→移动→攻击；攻击后未再移动的代表场景随即结束战斗，不构成漏用。当前三将专属测试无失败，未发现实现或AI偏离设计。</x:v>
       </x:c>
       <x:c r="M68" t="str">
         <x:v>2026-09-06用户调整：连续分批完成全部已开发武将及AI的设计优先检查修改；保留测试用例和静态检查，中途不运行测试、不等待逐批签收，全部完成后统一测试。</x:v>
@@ -26456,40 +26708,40 @@
     </x:row>
     <x:row r="69">
       <x:c r="A69" t="str">
-        <x:v>excel_r291</x:v>
+        <x:v>excel_r198</x:v>
       </x:c>
       <x:c r="B69" t="str">
-        <x:v>机甲忍者。赤</x:v>
+        <x:v>三轮车人</x:v>
       </x:c>
       <x:c r="C69" t="str">
-        <x:v>2026-09-06复核新10场：45次声明逐条对应45条公开随机破魔日志，无遗漏或重复；专属测试未列入失败。本批随太阳神测试修正保持待复测。</x:v>
+        <x:v>已完整验收：设计、5项设计推断、战斗实现、AI、测试与两轮用户日志均已逐层审查；召唤顺序、攻击后移动经济与AI重规划符合设计，2026-09-02复测未发现新缺陷</x:v>
       </x:c>
       <x:c r="D69" t="str">
-        <x:v>战斗实现</x:v>
+        <x:v>测试</x:v>
       </x:c>
       <x:c r="E69" t="str">
-        <x:v>追击只强化赤对绑定单位的下一份直接伤害一次；本发铁锁、场地伤害、队友伤害和其他目标不能消费。</x:v>
+        <x:v>测试需覆盖独立召唤分支、入场禁动、移动增益/重置、级联和AI重规划。</x:v>
       </x:c>
       <x:c r="F69" t="str">
-        <x:v>RedNextDamageStatus在本发完成后添加；on_before_damage核对source与target并排除from_field_effect，修改该DamageContext后立即移除；duration=1且any_turn_end使其在当前回合末失效。</x:v>
+        <x:v>tests/test_battle.py与tests/test_behavior.py已扩充上述场景；本轮不运行动态测试。</x:v>
       </x:c>
       <x:c r="G69" t="str">
-        <x:v>符合</x:v>
+        <x:v>已补充待验证</x:v>
       </x:c>
       <x:c r="H69" t="str">
-        <x:v>P2</x:v>
+        <x:v>P1</x:v>
       </x:c>
       <x:c r="I69" t="str">
-        <x:v>保留实现，并由当前批次定向与审计日志核对一次性消费。</x:v>
+        <x:v>由用户运行当前批次统一测试。</x:v>
       </x:c>
       <x:c r="J69" t="str">
-        <x:v>已审查，待用户当前批次测试</x:v>
+        <x:v>首轮日志符合，待统一回归重跑</x:v>
       </x:c>
       <x:c r="K69" t="str">
-        <x:v>docs/武将设计思想.json#excel_r291</x:v>
+        <x:v>docs/武将设计思想.json#excel_r198</x:v>
       </x:c>
       <x:c r="L69" t="str">
-        <x:v>9月4日新10场3胜7负、铁锁7次、吸魔3次、回避27次。逐场声明/公开随机日志数为2/2、6/6、7/7、2/2、2/2、6/6、2/2、6/6、10/10、2/2，共45/45；每次声明同一步均有对应结果。929项回归没有赤专属失败。</x:v>
+        <x:v>reports/current-hero-deep-audit/excel_r142--excel_r198--excel_r206：2026-09-02全新复测10场、2胜8负、自动高信号0/P3；二轮车召唤10/13个有效机会，一轮车召唤1/1。人工逐步对照再次确认本体召唤→神速/移动→普攻→再次移动，以及二轮车召唤子车→移动→攻击；攻击后未再移动的代表场景随即结束战斗，不构成漏用。当前三将专属测试无失败，未发现实现或AI偏离设计。</x:v>
       </x:c>
       <x:c r="M69" t="str">
         <x:v>2026-09-06用户调整：连续分批完成全部已开发武将及AI的设计优先检查修改；保留测试用例和静态检查，中途不运行测试、不等待逐批签收，全部完成后统一测试。</x:v>
@@ -26497,22 +26749,22 @@
     </x:row>
     <x:row r="70">
       <x:c r="A70" t="str">
-        <x:v>excel_r291</x:v>
+        <x:v>excel_r206</x:v>
       </x:c>
       <x:c r="B70" t="str">
-        <x:v>机甲忍者。赤</x:v>
+        <x:v>反击拳手</x:v>
       </x:c>
       <x:c r="C70" t="str">
-        <x:v>2026-09-06复核新10场：45次声明逐条对应45条公开随机破魔日志，无遗漏或重复；专属测试未列入失败。本批随太阳神测试修正保持待复测。</x:v>
+        <x:v>已完整验收：设计、6项设计推断、战斗实现、通用AI、测试与两轮用户日志均已逐层审查；嘲讽服从、反应选择、临时防御与吸血符合设计，2026-09-02复测未发现新缺陷</x:v>
       </x:c>
       <x:c r="D70" t="str">
         <x:v>战斗实现</x:v>
       </x:c>
       <x:c r="E70" t="str">
-        <x:v>随机破魔必须每个声明恰采样一次、公开结果、同动作共享，且不能泄漏到后续动作。</x:v>
+        <x:v>擂台嘲讽必须对周围8格敌我双方造成当前攻3破魔伤害，再给存活命中单位施加指定攻击。</x:v>
       </x:c>
       <x:c r="F70" t="str">
-        <x:v>RedRandomPierceTrait在on_owner_action_declared单次采样并把结果写入动作payload；2026-09-03日志发现用普通battle.log写结果时，对隐身目标的动作会被隐身抑制。现改用带来源的公开事件接口，保证随机结果公开，同时仍只存在于本次payload。</x:v>
+        <x:v>旧RingTauntSkill明确实现为敌方、无伤害；现改为双方区域DamageContext、当前攻、ignore_shield，伤害成功且存活后才加状态。</x:v>
       </x:c>
       <x:c r="G70" t="str">
         <x:v>已修复待验证</x:v>
@@ -26521,16 +26773,16 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="I70" t="str">
-        <x:v>保留动作载荷传播；公开结果改走不可被隐身目标抑制的公开事件，并补隐身目标场景。</x:v>
+        <x:v>已补敌我伤害、破盾与控制顺序测试。</x:v>
       </x:c>
       <x:c r="J70" t="str">
-        <x:v>二次修复并补测试，待用户复跑当前批次</x:v>
+        <x:v>待用户当前批次测试</x:v>
       </x:c>
       <x:c r="K70" t="str">
-        <x:v>docs/武将设计思想.json#excel_r291</x:v>
+        <x:v>docs/武将设计思想.json#excel_r206</x:v>
       </x:c>
       <x:c r="L70" t="str">
-        <x:v>9月4日新10场3胜7负、铁锁7次、吸魔3次、回避27次。逐场声明/公开随机日志数为2/2、6/6、7/7、2/2、2/2、6/6、2/2、6/6、10/10、2/2，共45/45；每次声明同一步均有对应结果。929项回归没有赤专属失败。</x:v>
+        <x:v>reports/current-hero-deep-audit/excel_r142--excel_r198--excel_r206：2026-09-02全新复测10场、8胜2负、自动高信号0/P3；擂台嘲讽7/37，组合格挡反击33/35，保护3次、普通格挡4次。人工逐步对照再次确认被嘲讽单位服从指定攻击，组合反击先结算、临时守链尾清除、实际伤害触发吸血，AI会按威胁切换保护/格挡。普通反击因组合通常严格占优而未采用，合法候选与定向测试均保留；当前三将专属测试无失败，未发现新缺陷。</x:v>
       </x:c>
       <x:c r="M70" t="str">
         <x:v>2026-09-06用户调整：连续分批完成全部已开发武将及AI的设计优先检查修改；保留测试用例和静态检查，中途不运行测试、不等待逐批签收，全部完成后统一测试。</x:v>
@@ -26538,40 +26790,40 @@
     </x:row>
     <x:row r="71">
       <x:c r="A71" t="str">
-        <x:v>excel_r291</x:v>
+        <x:v>excel_r206</x:v>
       </x:c>
       <x:c r="B71" t="str">
-        <x:v>机甲忍者。赤</x:v>
+        <x:v>反击拳手</x:v>
       </x:c>
       <x:c r="C71" t="str">
-        <x:v>2026-09-06复核新10场：45次声明逐条对应45条公开随机破魔日志，无遗漏或重复；专属测试未列入失败。本批随太阳神测试修正保持待复测。</x:v>
+        <x:v>已完整验收：设计、6项设计推断、战斗实现、通用AI、测试与两轮用户日志均已逐层审查；嘲讽服从、反应选择、临时防御与吸血符合设计，2026-09-02复测未发现新缺陷</x:v>
       </x:c>
       <x:c r="D71" t="str">
-        <x:v>AI</x:v>
+        <x:v>战斗实现</x:v>
       </x:c>
       <x:c r="E71" t="str">
-        <x:v>铁锁评分必须接受强制最近锚点，计算实际落点风险和本回合追击兑现，不能只按线伤与免费奖励决策。</x:v>
+        <x:v>目标下回合有普攻资源时才激活指定攻击；声明消耗正常次数并解除，拳手离场/回合结束清除。</x:v>
       </x:c>
       <x:c r="F71" t="str">
-        <x:v>旧iron_chain_path_score只调用skill_damage_score、目标价值与首发+12。现复用战斗实现的anchor_for_cells/destination_for_anchor，加入真实落点移动价值、敌方可达伤害、多攻威胁、敌方单位追击收益、友军/地形锚机会成本；无敌方命中仍拒绝。</x:v>
+        <x:v>RequiredAttackStatus已实现声明解除、来源失效、owner_turn_end过期与最新覆盖；BoxerTauntStatus补充无可用攻击次数时不激活。</x:v>
       </x:c>
       <x:c r="G71" t="str">
         <x:v>已修复待验证</x:v>
       </x:c>
       <x:c r="H71" t="str">
-        <x:v>P1</x:v>
+        <x:v>P2</x:v>
       </x:c>
       <x:c r="I71" t="str">
-        <x:v>已补两条等伤线路中避开高攻敌人可达落点的AI行为测试。</x:v>
+        <x:v>补充无攻击数和友方强制目标测试。</x:v>
       </x:c>
       <x:c r="J71" t="str">
         <x:v>待用户当前批次测试</x:v>
       </x:c>
       <x:c r="K71" t="str">
-        <x:v>docs/武将设计思想.json#excel_r291</x:v>
+        <x:v>docs/武将设计思想.json#excel_r206</x:v>
       </x:c>
       <x:c r="L71" t="str">
-        <x:v>9月4日新10场3胜7负、铁锁7次、吸魔3次、回避27次。逐场声明/公开随机日志数为2/2、6/6、7/7、2/2、2/2、6/6、2/2、6/6、10/10、2/2，共45/45；每次声明同一步均有对应结果。929项回归没有赤专属失败。</x:v>
+        <x:v>reports/current-hero-deep-audit/excel_r142--excel_r198--excel_r206：2026-09-02全新复测10场、8胜2负、自动高信号0/P3；擂台嘲讽7/37，组合格挡反击33/35，保护3次、普通格挡4次。人工逐步对照再次确认被嘲讽单位服从指定攻击，组合反击先结算、临时守链尾清除、实际伤害触发吸血，AI会按威胁切换保护/格挡。普通反击因组合通常严格占优而未采用，合法候选与定向测试均保留；当前三将专属测试无失败，未发现新缺陷。</x:v>
       </x:c>
       <x:c r="M71" t="str">
         <x:v>2026-09-06用户调整：连续分批完成全部已开发武将及AI的设计优先检查修改；保留测试用例和静态检查，中途不运行测试、不等待逐批签收，全部完成后统一测试。</x:v>
@@ -26579,40 +26831,40 @@
     </x:row>
     <x:row r="72">
       <x:c r="A72" t="str">
-        <x:v>excel_r291</x:v>
+        <x:v>excel_r206</x:v>
       </x:c>
       <x:c r="B72" t="str">
-        <x:v>机甲忍者。赤</x:v>
+        <x:v>反击拳手</x:v>
       </x:c>
       <x:c r="C72" t="str">
-        <x:v>2026-09-06复核新10场：45次声明逐条对应45条公开随机破魔日志，无遗漏或重复；专属测试未列入失败。本批随太阳神测试修正保持待复测。</x:v>
+        <x:v>已完整验收：设计、6项设计推断、战斗实现、通用AI、测试与两轮用户日志均已逐层审查；嘲讽服从、反应选择、临时防御与吸血符合设计，2026-09-02复测未发现新缺陷</x:v>
       </x:c>
       <x:c r="D72" t="str">
-        <x:v>测试</x:v>
+        <x:v>通用战斗规则</x:v>
       </x:c>
       <x:c r="E72" t="str">
-        <x:v>测试矩阵必须覆盖锚点阵营/地形/顺序、严格位移、追击生命周期、费用与随机动作边界，并验证AI落位质量。</x:v>
+        <x:v>被擂台嘲讽命中的己方单位必须能合法普攻己方拳手。</x:v>
       </x:c>
       <x:c r="F72" t="str">
-        <x:v>已覆盖墙体锚、死亡锚点锁定、随机状态不残留、强制锚点落位风险、首发免费、单位追击和单动作单随机；本轮补隐身目标仍公开随机结果，并把致死样本血量改为真实可击破值、把墙体落点断言改为验证直线/5格/真实邻接而非唯一坐标。开发代理未运行动态测试。</x:v>
+        <x:v>Battle.forced_basic_attack_target及声明冻结许可同时服务猫叔与反击拳手；AI候选也允许只为完成契约而攻击指定己方目标。</x:v>
       </x:c>
       <x:c r="G72" t="str">
-        <x:v>已补充待验证</x:v>
+        <x:v>已修复待验证</x:v>
       </x:c>
       <x:c r="H72" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="I72" t="str">
-        <x:v>由用户运行python detail_test_all_wujiangs.py --current。</x:v>
+        <x:v>复用通用指定攻击测试。</x:v>
       </x:c>
       <x:c r="J72" t="str">
-        <x:v>测试夹具与公开日志场景已修，待用户复跑当前批次</x:v>
+        <x:v>待用户当前批次测试</x:v>
       </x:c>
       <x:c r="K72" t="str">
-        <x:v>docs/武将设计思想.json#excel_r291</x:v>
+        <x:v>docs/武将设计思想.json#excel_r206</x:v>
       </x:c>
       <x:c r="L72" t="str">
-        <x:v>9月4日新10场3胜7负、铁锁7次、吸魔3次、回避27次。逐场声明/公开随机日志数为2/2、6/6、7/7、2/2、2/2、6/6、2/2、6/6、10/10、2/2，共45/45；每次声明同一步均有对应结果。929项回归没有赤专属失败。</x:v>
+        <x:v>reports/current-hero-deep-audit/excel_r142--excel_r198--excel_r206：2026-09-02全新复测10场、8胜2负、自动高信号0/P3；擂台嘲讽7/37，组合格挡反击33/35，保护3次、普通格挡4次。人工逐步对照再次确认被嘲讽单位服从指定攻击，组合反击先结算、临时守链尾清除、实际伤害触发吸血，AI会按威胁切换保护/格挡。普通反击因组合通常严格占优而未采用，合法候选与定向测试均保留；当前三将专属测试无失败，未发现新缺陷。</x:v>
       </x:c>
       <x:c r="M72" t="str">
         <x:v>2026-09-06用户调整：连续分批完成全部已开发武将及AI的设计优先检查修改；保留测试用例和静态检查，中途不运行测试、不等待逐批签收，全部完成后统一测试。</x:v>
@@ -26620,22 +26872,22 @@
     </x:row>
     <x:row r="73">
       <x:c r="A73" t="str">
-        <x:v>excel_r356</x:v>
+        <x:v>excel_r206</x:v>
       </x:c>
       <x:c r="B73" t="str">
-        <x:v>强袭犀牛</x:v>
+        <x:v>反击拳手</x:v>
       </x:c>
       <x:c r="C73" t="str">
-        <x:v>2026-09-06复核新10场：24拳包含7个完整三拳回合，4次到期无锚等待日志可见。龙息与实际回归仍为随机局覆盖缺口，专属定向测试未列入失败；本批随太阳神测试修正保持待复测。</x:v>
+        <x:v>已完整验收：设计、6项设计推断、战斗实现、通用AI、测试与两轮用户日志均已逐层审查；嘲讽服从、反应选择、临时防御与吸血符合设计，2026-09-02复测未发现新缺陷</x:v>
       </x:c>
       <x:c r="D73" t="str">
         <x:v>战斗实现</x:v>
       </x:c>
       <x:c r="E73" t="str">
-        <x:v>面板与神速、龙息、震开、变硬、每回合三次普攻必须完整映射源表。</x:v>
+        <x:v>普通格挡、普通反击和组合格挡反击必须同时保留；组合只对敌方速度1、来源在范围的动作开放。</x:v>
       </x:c>
       <x:c r="F73" t="str">
-        <x:v>excel_r356使用通用ShensuSkill、DragonBreathSkill、KnockbackSkill、HardenSkill，并由AttackCountTrait把每回合普攻数改为3。</x:v>
+        <x:v>BlockCounterTrait提供普通两个候选；BoxerBlockCounterSkill为额外被动技能，can_react_to检查敌方、速度与attack_target_allowed范围。</x:v>
       </x:c>
       <x:c r="G73" t="str">
         <x:v>符合</x:v>
@@ -26644,16 +26896,16 @@
         <x:v>P3</x:v>
       </x:c>
       <x:c r="I73" t="str">
-        <x:v>不改通用技能数值，补AI连续三拳行为断言。</x:v>
+        <x:v>保留实现，补远程来源不生成组合测试。</x:v>
       </x:c>
       <x:c r="J73" t="str">
-        <x:v>已审查，待用户当前批次测试</x:v>
+        <x:v>待用户当前批次测试</x:v>
       </x:c>
       <x:c r="K73" t="str">
-        <x:v>docs/武将设计思想.json#excel_r356</x:v>
+        <x:v>docs/武将设计思想.json#excel_r206</x:v>
       </x:c>
       <x:c r="L73" t="str">
-        <x:v>9月4日新10场5胜5负、神速8次、普攻24次、变硬6次、震开3次。第2/3/5/6/7/9/10场各有一次完整三拳，另第3场后续2拳、第4场1拳。第7场步骤67/72/74/76均记录到期等待回归。龙息8个可用节点无有效候选；随机局未满足全部回归条件，保留条件覆盖缺口。929项回归无犀牛专属失败。</x:v>
+        <x:v>reports/current-hero-deep-audit/excel_r142--excel_r198--excel_r206：2026-09-02全新复测10场、8胜2负、自动高信号0/P3；擂台嘲讽7/37，组合格挡反击33/35，保护3次、普通格挡4次。人工逐步对照再次确认被嘲讽单位服从指定攻击，组合反击先结算、临时守链尾清除、实际伤害触发吸血，AI会按威胁切换保护/格挡。普通反击因组合通常严格占优而未采用，合法候选与定向测试均保留；当前三将专属测试无失败，未发现新缺陷。</x:v>
       </x:c>
       <x:c r="M73" t="str">
         <x:v>2026-09-06用户调整：连续分批完成全部已开发武将及AI的设计优先检查修改；保留测试用例和静态检查，中途不运行测试、不等待逐批签收，全部完成后统一测试。</x:v>
@@ -26661,40 +26913,40 @@
     </x:row>
     <x:row r="74">
       <x:c r="A74" t="str">
-        <x:v>excel_r356</x:v>
+        <x:v>excel_r206</x:v>
       </x:c>
       <x:c r="B74" t="str">
-        <x:v>强袭犀牛</x:v>
+        <x:v>反击拳手</x:v>
       </x:c>
       <x:c r="C74" t="str">
-        <x:v>2026-09-06复核新10场：24拳包含7个完整三拳回合，4次到期无锚等待日志可见。龙息与实际回归仍为随机局覆盖缺口，专属定向测试未列入失败；本批随太阳神测试修正保持待复测。</x:v>
+        <x:v>已完整验收：设计、6项设计推断、战斗实现、通用AI、测试与两轮用户日志均已逐层审查；嘲讽服从、反应选择、临时防御与吸血符合设计，2026-09-02复测未发现新缺陷</x:v>
       </x:c>
       <x:c r="D74" t="str">
         <x:v>战斗实现</x:v>
       </x:c>
       <x:c r="E74" t="str">
-        <x:v>每次真实破坏都应触发一次遗志和一个回归计时；同一条生命不得重复触发，但回归后的下一条生命必须重新具备资格。</x:v>
+        <x:v>组合反应先临时守+1、再进行普攻式反击，链尾清除；反击伤害触发吸血。</x:v>
       </x:c>
       <x:c r="F74" t="str">
-        <x:v>RhinoDeathTrait以triggered防止伤害钩子与移除钩子重复。审查发现旧triggered只在初次入场重置，回归后第二次死亡会永久失效；现回归前明确重置，add_unit入场钩子再次确认新生命状态。</x:v>
+        <x:v>react先加expire_with_chain TemporaryDefenseStatus，再resolve_attack_damage；该上下文is_skill=false且带attack标签，AttackLifeStealTrait会在实际伤害后回复，finalize_reaction_window清除临时守。</x:v>
       </x:c>
       <x:c r="G74" t="str">
-        <x:v>已修复待验证</x:v>
+        <x:v>符合</x:v>
       </x:c>
       <x:c r="H74" t="str">
-        <x:v>P1</x:v>
+        <x:v>P3</x:v>
       </x:c>
       <x:c r="I74" t="str">
-        <x:v>已补同一犀牛回归后第二次破坏再次产生单个回归记录、刷新而不叠遗志的测试。</x:v>
+        <x:v>补足吸血、链尾清理和穿刺不吸血断言。</x:v>
       </x:c>
       <x:c r="J74" t="str">
         <x:v>待用户当前批次测试</x:v>
       </x:c>
       <x:c r="K74" t="str">
-        <x:v>docs/武将设计思想.json#excel_r356</x:v>
+        <x:v>docs/武将设计思想.json#excel_r206</x:v>
       </x:c>
       <x:c r="L74" t="str">
-        <x:v>9月4日新10场5胜5负、神速8次、普攻24次、变硬6次、震开3次。第2/3/5/6/7/9/10场各有一次完整三拳，另第3场后续2拳、第4场1拳。第7场步骤67/72/74/76均记录到期等待回归。龙息8个可用节点无有效候选；随机局未满足全部回归条件，保留条件覆盖缺口。929项回归无犀牛专属失败。</x:v>
+        <x:v>reports/current-hero-deep-audit/excel_r142--excel_r198--excel_r206：2026-09-02全新复测10场、8胜2负、自动高信号0/P3；擂台嘲讽7/37，组合格挡反击33/35，保护3次、普通格挡4次。人工逐步对照再次确认被嘲讽单位服从指定攻击，组合反击先结算、临时守链尾清除、实际伤害触发吸血，AI会按威胁切换保护/格挡。普通反击因组合通常严格占优而未采用，合法候选与定向测试均保留；当前三将专属测试无失败，未发现新缺陷。</x:v>
       </x:c>
       <x:c r="M74" t="str">
         <x:v>2026-09-06用户调整：连续分批完成全部已开发武将及AI的设计优先检查修改；保留测试用例和静态检查，中途不运行测试、不等待逐批签收，全部完成后统一测试。</x:v>
@@ -26702,40 +26954,40 @@
     </x:row>
     <x:row r="75">
       <x:c r="A75" t="str">
-        <x:v>excel_r356</x:v>
+        <x:v>excel_r206</x:v>
       </x:c>
       <x:c r="B75" t="str">
-        <x:v>强袭犀牛</x:v>
+        <x:v>反击拳手</x:v>
       </x:c>
       <x:c r="C75" t="str">
-        <x:v>2026-09-06复核新10场：24拳包含7个完整三拳回合，4次到期无锚等待日志可见。龙息与实际回归仍为随机局覆盖缺口，专属定向测试未列入失败；本批随太阳神测试修正保持待复测。</x:v>
+        <x:v>已完整验收：设计、6项设计推断、战斗实现、通用AI、测试与两轮用户日志均已逐层审查；嘲讽服从、反应选择、临时防御与吸血符合设计，2026-09-02复测未发现新缺陷</x:v>
       </x:c>
       <x:c r="D75" t="str">
-        <x:v>战斗实现</x:v>
+        <x:v>AI</x:v>
       </x:c>
       <x:c r="E75" t="str">
-        <x:v>遗志只给破坏瞬间仍在场的其他友军，持续各自3回合；同名效果不叠加只刷新。</x:v>
+        <x:v>嘲讽评分必须同时计算攻3伤害、友伤、控制价值、预计承伤、可反击与吸血收益。</x:v>
       </x:c>
       <x:c r="F75" t="str">
-        <x:v>trigger_legacy快照player_units、排除owner和离场单位，包含正常召唤/分身；已有同名状态先移除再添加RhinoLegacyStatus(duration=3, owner_turn_end)。</x:v>
+        <x:v>旧taunt_control_score只数敌方控制；现按真实技能伤害探针、敌我阵营、未来攻击资源、预计敌方伤害和拳手反击伤害综合评分。</x:v>
       </x:c>
       <x:c r="G75" t="str">
-        <x:v>符合</x:v>
+        <x:v>已修复待验证</x:v>
       </x:c>
       <x:c r="H75" t="str">
-        <x:v>P2</x:v>
+        <x:v>P1</x:v>
       </x:c>
       <x:c r="I75" t="str">
-        <x:v>保留实现，当前批次检查接收者数量、层数与刷新时长。</x:v>
+        <x:v>已补两名队友邻接时拒绝擂台嘲讽的AI测试。</x:v>
       </x:c>
       <x:c r="J75" t="str">
-        <x:v>已审查，待用户当前批次测试</x:v>
+        <x:v>待用户当前批次测试</x:v>
       </x:c>
       <x:c r="K75" t="str">
-        <x:v>docs/武将设计思想.json#excel_r356</x:v>
+        <x:v>docs/武将设计思想.json#excel_r206</x:v>
       </x:c>
       <x:c r="L75" t="str">
-        <x:v>9月4日新10场5胜5负、神速8次、普攻24次、变硬6次、震开3次。第2/3/5/6/7/9/10场各有一次完整三拳，另第3场后续2拳、第4场1拳。第7场步骤67/72/74/76均记录到期等待回归。龙息8个可用节点无有效候选；随机局未满足全部回归条件，保留条件覆盖缺口。929项回归无犀牛专属失败。</x:v>
+        <x:v>reports/current-hero-deep-audit/excel_r142--excel_r198--excel_r206：2026-09-02全新复测10场、8胜2负、自动高信号0/P3；擂台嘲讽7/37，组合格挡反击33/35，保护3次、普通格挡4次。人工逐步对照再次确认被嘲讽单位服从指定攻击，组合反击先结算、临时守链尾清除、实际伤害触发吸血，AI会按威胁切换保护/格挡。普通反击因组合通常严格占优而未采用，合法候选与定向测试均保留；当前三将专属测试无失败，未发现新缺陷。</x:v>
       </x:c>
       <x:c r="M75" t="str">
         <x:v>2026-09-06用户调整：连续分批完成全部已开发武将及AI的设计优先检查修改；保留测试用例和静态检查，中途不运行测试、不等待逐批签收，全部完成后统一测试。</x:v>
@@ -26743,40 +26995,40 @@
     </x:row>
     <x:row r="76">
       <x:c r="A76" t="str">
-        <x:v>excel_r356</x:v>
+        <x:v>excel_r206</x:v>
       </x:c>
       <x:c r="B76" t="str">
-        <x:v>强袭犀牛</x:v>
+        <x:v>反击拳手</x:v>
       </x:c>
       <x:c r="C76" t="str">
-        <x:v>2026-09-06复核新10场：24拳包含7个完整三拳回合，4次到期无锚等待日志可见。龙息与实际回归仍为随机局覆盖缺口，专属定向测试未列入失败；本批随太阳神测试修正保持待复测。</x:v>
+        <x:v>已完整验收：设计、6项设计推断、战斗实现、通用AI、测试与两轮用户日志均已逐层审查；嘲讽服从、反应选择、临时防御与吸血符合设计，2026-09-02复测未发现新缺陷</x:v>
       </x:c>
       <x:c r="D76" t="str">
-        <x:v>战斗实现</x:v>
+        <x:v>通用AI</x:v>
       </x:c>
       <x:c r="E76" t="str">
-        <x:v>回归要等待死亡后3个完整全局行动环；到期无兽人本体或无合法格必须保留记录并在以后每个武将回合重试。</x:v>
+        <x:v>格挡类AI要按守+1实际减少的伤害评分，不能把破魔误当成无视防御；组合还要计算反击击杀与吸血。</x:v>
       </x:c>
       <x:c r="F76" t="str">
-        <x:v>return_turn_number=death_turn_number+固定turn_order槽数×3；turn_number会为死亡槽也推进。on_turn_start未到期或无候选时保留field effect；兽人候选排除召唤和分身。为让设计规定的持续重试可观察，现于到期但没有合法兽人/落点时记录明确等待日志。</x:v>
+        <x:v>旧block分支遇ignore_shield直接否决，混淆破魔与守+1；现temporary_defense_prevention_score在回滚探针内比较守+1前后威胁，组合评分再加入反击、击杀与缺血吸血价值。</x:v>
       </x:c>
       <x:c r="G76" t="str">
-        <x:v>符合并补测试</x:v>
+        <x:v>已修复待验证</x:v>
       </x:c>
       <x:c r="H76" t="str">
-        <x:v>P2</x:v>
+        <x:v>P1</x:v>
       </x:c>
       <x:c r="I76" t="str">
-        <x:v>保留重试机制；补所有兽人邻格阻塞时保留记录、腾格后自动回归，并断言到期等待日志。</x:v>
+        <x:v>保留普通格挡/反击作为合法替代，当前批次观察组合采用质量。</x:v>
       </x:c>
       <x:c r="J76" t="str">
-        <x:v>等待日志与断言已补，待用户复跑当前批次</x:v>
+        <x:v>待用户当前批次测试</x:v>
       </x:c>
       <x:c r="K76" t="str">
-        <x:v>docs/武将设计思想.json#excel_r356</x:v>
+        <x:v>docs/武将设计思想.json#excel_r206</x:v>
       </x:c>
       <x:c r="L76" t="str">
-        <x:v>9月4日新10场5胜5负、神速8次、普攻24次、变硬6次、震开3次。第2/3/5/6/7/9/10场各有一次完整三拳，另第3场后续2拳、第4场1拳。第7场步骤67/72/74/76均记录到期等待回归。龙息8个可用节点无有效候选；随机局未满足全部回归条件，保留条件覆盖缺口。929项回归无犀牛专属失败。</x:v>
+        <x:v>reports/current-hero-deep-audit/excel_r142--excel_r198--excel_r206：2026-09-02全新复测10场、8胜2负、自动高信号0/P3；擂台嘲讽7/37，组合格挡反击33/35，保护3次、普通格挡4次。人工逐步对照再次确认被嘲讽单位服从指定攻击，组合反击先结算、临时守链尾清除、实际伤害触发吸血，AI会按威胁切换保护/格挡。普通反击因组合通常严格占优而未采用，合法候选与定向测试均保留；当前三将专属测试无失败，未发现新缺陷。</x:v>
       </x:c>
       <x:c r="M76" t="str">
         <x:v>2026-09-06用户调整：连续分批完成全部已开发武将及AI的设计优先检查修改；保留测试用例和静态检查，中途不运行测试、不等待逐批签收，全部完成后统一测试。</x:v>
@@ -26784,40 +27036,40 @@
     </x:row>
     <x:row r="77">
       <x:c r="A77" t="str">
-        <x:v>excel_r356</x:v>
+        <x:v>excel_r206</x:v>
       </x:c>
       <x:c r="B77" t="str">
-        <x:v>强袭犀牛</x:v>
+        <x:v>反击拳手</x:v>
       </x:c>
       <x:c r="C77" t="str">
-        <x:v>2026-09-06复核新10场：24拳包含7个完整三拳回合，4次到期无锚等待日志可见。龙息与实际回归仍为随机局覆盖缺口，专属定向测试未列入失败；本批随太阳神测试修正保持待复测。</x:v>
+        <x:v>已完整验收：设计、6项设计推断、战斗实现、通用AI、测试与两轮用户日志均已逐层审查；嘲讽服从、反应选择、临时防御与吸血符合设计，2026-09-02复测未发现新缺陷</x:v>
       </x:c>
       <x:c r="D77" t="str">
-        <x:v>战斗实现</x:v>
+        <x:v>测试</x:v>
       </x:c>
       <x:c r="E77" t="str">
-        <x:v>多个兽人锚必须按固定行动槽选择第一个有合法格者，落点使用稳定格序。</x:v>
+        <x:v>测试需覆盖双方嘲讽、普攻资源门槛、三个反应候选、临时守、反击吸血与AI选择。</x:v>
       </x:c>
       <x:c r="F77" t="str">
-        <x:v>旧实现按等级降序、unit_id选锚，会让高等级后槽越过前槽。现按turn_order_unit_ids索引再按unit_id排序，周围格继续按y/x稳定顺序。</x:v>
+        <x:v>tests/test_battle.py与tests/test_behavior.py已扩充对应场景；本轮只做静态编译。</x:v>
       </x:c>
       <x:c r="G77" t="str">
-        <x:v>已修复待验证</x:v>
+        <x:v>已补充待验证</x:v>
       </x:c>
       <x:c r="H77" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="I77" t="str">
-        <x:v>已补前槽4级兽人优先于后槽5级兽人的阻塞重试测试。</x:v>
+        <x:v>由用户运行当前批次统一测试。</x:v>
       </x:c>
       <x:c r="J77" t="str">
-        <x:v>待用户当前批次测试</x:v>
+        <x:v>首轮日志符合，待统一回归重跑</x:v>
       </x:c>
       <x:c r="K77" t="str">
-        <x:v>docs/武将设计思想.json#excel_r356</x:v>
+        <x:v>docs/武将设计思想.json#excel_r206</x:v>
       </x:c>
       <x:c r="L77" t="str">
-        <x:v>9月4日新10场5胜5负、神速8次、普攻24次、变硬6次、震开3次。第2/3/5/6/7/9/10场各有一次完整三拳，另第3场后续2拳、第4场1拳。第7场步骤67/72/74/76均记录到期等待回归。龙息8个可用节点无有效候选；随机局未满足全部回归条件，保留条件覆盖缺口。929项回归无犀牛专属失败。</x:v>
+        <x:v>reports/current-hero-deep-audit/excel_r142--excel_r198--excel_r206：2026-09-02全新复测10场、8胜2负、自动高信号0/P3；擂台嘲讽7/37，组合格挡反击33/35，保护3次、普通格挡4次。人工逐步对照再次确认被嘲讽单位服从指定攻击，组合反击先结算、临时守链尾清除、实际伤害触发吸血，AI会按威胁切换保护/格挡。普通反击因组合通常严格占优而未采用，合法候选与定向测试均保留；当前三将专属测试无失败，未发现新缺陷。</x:v>
       </x:c>
       <x:c r="M77" t="str">
         <x:v>2026-09-06用户调整：连续分批完成全部已开发武将及AI的设计优先检查修改；保留测试用例和静态检查，中途不运行测试、不等待逐批签收，全部完成后统一测试。</x:v>
@@ -26825,40 +27077,40 @@
     </x:row>
     <x:row r="78">
       <x:c r="A78" t="str">
-        <x:v>excel_r356</x:v>
+        <x:v>excel_r291</x:v>
       </x:c>
       <x:c r="B78" t="str">
-        <x:v>强袭犀牛</x:v>
+        <x:v>机甲忍者。赤</x:v>
       </x:c>
       <x:c r="C78" t="str">
-        <x:v>2026-09-06复核新10场：24拳包含7个完整三拳回合，4次到期无锚等待日志可见。龙息与实际回归仍为随机局覆盖缺口，专属定向测试未列入失败；本批随太阳神测试修正保持待复测。</x:v>
+        <x:v>2026-09-06复核新10场：45次声明逐条对应45条公开随机破魔日志，无遗漏或重复；专属测试未列入失败。本批随太阳神测试修正保持待复测。</x:v>
       </x:c>
       <x:c r="D78" t="str">
         <x:v>战斗实现</x:v>
       </x:c>
       <x:c r="E78" t="str">
-        <x:v>回归应满血满魔、清上一生命临时状态，保留永久数值变化、身份、固定行动槽、冷却和本场使用记录，并且不赠送即时行动。</x:v>
+        <x:v>面板及回避、吸魔、铁锁路径必须映射源表；铁锁每回合首发免费、后续0.5魔且无次数上限，只伤敌方并固定破魔。</x:v>
       </x:c>
       <x:c r="F78" t="str">
-        <x:v>旧实现无条件移除全部status，误删duration=None的永久StatModifierStatus。现只保留无期限数值状态，清除其他临时状态；沿用原对象与skill对象，恢复血魔并把turn_ready及当前回合动作字段清零，固定turn_order不改。</x:v>
+        <x:v>excel_r291专用工厂映射IronChainPathSkill与RedDrainManaSkill；通用回避保留。mana_cost_for_payload按uses_this_turn首发归零，后续回到0.5；max_uses_per_turn未设置；affected_units过滤友军，resolve_hit固定ignore_shield。</x:v>
       </x:c>
       <x:c r="G78" t="str">
-        <x:v>已修复待验证</x:v>
+        <x:v>符合</x:v>
       </x:c>
       <x:c r="H78" t="str">
-        <x:v>P1</x:v>
+        <x:v>P3</x:v>
       </x:c>
       <x:c r="I78" t="str">
-        <x:v>已补永久/临时状态分离、技能记录/冷却、固定槽及无即时行动断言。</x:v>
+        <x:v>保留数值与资源规则，补首发/后续费用、敌友过滤和固定破魔断言。</x:v>
       </x:c>
       <x:c r="J78" t="str">
-        <x:v>待用户当前批次测试</x:v>
+        <x:v>已审查，待用户当前批次测试</x:v>
       </x:c>
       <x:c r="K78" t="str">
-        <x:v>docs/武将设计思想.json#excel_r356</x:v>
+        <x:v>docs/武将设计思想.json#excel_r291</x:v>
       </x:c>
       <x:c r="L78" t="str">
-        <x:v>9月4日新10场5胜5负、神速8次、普攻24次、变硬6次、震开3次。第2/3/5/6/7/9/10场各有一次完整三拳，另第3场后续2拳、第4场1拳。第7场步骤67/72/74/76均记录到期等待回归。龙息8个可用节点无有效候选；随机局未满足全部回归条件，保留条件覆盖缺口。929项回归无犀牛专属失败。</x:v>
+        <x:v>9月4日新10场3胜7负、铁锁7次、吸魔3次、回避27次。逐场声明/公开随机日志数为2/2、6/6、7/7、2/2、2/2、6/6、2/2、6/6、10/10、2/2，共45/45；每次声明同一步均有对应结果。929项回归没有赤专属失败。</x:v>
       </x:c>
       <x:c r="M78" t="str">
         <x:v>2026-09-06用户调整：连续分批完成全部已开发武将及AI的设计优先检查修改；保留测试用例和静态检查，中途不运行测试、不等待逐批签收，全部完成后统一测试。</x:v>
@@ -26866,40 +27118,40 @@
     </x:row>
     <x:row r="79">
       <x:c r="A79" t="str">
-        <x:v>excel_r356</x:v>
+        <x:v>excel_r291</x:v>
       </x:c>
       <x:c r="B79" t="str">
-        <x:v>强袭犀牛</x:v>
+        <x:v>机甲忍者。赤</x:v>
       </x:c>
       <x:c r="C79" t="str">
-        <x:v>2026-09-06复核新10场：24拳包含7个完整三拳回合，4次到期无锚等待日志可见。龙息与实际回归仍为随机局覆盖缺口，专属定向测试未列入失败；本批随太阳神测试修正保持待复测。</x:v>
+        <x:v>2026-09-06复核新10场：45次声明逐条对应45条公开随机破魔日志，无遗漏或重复；专属测试未列入失败。本批随太阳神测试修正保持待复测。</x:v>
       </x:c>
       <x:c r="D79" t="str">
-        <x:v>通用AI</x:v>
+        <x:v>战斗实现</x:v>
       </x:c>
       <x:c r="E79" t="str">
-        <x:v>三次普攻必须作为三次依次声明的动作，每拳后重新生成候选，不能打一拳便结束。</x:v>
+        <x:v>铁锁必须把纯墙体、地形场和地形单位纳入最近锚点；地形只移动，不产生追击。</x:v>
       </x:c>
       <x:c r="F79" t="str">
-        <x:v>choose_turn_action和choose_turn_bundle_action每次调用重新读取action_snapshot；Battle每拳只递增一次attacks_used，达到attack_actions_per_turn前继续提供普攻候选。旧集中审计中犀牛已有稳定多拳信号，未发现需改通用评分的证据。</x:v>
+        <x:v>旧anchor_for_cells只检查units_at，纯blocked_cells墙体和is_terrain场地无法成为锚。现按声明线近到远检查稳定单位、墙体和地形场；带地形语义的单位归类为terrain，不创建RedNextDamageStatus。</x:v>
       </x:c>
       <x:c r="G79" t="str">
-        <x:v>符合并补测试</x:v>
+        <x:v>已修复待验证</x:v>
       </x:c>
       <x:c r="H79" t="str">
-        <x:v>P2</x:v>
+        <x:v>P1</x:v>
       </x:c>
       <x:c r="I79" t="str">
-        <x:v>保留通用重规划架构，新增0魔且持续有目标时连续选择并执行三次普攻的行为测试。</x:v>
+        <x:v>已加入墙体位于敌人之前时优先锁墙、只伤敌人并且无追击状态的定向测试。</x:v>
       </x:c>
       <x:c r="J79" t="str">
         <x:v>待用户当前批次测试</x:v>
       </x:c>
       <x:c r="K79" t="str">
-        <x:v>docs/武将设计思想.json#excel_r356</x:v>
+        <x:v>docs/武将设计思想.json#excel_r291</x:v>
       </x:c>
       <x:c r="L79" t="str">
-        <x:v>9月4日新10场5胜5负、神速8次、普攻24次、变硬6次、震开3次。第2/3/5/6/7/9/10场各有一次完整三拳，另第3场后续2拳、第4场1拳。第7场步骤67/72/74/76均记录到期等待回归。龙息8个可用节点无有效候选；随机局未满足全部回归条件，保留条件覆盖缺口。929项回归无犀牛专属失败。</x:v>
+        <x:v>9月4日新10场3胜7负、铁锁7次、吸魔3次、回避27次。逐场声明/公开随机日志数为2/2、6/6、7/7、2/2、2/2、6/6、2/2、6/6、10/10、2/2，共45/45；每次声明同一步均有对应结果。929项回归没有赤专属失败。</x:v>
       </x:c>
       <x:c r="M79" t="str">
         <x:v>2026-09-06用户调整：连续分批完成全部已开发武将及AI的设计优先检查修改；保留测试用例和静态检查，中途不运行测试、不等待逐批签收，全部完成后统一测试。</x:v>
@@ -26907,49 +27159,541 @@
     </x:row>
     <x:row r="80">
       <x:c r="A80" t="str">
-        <x:v>excel_r356</x:v>
+        <x:v>excel_r291</x:v>
       </x:c>
       <x:c r="B80" t="str">
-        <x:v>强袭犀牛</x:v>
+        <x:v>机甲忍者。赤</x:v>
       </x:c>
       <x:c r="C80" t="str">
-        <x:v>2026-09-06复核新10场：24拳包含7个完整三拳回合，4次到期无锚等待日志可见。龙息与实际回归仍为随机局覆盖缺口，专属定向测试未列入失败；本批随太阳神测试修正保持待复测。</x:v>
+        <x:v>2026-09-06复核新10场：45次声明逐条对应45条公开随机破魔日志，无遗漏或重复；专属测试未列入失败。本批随太阳神测试修正保持待复测。</x:v>
       </x:c>
       <x:c r="D80" t="str">
-        <x:v>测试</x:v>
+        <x:v>战斗实现</x:v>
       </x:c>
       <x:c r="E80" t="str">
-        <x:v>测试矩阵必须覆盖两次死亡、遗志刷新、完整行动环、无兽人/无格重试、固定槽选锚、回归保留边界和三拳AI。</x:v>
+        <x:v>锚点在伤害前锁定；位移只能在5格内沿一条直线到达锚点真正周围，失败不回滚伤害或单位追击。</x:v>
       </x:c>
       <x:c r="F80" t="str">
-        <x:v>已在伤害/非伤害破坏和三环计时基础上覆盖第二次死亡、状态与场次记录、固定槽、阻塞重试及逐拳重规划；本轮再断言到期无合法锚/落点时输出等待日志。审计工具同时区分‘技能可用但无有效候选’与真实错失，并隔离其他武将同名日志。开发代理未运行动态测试。</x:v>
+        <x:v>旧实现只有活着且仍有position的单位锚才能继续，并调用可跨全图且只求最近距离的通用拉近函数。现先保存锚点及占格，再结算伤害；destination_for_anchor仅枚举5格直线可达点并要求与锚占格距离恰为1；失败后仍建立单位追击。</x:v>
       </x:c>
       <x:c r="G80" t="str">
-        <x:v>已补充待验证</x:v>
+        <x:v>已修复待验证</x:v>
       </x:c>
       <x:c r="H80" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="I80" t="str">
+        <x:v>已补锚点被本发击破后仍保留追击，以及墙体阻路只到合法邻格的测试。</x:v>
+      </x:c>
+      <x:c r="J80" t="str">
+        <x:v>待用户当前批次测试</x:v>
+      </x:c>
+      <x:c r="K80" t="str">
+        <x:v>docs/武将设计思想.json#excel_r291</x:v>
+      </x:c>
+      <x:c r="L80" t="str">
+        <x:v>9月4日新10场3胜7负、铁锁7次、吸魔3次、回避27次。逐场声明/公开随机日志数为2/2、6/6、7/7、2/2、2/2、6/6、2/2、6/6、10/10、2/2，共45/45；每次声明同一步均有对应结果。929项回归没有赤专属失败。</x:v>
+      </x:c>
+      <x:c r="M80" t="str">
+        <x:v>2026-09-06用户调整：连续分批完成全部已开发武将及AI的设计优先检查修改；保留测试用例和静态检查，中途不运行测试、不等待逐批签收，全部完成后统一测试。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="81">
+      <x:c r="A81" t="str">
+        <x:v>excel_r291</x:v>
+      </x:c>
+      <x:c r="B81" t="str">
+        <x:v>机甲忍者。赤</x:v>
+      </x:c>
+      <x:c r="C81" t="str">
+        <x:v>2026-09-06复核新10场：45次声明逐条对应45条公开随机破魔日志，无遗漏或重复；专属测试未列入失败。本批随太阳神测试修正保持待复测。</x:v>
+      </x:c>
+      <x:c r="D81" t="str">
+        <x:v>战斗实现</x:v>
+      </x:c>
+      <x:c r="E81" t="str">
+        <x:v>追击只强化赤对绑定单位的下一份直接伤害一次；本发铁锁、场地伤害、队友伤害和其他目标不能消费。</x:v>
+      </x:c>
+      <x:c r="F81" t="str">
+        <x:v>RedNextDamageStatus在本发完成后添加；on_before_damage核对source与target并排除from_field_effect，修改该DamageContext后立即移除；duration=1且any_turn_end使其在当前回合末失效。</x:v>
+      </x:c>
+      <x:c r="G81" t="str">
+        <x:v>符合</x:v>
+      </x:c>
+      <x:c r="H81" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="I81" t="str">
+        <x:v>保留实现，并由当前批次定向与审计日志核对一次性消费。</x:v>
+      </x:c>
+      <x:c r="J81" t="str">
+        <x:v>已审查，待用户当前批次测试</x:v>
+      </x:c>
+      <x:c r="K81" t="str">
+        <x:v>docs/武将设计思想.json#excel_r291</x:v>
+      </x:c>
+      <x:c r="L81" t="str">
+        <x:v>9月4日新10场3胜7负、铁锁7次、吸魔3次、回避27次。逐场声明/公开随机日志数为2/2、6/6、7/7、2/2、2/2、6/6、2/2、6/6、10/10、2/2，共45/45；每次声明同一步均有对应结果。929项回归没有赤专属失败。</x:v>
+      </x:c>
+      <x:c r="M81" t="str">
+        <x:v>2026-09-06用户调整：连续分批完成全部已开发武将及AI的设计优先检查修改；保留测试用例和静态检查，中途不运行测试、不等待逐批签收，全部完成后统一测试。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="82">
+      <x:c r="A82" t="str">
+        <x:v>excel_r291</x:v>
+      </x:c>
+      <x:c r="B82" t="str">
+        <x:v>机甲忍者。赤</x:v>
+      </x:c>
+      <x:c r="C82" t="str">
+        <x:v>2026-09-06复核新10场：45次声明逐条对应45条公开随机破魔日志，无遗漏或重复；专属测试未列入失败。本批随太阳神测试修正保持待复测。</x:v>
+      </x:c>
+      <x:c r="D82" t="str">
+        <x:v>战斗实现</x:v>
+      </x:c>
+      <x:c r="E82" t="str">
+        <x:v>随机破魔必须每个声明恰采样一次、公开结果、同动作共享，且不能泄漏到后续动作。</x:v>
+      </x:c>
+      <x:c r="F82" t="str">
+        <x:v>RedRandomPierceTrait在on_owner_action_declared单次采样并把结果写入动作payload；2026-09-03日志发现用普通battle.log写结果时，对隐身目标的动作会被隐身抑制。现改用带来源的公开事件接口，保证随机结果公开，同时仍只存在于本次payload。</x:v>
+      </x:c>
+      <x:c r="G82" t="str">
+        <x:v>已修复待验证</x:v>
+      </x:c>
+      <x:c r="H82" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="I82" t="str">
+        <x:v>保留动作载荷传播；公开结果改走不可被隐身目标抑制的公开事件，并补隐身目标场景。</x:v>
+      </x:c>
+      <x:c r="J82" t="str">
+        <x:v>二次修复并补测试，待用户复跑当前批次</x:v>
+      </x:c>
+      <x:c r="K82" t="str">
+        <x:v>docs/武将设计思想.json#excel_r291</x:v>
+      </x:c>
+      <x:c r="L82" t="str">
+        <x:v>9月4日新10场3胜7负、铁锁7次、吸魔3次、回避27次。逐场声明/公开随机日志数为2/2、6/6、7/7、2/2、2/2、6/6、2/2、6/6、10/10、2/2，共45/45；每次声明同一步均有对应结果。929项回归没有赤专属失败。</x:v>
+      </x:c>
+      <x:c r="M82" t="str">
+        <x:v>2026-09-06用户调整：连续分批完成全部已开发武将及AI的设计优先检查修改；保留测试用例和静态检查，中途不运行测试、不等待逐批签收，全部完成后统一测试。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="83">
+      <x:c r="A83" t="str">
+        <x:v>excel_r291</x:v>
+      </x:c>
+      <x:c r="B83" t="str">
+        <x:v>机甲忍者。赤</x:v>
+      </x:c>
+      <x:c r="C83" t="str">
+        <x:v>2026-09-06复核新10场：45次声明逐条对应45条公开随机破魔日志，无遗漏或重复；专属测试未列入失败。本批随太阳神测试修正保持待复测。</x:v>
+      </x:c>
+      <x:c r="D83" t="str">
+        <x:v>AI</x:v>
+      </x:c>
+      <x:c r="E83" t="str">
+        <x:v>铁锁评分必须接受强制最近锚点，计算实际落点风险和本回合追击兑现，不能只按线伤与免费奖励决策。</x:v>
+      </x:c>
+      <x:c r="F83" t="str">
+        <x:v>旧iron_chain_path_score只调用skill_damage_score、目标价值与首发+12。现复用战斗实现的anchor_for_cells/destination_for_anchor，加入真实落点移动价值、敌方可达伤害、多攻威胁、敌方单位追击收益、友军/地形锚机会成本；无敌方命中仍拒绝。</x:v>
+      </x:c>
+      <x:c r="G83" t="str">
+        <x:v>已修复待验证</x:v>
+      </x:c>
+      <x:c r="H83" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="I83" t="str">
+        <x:v>已补两条等伤线路中避开高攻敌人可达落点的AI行为测试。</x:v>
+      </x:c>
+      <x:c r="J83" t="str">
+        <x:v>待用户当前批次测试</x:v>
+      </x:c>
+      <x:c r="K83" t="str">
+        <x:v>docs/武将设计思想.json#excel_r291</x:v>
+      </x:c>
+      <x:c r="L83" t="str">
+        <x:v>9月4日新10场3胜7负、铁锁7次、吸魔3次、回避27次。逐场声明/公开随机日志数为2/2、6/6、7/7、2/2、2/2、6/6、2/2、6/6、10/10、2/2，共45/45；每次声明同一步均有对应结果。929项回归没有赤专属失败。</x:v>
+      </x:c>
+      <x:c r="M83" t="str">
+        <x:v>2026-09-06用户调整：连续分批完成全部已开发武将及AI的设计优先检查修改；保留测试用例和静态检查，中途不运行测试、不等待逐批签收，全部完成后统一测试。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="84">
+      <x:c r="A84" t="str">
+        <x:v>excel_r291</x:v>
+      </x:c>
+      <x:c r="B84" t="str">
+        <x:v>机甲忍者。赤</x:v>
+      </x:c>
+      <x:c r="C84" t="str">
+        <x:v>2026-09-06复核新10场：45次声明逐条对应45条公开随机破魔日志，无遗漏或重复；专属测试未列入失败。本批随太阳神测试修正保持待复测。</x:v>
+      </x:c>
+      <x:c r="D84" t="str">
+        <x:v>测试</x:v>
+      </x:c>
+      <x:c r="E84" t="str">
+        <x:v>测试矩阵必须覆盖锚点阵营/地形/顺序、严格位移、追击生命周期、费用与随机动作边界，并验证AI落位质量。</x:v>
+      </x:c>
+      <x:c r="F84" t="str">
+        <x:v>已覆盖墙体锚、死亡锚点锁定、随机状态不残留、强制锚点落位风险、首发免费、单位追击和单动作单随机；本轮补隐身目标仍公开随机结果，并把致死样本血量改为真实可击破值、把墙体落点断言改为验证直线/5格/真实邻接而非唯一坐标。开发代理未运行动态测试。</x:v>
+      </x:c>
+      <x:c r="G84" t="str">
+        <x:v>已补充待验证</x:v>
+      </x:c>
+      <x:c r="H84" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="I84" t="str">
         <x:v>由用户运行python detail_test_all_wujiangs.py --current。</x:v>
       </x:c>
-      <x:c r="J80" t="str">
+      <x:c r="J84" t="str">
+        <x:v>测试夹具与公开日志场景已修，待用户复跑当前批次</x:v>
+      </x:c>
+      <x:c r="K84" t="str">
+        <x:v>docs/武将设计思想.json#excel_r291</x:v>
+      </x:c>
+      <x:c r="L84" t="str">
+        <x:v>9月4日新10场3胜7负、铁锁7次、吸魔3次、回避27次。逐场声明/公开随机日志数为2/2、6/6、7/7、2/2、2/2、6/6、2/2、6/6、10/10、2/2，共45/45；每次声明同一步均有对应结果。929项回归没有赤专属失败。</x:v>
+      </x:c>
+      <x:c r="M84" t="str">
+        <x:v>2026-09-06用户调整：连续分批完成全部已开发武将及AI的设计优先检查修改；保留测试用例和静态检查，中途不运行测试、不等待逐批签收，全部完成后统一测试。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="85">
+      <x:c r="A85" t="str">
+        <x:v>excel_r356</x:v>
+      </x:c>
+      <x:c r="B85" t="str">
+        <x:v>强袭犀牛</x:v>
+      </x:c>
+      <x:c r="C85" t="str">
+        <x:v>2026-09-06复核新10场：24拳包含7个完整三拳回合，4次到期无锚等待日志可见。龙息与实际回归仍为随机局覆盖缺口，专属定向测试未列入失败；本批随太阳神测试修正保持待复测。</x:v>
+      </x:c>
+      <x:c r="D85" t="str">
+        <x:v>战斗实现</x:v>
+      </x:c>
+      <x:c r="E85" t="str">
+        <x:v>面板与神速、龙息、震开、变硬、每回合三次普攻必须完整映射源表。</x:v>
+      </x:c>
+      <x:c r="F85" t="str">
+        <x:v>excel_r356使用通用ShensuSkill、DragonBreathSkill、KnockbackSkill、HardenSkill，并由AttackCountTrait把每回合普攻数改为3。</x:v>
+      </x:c>
+      <x:c r="G85" t="str">
+        <x:v>符合</x:v>
+      </x:c>
+      <x:c r="H85" t="str">
+        <x:v>P3</x:v>
+      </x:c>
+      <x:c r="I85" t="str">
+        <x:v>不改通用技能数值，补AI连续三拳行为断言。</x:v>
+      </x:c>
+      <x:c r="J85" t="str">
+        <x:v>已审查，待用户当前批次测试</x:v>
+      </x:c>
+      <x:c r="K85" t="str">
+        <x:v>docs/武将设计思想.json#excel_r356</x:v>
+      </x:c>
+      <x:c r="L85" t="str">
+        <x:v>9月4日新10场5胜5负、神速8次、普攻24次、变硬6次、震开3次。第2/3/5/6/7/9/10场各有一次完整三拳，另第3场后续2拳、第4场1拳。第7场步骤67/72/74/76均记录到期等待回归。龙息8个可用节点无有效候选；随机局未满足全部回归条件，保留条件覆盖缺口。929项回归无犀牛专属失败。</x:v>
+      </x:c>
+      <x:c r="M85" t="str">
+        <x:v>2026-09-06用户调整：连续分批完成全部已开发武将及AI的设计优先检查修改；保留测试用例和静态检查，中途不运行测试、不等待逐批签收，全部完成后统一测试。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="86">
+      <x:c r="A86" t="str">
+        <x:v>excel_r356</x:v>
+      </x:c>
+      <x:c r="B86" t="str">
+        <x:v>强袭犀牛</x:v>
+      </x:c>
+      <x:c r="C86" t="str">
+        <x:v>2026-09-06复核新10场：24拳包含7个完整三拳回合，4次到期无锚等待日志可见。龙息与实际回归仍为随机局覆盖缺口，专属定向测试未列入失败；本批随太阳神测试修正保持待复测。</x:v>
+      </x:c>
+      <x:c r="D86" t="str">
+        <x:v>战斗实现</x:v>
+      </x:c>
+      <x:c r="E86" t="str">
+        <x:v>每次真实破坏都应触发一次遗志和一个回归计时；同一条生命不得重复触发，但回归后的下一条生命必须重新具备资格。</x:v>
+      </x:c>
+      <x:c r="F86" t="str">
+        <x:v>RhinoDeathTrait以triggered防止伤害钩子与移除钩子重复。审查发现旧triggered只在初次入场重置，回归后第二次死亡会永久失效；现回归前明确重置，add_unit入场钩子再次确认新生命状态。</x:v>
+      </x:c>
+      <x:c r="G86" t="str">
+        <x:v>已修复待验证</x:v>
+      </x:c>
+      <x:c r="H86" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="I86" t="str">
+        <x:v>已补同一犀牛回归后第二次破坏再次产生单个回归记录、刷新而不叠遗志的测试。</x:v>
+      </x:c>
+      <x:c r="J86" t="str">
+        <x:v>待用户当前批次测试</x:v>
+      </x:c>
+      <x:c r="K86" t="str">
+        <x:v>docs/武将设计思想.json#excel_r356</x:v>
+      </x:c>
+      <x:c r="L86" t="str">
+        <x:v>9月4日新10场5胜5负、神速8次、普攻24次、变硬6次、震开3次。第2/3/5/6/7/9/10场各有一次完整三拳，另第3场后续2拳、第4场1拳。第7场步骤67/72/74/76均记录到期等待回归。龙息8个可用节点无有效候选；随机局未满足全部回归条件，保留条件覆盖缺口。929项回归无犀牛专属失败。</x:v>
+      </x:c>
+      <x:c r="M86" t="str">
+        <x:v>2026-09-06用户调整：连续分批完成全部已开发武将及AI的设计优先检查修改；保留测试用例和静态检查，中途不运行测试、不等待逐批签收，全部完成后统一测试。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="87">
+      <x:c r="A87" t="str">
+        <x:v>excel_r356</x:v>
+      </x:c>
+      <x:c r="B87" t="str">
+        <x:v>强袭犀牛</x:v>
+      </x:c>
+      <x:c r="C87" t="str">
+        <x:v>2026-09-06复核新10场：24拳包含7个完整三拳回合，4次到期无锚等待日志可见。龙息与实际回归仍为随机局覆盖缺口，专属定向测试未列入失败；本批随太阳神测试修正保持待复测。</x:v>
+      </x:c>
+      <x:c r="D87" t="str">
+        <x:v>战斗实现</x:v>
+      </x:c>
+      <x:c r="E87" t="str">
+        <x:v>遗志只给破坏瞬间仍在场的其他友军，持续各自3回合；同名效果不叠加只刷新。</x:v>
+      </x:c>
+      <x:c r="F87" t="str">
+        <x:v>trigger_legacy快照player_units、排除owner和离场单位，包含正常召唤/分身；已有同名状态先移除再添加RhinoLegacyStatus(duration=3, owner_turn_end)。</x:v>
+      </x:c>
+      <x:c r="G87" t="str">
+        <x:v>符合</x:v>
+      </x:c>
+      <x:c r="H87" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="I87" t="str">
+        <x:v>保留实现，当前批次检查接收者数量、层数与刷新时长。</x:v>
+      </x:c>
+      <x:c r="J87" t="str">
+        <x:v>已审查，待用户当前批次测试</x:v>
+      </x:c>
+      <x:c r="K87" t="str">
+        <x:v>docs/武将设计思想.json#excel_r356</x:v>
+      </x:c>
+      <x:c r="L87" t="str">
+        <x:v>9月4日新10场5胜5负、神速8次、普攻24次、变硬6次、震开3次。第2/3/5/6/7/9/10场各有一次完整三拳，另第3场后续2拳、第4场1拳。第7场步骤67/72/74/76均记录到期等待回归。龙息8个可用节点无有效候选；随机局未满足全部回归条件，保留条件覆盖缺口。929项回归无犀牛专属失败。</x:v>
+      </x:c>
+      <x:c r="M87" t="str">
+        <x:v>2026-09-06用户调整：连续分批完成全部已开发武将及AI的设计优先检查修改；保留测试用例和静态检查，中途不运行测试、不等待逐批签收，全部完成后统一测试。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="88">
+      <x:c r="A88" t="str">
+        <x:v>excel_r356</x:v>
+      </x:c>
+      <x:c r="B88" t="str">
+        <x:v>强袭犀牛</x:v>
+      </x:c>
+      <x:c r="C88" t="str">
+        <x:v>2026-09-06复核新10场：24拳包含7个完整三拳回合，4次到期无锚等待日志可见。龙息与实际回归仍为随机局覆盖缺口，专属定向测试未列入失败；本批随太阳神测试修正保持待复测。</x:v>
+      </x:c>
+      <x:c r="D88" t="str">
+        <x:v>战斗实现</x:v>
+      </x:c>
+      <x:c r="E88" t="str">
+        <x:v>回归要等待死亡后3个完整全局行动环；到期无兽人本体或无合法格必须保留记录并在以后每个武将回合重试。</x:v>
+      </x:c>
+      <x:c r="F88" t="str">
+        <x:v>return_turn_number=death_turn_number+固定turn_order槽数×3；turn_number会为死亡槽也推进。on_turn_start未到期或无候选时保留field effect；兽人候选排除召唤和分身。为让设计规定的持续重试可观察，现于到期但没有合法兽人/落点时记录明确等待日志。</x:v>
+      </x:c>
+      <x:c r="G88" t="str">
+        <x:v>符合并补测试</x:v>
+      </x:c>
+      <x:c r="H88" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="I88" t="str">
+        <x:v>保留重试机制；补所有兽人邻格阻塞时保留记录、腾格后自动回归，并断言到期等待日志。</x:v>
+      </x:c>
+      <x:c r="J88" t="str">
+        <x:v>等待日志与断言已补，待用户复跑当前批次</x:v>
+      </x:c>
+      <x:c r="K88" t="str">
+        <x:v>docs/武将设计思想.json#excel_r356</x:v>
+      </x:c>
+      <x:c r="L88" t="str">
+        <x:v>9月4日新10场5胜5负、神速8次、普攻24次、变硬6次、震开3次。第2/3/5/6/7/9/10场各有一次完整三拳，另第3场后续2拳、第4场1拳。第7场步骤67/72/74/76均记录到期等待回归。龙息8个可用节点无有效候选；随机局未满足全部回归条件，保留条件覆盖缺口。929项回归无犀牛专属失败。</x:v>
+      </x:c>
+      <x:c r="M88" t="str">
+        <x:v>2026-09-06用户调整：连续分批完成全部已开发武将及AI的设计优先检查修改；保留测试用例和静态检查，中途不运行测试、不等待逐批签收，全部完成后统一测试。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="89">
+      <x:c r="A89" t="str">
+        <x:v>excel_r356</x:v>
+      </x:c>
+      <x:c r="B89" t="str">
+        <x:v>强袭犀牛</x:v>
+      </x:c>
+      <x:c r="C89" t="str">
+        <x:v>2026-09-06复核新10场：24拳包含7个完整三拳回合，4次到期无锚等待日志可见。龙息与实际回归仍为随机局覆盖缺口，专属定向测试未列入失败；本批随太阳神测试修正保持待复测。</x:v>
+      </x:c>
+      <x:c r="D89" t="str">
+        <x:v>战斗实现</x:v>
+      </x:c>
+      <x:c r="E89" t="str">
+        <x:v>多个兽人锚必须按固定行动槽选择第一个有合法格者，落点使用稳定格序。</x:v>
+      </x:c>
+      <x:c r="F89" t="str">
+        <x:v>旧实现按等级降序、unit_id选锚，会让高等级后槽越过前槽。现按turn_order_unit_ids索引再按unit_id排序，周围格继续按y/x稳定顺序。</x:v>
+      </x:c>
+      <x:c r="G89" t="str">
+        <x:v>已修复待验证</x:v>
+      </x:c>
+      <x:c r="H89" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="I89" t="str">
+        <x:v>已补前槽4级兽人优先于后槽5级兽人的阻塞重试测试。</x:v>
+      </x:c>
+      <x:c r="J89" t="str">
+        <x:v>待用户当前批次测试</x:v>
+      </x:c>
+      <x:c r="K89" t="str">
+        <x:v>docs/武将设计思想.json#excel_r356</x:v>
+      </x:c>
+      <x:c r="L89" t="str">
+        <x:v>9月4日新10场5胜5负、神速8次、普攻24次、变硬6次、震开3次。第2/3/5/6/7/9/10场各有一次完整三拳，另第3场后续2拳、第4场1拳。第7场步骤67/72/74/76均记录到期等待回归。龙息8个可用节点无有效候选；随机局未满足全部回归条件，保留条件覆盖缺口。929项回归无犀牛专属失败。</x:v>
+      </x:c>
+      <x:c r="M89" t="str">
+        <x:v>2026-09-06用户调整：连续分批完成全部已开发武将及AI的设计优先检查修改；保留测试用例和静态检查，中途不运行测试、不等待逐批签收，全部完成后统一测试。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="90">
+      <x:c r="A90" t="str">
+        <x:v>excel_r356</x:v>
+      </x:c>
+      <x:c r="B90" t="str">
+        <x:v>强袭犀牛</x:v>
+      </x:c>
+      <x:c r="C90" t="str">
+        <x:v>2026-09-06复核新10场：24拳包含7个完整三拳回合，4次到期无锚等待日志可见。龙息与实际回归仍为随机局覆盖缺口，专属定向测试未列入失败；本批随太阳神测试修正保持待复测。</x:v>
+      </x:c>
+      <x:c r="D90" t="str">
+        <x:v>战斗实现</x:v>
+      </x:c>
+      <x:c r="E90" t="str">
+        <x:v>回归应满血满魔、清上一生命临时状态，保留永久数值变化、身份、固定行动槽、冷却和本场使用记录，并且不赠送即时行动。</x:v>
+      </x:c>
+      <x:c r="F90" t="str">
+        <x:v>旧实现无条件移除全部status，误删duration=None的永久StatModifierStatus。现只保留无期限数值状态，清除其他临时状态；沿用原对象与skill对象，恢复血魔并把turn_ready及当前回合动作字段清零，固定turn_order不改。</x:v>
+      </x:c>
+      <x:c r="G90" t="str">
+        <x:v>已修复待验证</x:v>
+      </x:c>
+      <x:c r="H90" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="I90" t="str">
+        <x:v>已补永久/临时状态分离、技能记录/冷却、固定槽及无即时行动断言。</x:v>
+      </x:c>
+      <x:c r="J90" t="str">
+        <x:v>待用户当前批次测试</x:v>
+      </x:c>
+      <x:c r="K90" t="str">
+        <x:v>docs/武将设计思想.json#excel_r356</x:v>
+      </x:c>
+      <x:c r="L90" t="str">
+        <x:v>9月4日新10场5胜5负、神速8次、普攻24次、变硬6次、震开3次。第2/3/5/6/7/9/10场各有一次完整三拳，另第3场后续2拳、第4场1拳。第7场步骤67/72/74/76均记录到期等待回归。龙息8个可用节点无有效候选；随机局未满足全部回归条件，保留条件覆盖缺口。929项回归无犀牛专属失败。</x:v>
+      </x:c>
+      <x:c r="M90" t="str">
+        <x:v>2026-09-06用户调整：连续分批完成全部已开发武将及AI的设计优先检查修改；保留测试用例和静态检查，中途不运行测试、不等待逐批签收，全部完成后统一测试。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="91">
+      <x:c r="A91" t="str">
+        <x:v>excel_r356</x:v>
+      </x:c>
+      <x:c r="B91" t="str">
+        <x:v>强袭犀牛</x:v>
+      </x:c>
+      <x:c r="C91" t="str">
+        <x:v>2026-09-06复核新10场：24拳包含7个完整三拳回合，4次到期无锚等待日志可见。龙息与实际回归仍为随机局覆盖缺口，专属定向测试未列入失败；本批随太阳神测试修正保持待复测。</x:v>
+      </x:c>
+      <x:c r="D91" t="str">
+        <x:v>通用AI</x:v>
+      </x:c>
+      <x:c r="E91" t="str">
+        <x:v>三次普攻必须作为三次依次声明的动作，每拳后重新生成候选，不能打一拳便结束。</x:v>
+      </x:c>
+      <x:c r="F91" t="str">
+        <x:v>choose_turn_action和choose_turn_bundle_action每次调用重新读取action_snapshot；Battle每拳只递增一次attacks_used，达到attack_actions_per_turn前继续提供普攻候选。旧集中审计中犀牛已有稳定多拳信号，未发现需改通用评分的证据。</x:v>
+      </x:c>
+      <x:c r="G91" t="str">
+        <x:v>符合并补测试</x:v>
+      </x:c>
+      <x:c r="H91" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="I91" t="str">
+        <x:v>保留通用重规划架构，新增0魔且持续有目标时连续选择并执行三次普攻的行为测试。</x:v>
+      </x:c>
+      <x:c r="J91" t="str">
+        <x:v>待用户当前批次测试</x:v>
+      </x:c>
+      <x:c r="K91" t="str">
+        <x:v>docs/武将设计思想.json#excel_r356</x:v>
+      </x:c>
+      <x:c r="L91" t="str">
+        <x:v>9月4日新10场5胜5负、神速8次、普攻24次、变硬6次、震开3次。第2/3/5/6/7/9/10场各有一次完整三拳，另第3场后续2拳、第4场1拳。第7场步骤67/72/74/76均记录到期等待回归。龙息8个可用节点无有效候选；随机局未满足全部回归条件，保留条件覆盖缺口。929项回归无犀牛专属失败。</x:v>
+      </x:c>
+      <x:c r="M91" t="str">
+        <x:v>2026-09-06用户调整：连续分批完成全部已开发武将及AI的设计优先检查修改；保留测试用例和静态检查，中途不运行测试、不等待逐批签收，全部完成后统一测试。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="92">
+      <x:c r="A92" t="str">
+        <x:v>excel_r356</x:v>
+      </x:c>
+      <x:c r="B92" t="str">
+        <x:v>强袭犀牛</x:v>
+      </x:c>
+      <x:c r="C92" t="str">
+        <x:v>2026-09-06复核新10场：24拳包含7个完整三拳回合，4次到期无锚等待日志可见。龙息与实际回归仍为随机局覆盖缺口，专属定向测试未列入失败；本批随太阳神测试修正保持待复测。</x:v>
+      </x:c>
+      <x:c r="D92" t="str">
+        <x:v>测试</x:v>
+      </x:c>
+      <x:c r="E92" t="str">
+        <x:v>测试矩阵必须覆盖两次死亡、遗志刷新、完整行动环、无兽人/无格重试、固定槽选锚、回归保留边界和三拳AI。</x:v>
+      </x:c>
+      <x:c r="F92" t="str">
+        <x:v>已在伤害/非伤害破坏和三环计时基础上覆盖第二次死亡、状态与场次记录、固定槽、阻塞重试及逐拳重规划；本轮再断言到期无合法锚/落点时输出等待日志。审计工具同时区分‘技能可用但无有效候选’与真实错失，并隔离其他武将同名日志。开发代理未运行动态测试。</x:v>
+      </x:c>
+      <x:c r="G92" t="str">
+        <x:v>已补充待验证</x:v>
+      </x:c>
+      <x:c r="H92" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="I92" t="str">
+        <x:v>由用户运行python detail_test_all_wujiangs.py --current。</x:v>
+      </x:c>
+      <x:c r="J92" t="str">
         <x:v>等待可观察性与审计分类已补，待用户复跑当前批次</x:v>
       </x:c>
-      <x:c r="K80" t="str">
+      <x:c r="K92" t="str">
         <x:v>docs/武将设计思想.json#excel_r356</x:v>
       </x:c>
-      <x:c r="L80" t="str">
+      <x:c r="L92" t="str">
         <x:v>9月4日新10场5胜5负、神速8次、普攻24次、变硬6次、震开3次。第2/3/5/6/7/9/10场各有一次完整三拳，另第3场后续2拳、第4场1拳。第7场步骤67/72/74/76均记录到期等待回归。龙息8个可用节点无有效候选；随机局未满足全部回归条件，保留条件覆盖缺口。929项回归无犀牛专属失败。</x:v>
       </x:c>
-      <x:c r="M80" t="str">
+      <x:c r="M92" t="str">
         <x:v>2026-09-06用户调整：连续分批完成全部已开发武将及AI的设计优先检查修改；保留测试用例和静态检查，中途不运行测试、不等待逐批签收，全部完成后统一测试。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R19835b2e15dd4a5e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb4617ddbdd5d4d8d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>